<commit_message>
Edit BCIO_Schedule.xlsx: update 2, add 8
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +40,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007fffd4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
       </patternFill>
     </fill>
     <fill>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V65"/>
+  <dimension ref="A1:V73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1009,7 +1015,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is how often intervention temporal parts occur within a BCI.</t>
+          <t>An &lt;intervention temporal part frequency&gt; that is how often intervention temporal parts occur within a BCI.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1019,7 +1025,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>intervention temporal part frequency</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1039,7 +1045,7 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
@@ -1220,131 +1226,107 @@
       <c r="V12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050505</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event duration statistic</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event durations.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event duration</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="n"/>
-      <c r="P13" s="2" t="n"/>
-      <c r="Q13" s="2" t="n"/>
-      <c r="R13" s="2" t="n"/>
-      <c r="S13" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="T13" s="2" t="n"/>
-      <c r="U13" s="2" t="n"/>
-      <c r="V13" s="2" t="n"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050999</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>interval between intervention temporal parts</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the end of one intervention temporal part and the beginning of a subsequent intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr"/>
+      <c r="N13" s="3" t="inlineStr"/>
+      <c r="O13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr"/>
+      <c r="R13" s="3" t="inlineStr"/>
+      <c r="S13" s="3" t="inlineStr"/>
+      <c r="T13" s="3" t="inlineStr"/>
+      <c r="U13" s="3" t="inlineStr"/>
+      <c r="V13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050903</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event frequency statistic</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event frequency</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="n"/>
-      <c r="Q14" s="2" t="n"/>
-      <c r="R14" s="2" t="n"/>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="T14" s="2" t="n"/>
-      <c r="U14" s="2" t="n"/>
-      <c r="V14" s="2" t="n"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051000</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr"/>
+      <c r="R14" s="3" t="inlineStr"/>
+      <c r="S14" s="3" t="inlineStr"/>
+      <c r="T14" s="3" t="inlineStr"/>
+      <c r="U14" s="3" t="inlineStr"/>
+      <c r="V14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050904</t>
+          <t>BCIO:050505</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D15" s="2" t="n"/>
@@ -1369,7 +1351,7 @@
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M15" s="2" t="n"/>
@@ -1388,75 +1370,63 @@
       <c r="V15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050905</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>intervention duration statistic</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051001</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event frequency</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>BCI duration</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="n"/>
-      <c r="O16" s="2" t="n"/>
-      <c r="P16" s="2" t="n"/>
-      <c r="Q16" s="2" t="n"/>
-      <c r="R16" s="2" t="n"/>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="T16" s="2" t="n"/>
-      <c r="U16" s="2" t="n"/>
-      <c r="V16" s="2" t="n"/>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr"/>
+      <c r="N16" s="3" t="inlineStr"/>
+      <c r="O16" s="3" t="inlineStr"/>
+      <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr"/>
+      <c r="R16" s="3" t="inlineStr"/>
+      <c r="S16" s="3" t="inlineStr"/>
+      <c r="T16" s="3" t="inlineStr"/>
+      <c r="U16" s="3" t="inlineStr"/>
+      <c r="V16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050506</t>
+          <t>BCIO:050903</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention temporal part durations.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -1481,7 +1451,7 @@
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M17" s="2" t="n"/>
@@ -1502,17 +1472,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050516</t>
+          <t>BCIO:050904</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention temporal part frequencies.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -1537,7 +1507,7 @@
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M18" s="2" t="n"/>
@@ -1556,94 +1526,69 @@
       <c r="V18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:008540</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>irregular intervention schedule</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or BCI.  </t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>BCI schedule of delivery</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
-Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks" </t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="n"/>
-      <c r="Q19" s="2" t="inlineStr">
-        <is>
-          <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
-        </is>
-      </c>
-      <c r="R19" s="2" t="n"/>
-      <c r="S19" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
-      <c r="T19" s="2" t="inlineStr">
-        <is>
-          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
-        </is>
-      </c>
-      <c r="U19" s="2" t="n"/>
-      <c r="V19" s="2" t="n"/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051002</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>intervention duration</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr"/>
+      <c r="N19" s="3" t="inlineStr"/>
+      <c r="O19" s="3" t="inlineStr"/>
+      <c r="P19" s="3" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr"/>
+      <c r="R19" s="3" t="inlineStr"/>
+      <c r="S19" s="3" t="inlineStr"/>
+      <c r="T19" s="3" t="inlineStr"/>
+      <c r="U19" s="3" t="inlineStr"/>
+      <c r="V19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050507</t>
+          <t>BCIO:050905</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event duration</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1662,7 +1607,7 @@
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M20" s="2" t="n"/>
@@ -1681,81 +1626,69 @@
       <c r="V20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050906</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>maximum intervention contact event frequency</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event frequency statistic</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event frequency</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
-      <c r="O21" s="2" t="n"/>
-      <c r="P21" s="2" t="n"/>
-      <c r="Q21" s="2" t="n"/>
-      <c r="R21" s="2" t="n"/>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="n"/>
-      <c r="U21" s="2" t="n"/>
-      <c r="V21" s="2" t="n"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051003</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>intervention temporal part duration</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr"/>
+      <c r="N21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr"/>
+      <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr"/>
+      <c r="R21" s="3" t="inlineStr"/>
+      <c r="S21" s="3" t="inlineStr"/>
+      <c r="T21" s="3" t="inlineStr"/>
+      <c r="U21" s="3" t="inlineStr"/>
+      <c r="V21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050907</t>
+          <t>BCIO:050506</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event number</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1774,7 +1707,7 @@
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M22" s="2" t="n"/>
@@ -1793,81 +1726,73 @@
       <c r="V22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050908</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>maximum intervention duration</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>intervention duration statistic</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>BCI duration</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="n"/>
-      <c r="R23" s="2" t="n"/>
-      <c r="S23" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="T23" s="2" t="n"/>
-      <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="n"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051004</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>intervention temporal part frequency</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is how often intervention temporal parts occur within an intervention.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is useful when grouping contact events together to the schedule of an intervention. For example, authors may describe participants as taking part in 90 minutes of physical activity weekly. These 90 minutes could be split across several contact events, however together these contact events form an intervention part which occurs weekly. </t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr"/>
+      <c r="N23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr"/>
+      <c r="R23" s="3" t="inlineStr"/>
+      <c r="S23" s="3" t="inlineStr"/>
+      <c r="T23" s="3" t="inlineStr"/>
+      <c r="U23" s="3" t="inlineStr"/>
+      <c r="V23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050508</t>
+          <t>BCIO:050516</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part duration</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1886,7 +1811,7 @@
       <c r="K24" s="2" t="n"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M24" s="2" t="n"/>
@@ -1907,32 +1832,37 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050517</t>
+          <t>BCIO:008540</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part frequency statistic</t>
+          <t>irregular intervention schedule</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="n"/>
+          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or BCI.  </t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
+        </is>
+      </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
+          <t>BCI schedule of delivery</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
+Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks" </t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -1940,46 +1870,54 @@
       </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>BCI temporal part frequency</t>
-        </is>
-      </c>
+      <c r="L25" s="2" t="n"/>
       <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P25" s="2" t="n"/>
-      <c r="Q25" s="2" t="n"/>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
+        </is>
+      </c>
       <c r="R25" s="2" t="n"/>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="T25" s="2" t="n"/>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
+        </is>
+      </c>
       <c r="U25" s="2" t="n"/>
       <c r="V25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050910</t>
+          <t>BCIO:050507</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>maximum total intervention contact event duration</t>
+          <t>maximum intervention contact event duration</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1998,7 +1936,7 @@
       <c r="K26" s="2" t="n"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M26" s="2" t="n"/>
@@ -2019,23 +1957,23 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050509</t>
+          <t>BCIO:050906</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event duration</t>
+          <t>maximum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2054,7 +1992,7 @@
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M27" s="2" t="n"/>
@@ -2075,23 +2013,23 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050911</t>
+          <t>BCIO:050907</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event frequency</t>
+          <t>maximum intervention contact event number</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2110,7 +2048,7 @@
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M28" s="2" t="n"/>
@@ -2131,23 +2069,23 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050912</t>
+          <t>BCIO:050908</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event number</t>
+          <t>maximum intervention duration</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2166,7 +2104,7 @@
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M29" s="2" t="n"/>
@@ -2187,23 +2125,23 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050909</t>
+          <t>BCIO:050508</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>mean intervention duration</t>
+          <t>maximum intervention temporal part duration</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2222,7 +2160,7 @@
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M30" s="2" t="n"/>
@@ -2243,23 +2181,23 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050510</t>
+          <t>BCIO:050517</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part duration</t>
+          <t>maximum intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2278,7 +2216,7 @@
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M31" s="2" t="n"/>
@@ -2299,23 +2237,23 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050518</t>
+          <t>BCIO:050910</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part frequency statistic</t>
+          <t>maximum total intervention contact event duration</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2334,7 +2272,7 @@
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M32" s="2" t="n"/>
@@ -2355,23 +2293,23 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050495</t>
+          <t>BCIO:050509</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>mean total intervention contact event duration</t>
+          <t>mean intervention contact event duration</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2390,7 +2328,7 @@
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M33" s="2" t="n"/>
@@ -2411,23 +2349,23 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050511</t>
+          <t>BCIO:050911</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event duration</t>
+          <t>mean intervention contact event frequency</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2446,7 +2384,7 @@
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M34" s="2" t="n"/>
@@ -2467,23 +2405,23 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050496</t>
+          <t>BCIO:050912</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event frequency</t>
+          <t>mean intervention contact event number</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2502,7 +2440,7 @@
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M35" s="2" t="n"/>
@@ -2523,23 +2461,23 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050497</t>
+          <t>BCIO:050909</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event number</t>
+          <t>mean intervention duration</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2558,7 +2496,7 @@
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M36" s="2" t="n"/>
@@ -2579,23 +2517,23 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050498</t>
+          <t>BCIO:050510</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>median intervention duration</t>
+          <t>mean intervention temporal part duration</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2614,7 +2552,7 @@
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M37" s="2" t="n"/>
@@ -2635,23 +2573,23 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050512</t>
+          <t>BCIO:050518</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part duration</t>
+          <t>mean intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2670,7 +2608,7 @@
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M38" s="2" t="n"/>
@@ -2691,23 +2629,23 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050519</t>
+          <t>BCIO:050495</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part frequency statistic</t>
+          <t>mean total intervention contact event duration</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2726,7 +2664,7 @@
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M39" s="2" t="n"/>
@@ -2747,23 +2685,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050499</t>
+          <t>BCIO:050511</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>median total intervention contact event duration</t>
+          <t>median intervention contact event duration</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2782,7 +2720,7 @@
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M40" s="2" t="n"/>
@@ -2803,23 +2741,23 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050513</t>
+          <t>BCIO:050496</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event duration</t>
+          <t>median intervention contact event frequency</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2838,7 +2776,7 @@
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M41" s="2" t="n"/>
@@ -2859,23 +2797,23 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050500</t>
+          <t>BCIO:050497</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event frequency</t>
+          <t>median intervention contact event number</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2894,7 +2832,7 @@
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M42" s="2" t="n"/>
@@ -2915,23 +2853,23 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050502</t>
+          <t>BCIO:050498</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event number</t>
+          <t>median intervention duration</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2950,7 +2888,7 @@
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M43" s="2" t="n"/>
@@ -2971,23 +2909,23 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050501</t>
+          <t>BCIO:050512</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention duration</t>
+          <t>median intervention temporal part duration</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3006,7 +2944,7 @@
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M44" s="2" t="n"/>
@@ -3027,23 +2965,23 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050514</t>
+          <t>BCIO:050519</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part duration</t>
+          <t>median intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -3062,7 +3000,7 @@
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M45" s="2" t="n"/>
@@ -3083,23 +3021,23 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050520</t>
+          <t>BCIO:050499</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part frequency statistic</t>
+          <t>median total intervention contact event duration</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3118,7 +3056,7 @@
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M46" s="2" t="n"/>
@@ -3139,23 +3077,23 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050503</t>
+          <t>BCIO:050513</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>minimum total intervention contact event duration</t>
+          <t>minimum intervention contact event duration</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3174,7 +3112,7 @@
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M47" s="2" t="n"/>
@@ -3195,38 +3133,32 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008515</t>
+          <t>BCIO:050500</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>minimum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is the number of contact events in a BCI temporal part.</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
-        </is>
-      </c>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="n"/>
+          <t>intervention contact event frequency statistic</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
-Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
-This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
-        </is>
-      </c>
+      <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -3236,65 +3168,53 @@
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M48" s="2" t="n"/>
       <c r="N48" s="2" t="n"/>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
+      <c r="O48" s="2" t="n"/>
       <c r="P48" s="2" t="n"/>
       <c r="Q48" s="2" t="n"/>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
+      <c r="R48" s="2" t="n"/>
       <c r="S48" s="2" t="inlineStr">
         <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
-      <c r="T48" s="2" t="inlineStr">
-        <is>
-          <t>one; 6; 12; twenty</t>
-        </is>
-      </c>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="n"/>
       <c r="U48" s="2" t="n"/>
       <c r="V48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008580</t>
+          <t>BCIO:050502</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">order of BCI temporal parts </t>
+          <t>minimum intervention contact event number</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>A &lt;BCI attribute&gt; that is the  temporal positioning of BCI temporal parts.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="n"/>
+          <t>intervention contact event number statistic</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G49" s="2" t="n"/>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>This is annotated as an open code when any aspect of order is described</t>
-        </is>
-      </c>
+      <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -3302,27 +3222,425 @@
       </c>
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
-      <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="inlineStr">
-        <is>
-          <t>BCI schedule of delivery</t>
-        </is>
-      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>number of BCI contact events</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="n"/>
       <c r="N49" s="2" t="n"/>
-      <c r="O49" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
+      <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="n"/>
       <c r="Q49" s="2" t="n"/>
       <c r="R49" s="2" t="n"/>
       <c r="S49" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="n"/>
+      <c r="U49" s="2" t="n"/>
+      <c r="V49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050501</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>minimum intervention duration</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>intervention duration statistic</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="n"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="n"/>
+      <c r="K50" s="2" t="n"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>BCI duration</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="n"/>
+      <c r="N50" s="2" t="n"/>
+      <c r="O50" s="2" t="n"/>
+      <c r="P50" s="2" t="n"/>
+      <c r="Q50" s="2" t="n"/>
+      <c r="R50" s="2" t="n"/>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="n"/>
+      <c r="U50" s="2" t="n"/>
+      <c r="V50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050514</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>minimum intervention temporal part duration</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>intervention temporal part duration statistic</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="n"/>
+      <c r="K51" s="2" t="n"/>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>BCI temporal part duration</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="n"/>
+      <c r="N51" s="2" t="n"/>
+      <c r="O51" s="2" t="n"/>
+      <c r="P51" s="2" t="n"/>
+      <c r="Q51" s="2" t="n"/>
+      <c r="R51" s="2" t="n"/>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="n"/>
+      <c r="U51" s="2" t="n"/>
+      <c r="V51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050520</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>minimum intervention temporal part frequency statistic</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>intervention temporal part frequency statistic</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="n"/>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>BCI temporal part frequency</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="n"/>
+      <c r="N52" s="2" t="n"/>
+      <c r="O52" s="2" t="n"/>
+      <c r="P52" s="2" t="n"/>
+      <c r="Q52" s="2" t="n"/>
+      <c r="R52" s="2" t="n"/>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="T52" s="2" t="n"/>
+      <c r="U52" s="2" t="n"/>
+      <c r="V52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050503</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>minimum total intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>total intervention contact event duration statistic</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="n"/>
+      <c r="K53" s="2" t="n"/>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>total BCI contact event duration</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="n"/>
+      <c r="N53" s="2" t="n"/>
+      <c r="O53" s="2" t="n"/>
+      <c r="P53" s="2" t="n"/>
+      <c r="Q53" s="2" t="n"/>
+      <c r="R53" s="2" t="n"/>
+      <c r="S53" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="T53" s="2" t="n"/>
+      <c r="U53" s="2" t="n"/>
+      <c r="V53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008515</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>number of BCI contact events</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
+Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
+This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="n"/>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="n"/>
+      <c r="N54" s="2" t="n"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="n"/>
+      <c r="Q54" s="2" t="n"/>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>one; 6; 12; twenty</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="n"/>
+      <c r="V54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051005</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>number of intervention contact events</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr"/>
+      <c r="G55" s="3" t="inlineStr"/>
+      <c r="H55" s="3" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr"/>
+      <c r="K55" s="3" t="inlineStr"/>
+      <c r="L55" s="3" t="inlineStr"/>
+      <c r="M55" s="3" t="inlineStr"/>
+      <c r="N55" s="3" t="inlineStr"/>
+      <c r="O55" s="3" t="inlineStr"/>
+      <c r="P55" s="3" t="inlineStr"/>
+      <c r="Q55" s="3" t="inlineStr"/>
+      <c r="R55" s="3" t="inlineStr"/>
+      <c r="S55" s="3" t="inlineStr"/>
+      <c r="T55" s="3" t="inlineStr"/>
+      <c r="U55" s="3" t="inlineStr"/>
+      <c r="V55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008580</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order of BCI temporal parts </t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;BCI attribute&gt; that is the  temporal positioning of BCI temporal parts.</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>BCI attribute</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>This is annotated as an open code when any aspect of order is described</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>BCI schedule of delivery</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="n"/>
+      <c r="Q56" s="2" t="n"/>
+      <c r="R56" s="2" t="n"/>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
           <t>CM; PS</t>
         </is>
       </c>
-      <c r="T49" s="2" t="inlineStr">
+      <c r="T56" s="2" t="inlineStr">
         <is>
           <t>"After questionnaires were completed, feedback was selected
 out of a database with messages for each possible combination
@@ -3331,470 +3649,470 @@
 levels to the PA guidelines."</t>
         </is>
       </c>
-      <c r="U49" s="2" t="n"/>
-      <c r="V49" s="2" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="U56" s="2" t="n"/>
+      <c r="V56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>BCIO:008595</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>q) same time (remove - this is a relation like before and after)</t>
         </is>
       </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
         </is>
       </c>
-      <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="3" t="n"/>
-      <c r="G50" s="3" t="n"/>
-      <c r="H50" s="3" t="inlineStr">
+      <c r="D57" s="4" t="n"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>This is not annotated</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J50" s="3" t="n"/>
-      <c r="K50" s="3" t="n"/>
-      <c r="L50" s="3" t="n"/>
-      <c r="M50" s="3" t="n"/>
-      <c r="N50" s="3" t="n"/>
-      <c r="O50" s="3" t="inlineStr">
+      <c r="J57" s="4" t="n"/>
+      <c r="K57" s="4" t="n"/>
+      <c r="L57" s="4" t="n"/>
+      <c r="M57" s="4" t="n"/>
+      <c r="N57" s="4" t="n"/>
+      <c r="O57" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P50" s="3" t="n"/>
-      <c r="Q50" s="3" t="n"/>
-      <c r="R50" s="3" t="n"/>
-      <c r="S50" s="3" t="inlineStr">
+      <c r="P57" s="4" t="n"/>
+      <c r="Q57" s="4" t="n"/>
+      <c r="R57" s="4" t="n"/>
+      <c r="S57" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>
       </c>
-      <c r="T50" s="3" t="n"/>
-      <c r="U50" s="3" t="n"/>
-      <c r="V50" s="3" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="T57" s="4" t="n"/>
+      <c r="U57" s="4" t="n"/>
+      <c r="V57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>BCIO:008585</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>r) before (to be removed and added to list of relations)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
         </is>
       </c>
-      <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="3" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="D58" s="4" t="n"/>
+      <c r="E58" s="4" t="n"/>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">This is not annotated </t>
         </is>
       </c>
-      <c r="I51" s="3" t="inlineStr">
+      <c r="I58" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J51" s="3" t="n"/>
-      <c r="K51" s="3" t="n"/>
-      <c r="L51" s="3" t="n"/>
-      <c r="M51" s="3" t="n"/>
-      <c r="N51" s="3" t="n"/>
-      <c r="O51" s="3" t="inlineStr">
+      <c r="J58" s="4" t="n"/>
+      <c r="K58" s="4" t="n"/>
+      <c r="L58" s="4" t="n"/>
+      <c r="M58" s="4" t="n"/>
+      <c r="N58" s="4" t="n"/>
+      <c r="O58" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P51" s="3" t="n"/>
-      <c r="Q51" s="3" t="n"/>
-      <c r="R51" s="3" t="n"/>
-      <c r="S51" s="3" t="inlineStr">
+      <c r="P58" s="4" t="n"/>
+      <c r="Q58" s="4" t="n"/>
+      <c r="R58" s="4" t="n"/>
+      <c r="S58" s="4" t="inlineStr">
         <is>
           <t>CM; RW</t>
         </is>
       </c>
-      <c r="T51" s="3" t="n"/>
-      <c r="U51" s="3" t="n"/>
-      <c r="V51" s="3" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="T58" s="4" t="n"/>
+      <c r="U58" s="4" t="n"/>
+      <c r="V58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>BCIO:008535</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>regular intervention schedule</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of a BCI or BCI part.  </t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention" </t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="n"/>
-      <c r="K52" s="2" t="n"/>
-      <c r="L52" s="2" t="n"/>
-      <c r="M52" s="2" t="n"/>
-      <c r="N52" s="2" t="n"/>
-      <c r="O52" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="n"/>
+      <c r="M59" s="2" t="n"/>
+      <c r="N59" s="2" t="n"/>
+      <c r="O59" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P52" s="2" t="n"/>
-      <c r="Q52" s="2" t="n"/>
-      <c r="R52" s="2" t="n"/>
-      <c r="S52" s="2" t="inlineStr">
+      <c r="P59" s="2" t="n"/>
+      <c r="Q59" s="2" t="n"/>
+      <c r="R59" s="2" t="n"/>
+      <c r="S59" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
-      <c r="T52" s="2" t="inlineStr">
+      <c r="T59" s="2" t="inlineStr">
         <is>
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
         </is>
       </c>
-      <c r="U52" s="2" t="n"/>
-      <c r="V52" s="2" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="U59" s="2" t="n"/>
+      <c r="V59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>BCIO:008590</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>s) after (to be removed and added to list of relations)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>A part of a BCI schedule which is the relation a specified temporal part is in when it starts following the end of another temporal part or timepoint</t>
         </is>
       </c>
-      <c r="D53" s="3" t="n"/>
-      <c r="E53" s="3" t="n"/>
-      <c r="F53" s="3" t="n"/>
-      <c r="G53" s="3" t="n"/>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="D60" s="4" t="n"/>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>This is not annotated</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
+      <c r="I60" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J53" s="3" t="n"/>
-      <c r="K53" s="3" t="n"/>
-      <c r="L53" s="3" t="n"/>
-      <c r="M53" s="3" t="n"/>
-      <c r="N53" s="3" t="n"/>
-      <c r="O53" s="3" t="inlineStr">
+      <c r="J60" s="4" t="n"/>
+      <c r="K60" s="4" t="n"/>
+      <c r="L60" s="4" t="n"/>
+      <c r="M60" s="4" t="n"/>
+      <c r="N60" s="4" t="n"/>
+      <c r="O60" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P53" s="3" t="n"/>
-      <c r="Q53" s="3" t="n"/>
-      <c r="R53" s="3" t="n"/>
-      <c r="S53" s="3" t="inlineStr">
+      <c r="P60" s="4" t="n"/>
+      <c r="Q60" s="4" t="n"/>
+      <c r="R60" s="4" t="n"/>
+      <c r="S60" s="4" t="inlineStr">
         <is>
           <t>CM; RW</t>
         </is>
       </c>
-      <c r="T53" s="3" t="n"/>
-      <c r="U53" s="3" t="n"/>
-      <c r="V53" s="3" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="T60" s="4" t="n"/>
+      <c r="U60" s="4" t="n"/>
+      <c r="V60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>BFO:0000038</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>A one-dimensional temporal region is a temporal region that is extended.</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr">
+      <c r="S61" t="inlineStr">
         <is>
           <t>JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>BCIO:050312</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">A temporal interval is a one-dimensional temporal region, namely that is self-connected (is without gaps or breaks).
 </t>
         </is>
       </c>
-      <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="D62" s="4" t="n"/>
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="F55" s="3" t="n"/>
-      <c r="G55" s="3" t="n"/>
-      <c r="H55" s="3" t="n"/>
-      <c r="I55" s="3" t="inlineStr">
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
+      <c r="I62" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J55" s="3" t="n"/>
-      <c r="K55" s="3" t="n"/>
-      <c r="L55" s="3" t="n"/>
-      <c r="M55" s="3" t="n"/>
-      <c r="N55" s="3" t="n"/>
-      <c r="O55" s="3" t="n"/>
-      <c r="P55" s="3" t="n"/>
-      <c r="Q55" s="3" t="n"/>
-      <c r="R55" s="3" t="n"/>
-      <c r="S55" s="3" t="inlineStr">
+      <c r="J62" s="4" t="n"/>
+      <c r="K62" s="4" t="n"/>
+      <c r="L62" s="4" t="n"/>
+      <c r="M62" s="4" t="n"/>
+      <c r="N62" s="4" t="n"/>
+      <c r="O62" s="4" t="n"/>
+      <c r="P62" s="4" t="n"/>
+      <c r="Q62" s="4" t="n"/>
+      <c r="R62" s="4" t="n"/>
+      <c r="S62" s="4" t="inlineStr">
         <is>
           <t>JH</t>
         </is>
       </c>
-      <c r="T55" s="3" t="n"/>
-      <c r="U55" s="3" t="n"/>
-      <c r="V55" s="3" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="T62" s="4" t="n"/>
+      <c r="U62" s="4" t="n"/>
+      <c r="V62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>BCIO:050515</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>temporal part</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>A data item between the start and end of an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="F56" s="3" t="n"/>
-      <c r="G56" s="3" t="n"/>
-      <c r="H56" s="3" t="n"/>
-      <c r="I56" s="3" t="inlineStr">
+      <c r="F63" s="4" t="n"/>
+      <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
+      <c r="I63" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J56" s="3" t="n"/>
-      <c r="K56" s="3" t="n"/>
-      <c r="L56" s="3" t="n"/>
-      <c r="M56" s="3" t="n"/>
-      <c r="N56" s="3" t="n"/>
-      <c r="O56" s="3" t="n"/>
-      <c r="P56" s="3" t="n"/>
-      <c r="Q56" s="3" t="n"/>
-      <c r="R56" s="3" t="n"/>
-      <c r="S56" s="3" t="inlineStr">
+      <c r="J63" s="4" t="n"/>
+      <c r="K63" s="4" t="n"/>
+      <c r="L63" s="4" t="n"/>
+      <c r="M63" s="4" t="n"/>
+      <c r="N63" s="4" t="n"/>
+      <c r="O63" s="4" t="n"/>
+      <c r="P63" s="4" t="n"/>
+      <c r="Q63" s="4" t="n"/>
+      <c r="R63" s="4" t="n"/>
+      <c r="S63" s="4" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="T56" s="3" t="inlineStr">
+      <c r="T63" s="4" t="inlineStr">
         <is>
           <t>6 weeks; 2 weeks</t>
         </is>
       </c>
-      <c r="U56" s="3" t="n"/>
-      <c r="V56" s="3" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="U63" s="4" t="n"/>
+      <c r="V63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>BCIO:008530</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>temporal reference associated with the intervention</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>A &lt;temporal region&gt; against which a BCI  temporal part is referenced.</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>temporal region</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>Temporal references are used by authors when there is a behaviourally relevant event which structures the schedule of a BCI. This can include things like quit dates, childbirth, medical operations etc.
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
 Example annotation in context: "A feedback call was scheduled to be delivered around 6 months after the birth of the baby".  </t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="K57" s="2" t="n"/>
-      <c r="L57" s="2" t="n"/>
-      <c r="M57" s="2" t="n"/>
-      <c r="N57" s="2" t="n"/>
-      <c r="O57" s="2" t="inlineStr">
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
+      <c r="M64" s="2" t="n"/>
+      <c r="N64" s="2" t="n"/>
+      <c r="O64" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P57" s="2" t="n"/>
-      <c r="Q57" s="2" t="n"/>
-      <c r="R57" s="2" t="n"/>
-      <c r="S57" s="2" t="inlineStr">
+      <c r="P64" s="2" t="n"/>
+      <c r="Q64" s="2" t="n"/>
+      <c r="R64" s="2" t="n"/>
+      <c r="S64" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
-      <c r="T57" s="2" t="inlineStr">
+      <c r="T64" s="2" t="inlineStr">
         <is>
           <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
         </is>
       </c>
-      <c r="U57" s="2" t="n"/>
-      <c r="V57" s="2" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="U64" s="2" t="n"/>
+      <c r="V64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>BCIO:008545</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>The planned total duration of all sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="F58" s="2" t="n"/>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>"is about" contact events or "is about" duration of contact events?</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
 When there is only one session, the total duration of contact events and the duration of a single contact event are technically the same. As a convention, we would annotate this using duration of contact event instead of total duration of contact event. 
@@ -3802,518 +4120,562 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="n"/>
-      <c r="K58" s="2" t="n"/>
-      <c r="L58" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="inlineStr">
         <is>
           <t>BCI contact event</t>
         </is>
       </c>
-      <c r="M58" s="2" t="n"/>
-      <c r="N58" s="2" t="n"/>
-      <c r="O58" s="2" t="inlineStr">
+      <c r="M65" s="2" t="n"/>
+      <c r="N65" s="2" t="n"/>
+      <c r="O65" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P58" s="2" t="n"/>
-      <c r="Q58" s="2" t="inlineStr">
+      <c r="P65" s="2" t="n"/>
+      <c r="Q65" s="2" t="inlineStr">
         <is>
           <t>what type of data item is this? (CM)</t>
         </is>
       </c>
-      <c r="R58" s="2" t="inlineStr">
+      <c r="R65" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S58" s="2" t="inlineStr">
+      <c r="S65" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
-      <c r="T58" s="2" t="inlineStr">
+      <c r="T65" s="2" t="inlineStr">
         <is>
           <t>150 minutes; 12 hours</t>
         </is>
       </c>
-      <c r="U58" s="2" t="n"/>
-      <c r="V58" s="2" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="U65" s="2" t="n"/>
+      <c r="V65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051006</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>total intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr"/>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr"/>
+      <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr"/>
+      <c r="N66" s="3" t="inlineStr"/>
+      <c r="O66" s="3" t="inlineStr"/>
+      <c r="P66" s="3" t="inlineStr"/>
+      <c r="Q66" s="3" t="inlineStr"/>
+      <c r="R66" s="3" t="inlineStr"/>
+      <c r="S66" s="3" t="inlineStr"/>
+      <c r="T66" s="3" t="inlineStr"/>
+      <c r="U66" s="3" t="inlineStr"/>
+      <c r="V66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>BCIO:050504</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="n"/>
-      <c r="H59" s="2" t="n"/>
-      <c r="I59" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="J59" s="2" t="n"/>
-      <c r="K59" s="2" t="n"/>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="n"/>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="M59" s="2" t="n"/>
-      <c r="N59" s="2" t="n"/>
-      <c r="O59" s="2" t="n"/>
-      <c r="P59" s="2" t="n"/>
-      <c r="Q59" s="2" t="n"/>
-      <c r="R59" s="2" t="n"/>
-      <c r="S59" s="2" t="inlineStr">
+      <c r="M67" s="2" t="n"/>
+      <c r="N67" s="2" t="n"/>
+      <c r="O67" s="2" t="n"/>
+      <c r="P67" s="2" t="n"/>
+      <c r="Q67" s="2" t="n"/>
+      <c r="R67" s="2" t="n"/>
+      <c r="S67" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="T59" s="2" t="n"/>
-      <c r="U59" s="2" t="n"/>
-      <c r="V59" s="2" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="T67" s="2" t="n"/>
+      <c r="U67" s="2" t="n"/>
+      <c r="V67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>BCIO:008605</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
         </is>
       </c>
-      <c r="D60" s="3" t="n"/>
-      <c r="E60" s="3" t="n"/>
-      <c r="F60" s="3" t="n"/>
-      <c r="G60" s="3" t="n"/>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="D68" s="4" t="n"/>
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
         </is>
       </c>
-      <c r="I60" s="3" t="inlineStr">
+      <c r="I68" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J60" s="3" t="n"/>
-      <c r="K60" s="3" t="n"/>
-      <c r="L60" s="3" t="inlineStr">
+      <c r="J68" s="4" t="n"/>
+      <c r="K68" s="4" t="n"/>
+      <c r="L68" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M60" s="3" t="n"/>
-      <c r="N60" s="3" t="n"/>
-      <c r="O60" s="3" t="inlineStr">
+      <c r="M68" s="4" t="n"/>
+      <c r="N68" s="4" t="n"/>
+      <c r="O68" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P60" s="3" t="n"/>
-      <c r="Q60" s="3" t="inlineStr">
+      <c r="P68" s="4" t="n"/>
+      <c r="Q68" s="4" t="inlineStr">
         <is>
           <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
         </is>
       </c>
-      <c r="R60" s="3" t="inlineStr">
+      <c r="R68" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S60" s="3" t="inlineStr">
+      <c r="S68" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>
       </c>
-      <c r="T60" s="3" t="inlineStr">
+      <c r="T68" s="4" t="inlineStr">
         <is>
           <t>Participants received "3" emails every 2 weeks</t>
         </is>
       </c>
-      <c r="U60" s="3" t="n"/>
-      <c r="V60" s="3" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+      <c r="U68" s="4" t="n"/>
+      <c r="V68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>BCIO:008550</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>z) contact event sum duration (still to confirm inclusion)</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
         </is>
       </c>
-      <c r="D61" s="3" t="n"/>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="D69" s="4" t="n"/>
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F61" s="3" t="n"/>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="F69" s="4" t="n"/>
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>is about contact events or is about duration of contact events?</t>
         </is>
       </c>
-      <c r="H61" s="3" t="inlineStr">
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
         </is>
       </c>
-      <c r="I61" s="3" t="inlineStr">
+      <c r="I69" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J61" s="3" t="n"/>
-      <c r="K61" s="3" t="n"/>
-      <c r="L61" s="3" t="inlineStr">
+      <c r="J69" s="4" t="n"/>
+      <c r="K69" s="4" t="n"/>
+      <c r="L69" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M61" s="3" t="n"/>
-      <c r="N61" s="3" t="n"/>
-      <c r="O61" s="3" t="inlineStr">
+      <c r="M69" s="4" t="n"/>
+      <c r="N69" s="4" t="n"/>
+      <c r="O69" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P61" s="3" t="n"/>
-      <c r="Q61" s="3" t="inlineStr">
+      <c r="P69" s="4" t="n"/>
+      <c r="Q69" s="4" t="inlineStr">
         <is>
           <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
-      <c r="R61" s="3" t="inlineStr">
+      <c r="R69" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S61" s="3" t="inlineStr">
+      <c r="S69" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>
       </c>
-      <c r="T61" s="3" t="inlineStr">
+      <c r="T69" s="4" t="inlineStr">
         <is>
           <t>The participants took part in "90" minutes of PA weekly</t>
         </is>
       </c>
-      <c r="U61" s="3" t="n"/>
-      <c r="V61" s="3" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="U69" s="4" t="n"/>
+      <c r="V69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>BCIO:008555</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
         </is>
       </c>
-      <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="D70" s="4" t="n"/>
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F62" s="3" t="n"/>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>is about contact events or is about duration of contact events?</t>
         </is>
       </c>
-      <c r="H62" s="3" t="inlineStr">
+      <c r="H70" s="4" t="inlineStr">
         <is>
           <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
         </is>
       </c>
-      <c r="I62" s="3" t="inlineStr">
+      <c r="I70" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J62" s="3" t="n"/>
-      <c r="K62" s="3" t="n"/>
-      <c r="L62" s="3" t="inlineStr">
+      <c r="J70" s="4" t="n"/>
+      <c r="K70" s="4" t="n"/>
+      <c r="L70" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M62" s="3" t="n"/>
-      <c r="N62" s="3" t="n"/>
-      <c r="O62" s="3" t="inlineStr">
+      <c r="M70" s="4" t="n"/>
+      <c r="N70" s="4" t="n"/>
+      <c r="O70" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P62" s="3" t="n"/>
-      <c r="Q62" s="3" t="inlineStr">
+      <c r="P70" s="4" t="n"/>
+      <c r="Q70" s="4" t="inlineStr">
         <is>
           <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
-      <c r="R62" s="3" t="inlineStr">
+      <c r="R70" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S62" s="3" t="inlineStr">
+      <c r="S70" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>
       </c>
-      <c r="T62" s="3" t="inlineStr">
+      <c r="T70" s="4" t="inlineStr">
         <is>
           <t>The participants took part in 90 minutes of PA "weekly"</t>
         </is>
       </c>
-      <c r="U62" s="3" t="n"/>
-      <c r="V62" s="3" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+      <c r="U70" s="4" t="n"/>
+      <c r="V70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>BCIO:008600</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>z) frequency period</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
         </is>
       </c>
-      <c r="D63" s="3" t="n"/>
-      <c r="E63" s="3" t="inlineStr">
+      <c r="D71" s="4" t="n"/>
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
         </is>
       </c>
-      <c r="F63" s="3" t="n"/>
-      <c r="G63" s="3" t="n"/>
-      <c r="H63" s="3" t="n"/>
-      <c r="I63" s="3" t="inlineStr">
+      <c r="F71" s="4" t="n"/>
+      <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
+      <c r="I71" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J63" s="3" t="n"/>
-      <c r="K63" s="3" t="n"/>
-      <c r="L63" s="3" t="inlineStr">
+      <c r="J71" s="4" t="n"/>
+      <c r="K71" s="4" t="n"/>
+      <c r="L71" s="4" t="inlineStr">
         <is>
           <t>intervention temporal part</t>
         </is>
       </c>
-      <c r="M63" s="3" t="n"/>
-      <c r="N63" s="3" t="n"/>
-      <c r="O63" s="3" t="inlineStr">
+      <c r="M71" s="4" t="n"/>
+      <c r="N71" s="4" t="n"/>
+      <c r="O71" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P63" s="3" t="n"/>
-      <c r="Q63" s="3" t="inlineStr">
+      <c r="P71" s="4" t="n"/>
+      <c r="Q71" s="4" t="inlineStr">
         <is>
           <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
         </is>
       </c>
-      <c r="R63" s="3" t="inlineStr">
+      <c r="R71" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S63" s="3" t="inlineStr">
+      <c r="S71" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>
       </c>
-      <c r="T63" s="3" t="inlineStr">
+      <c r="T71" s="4" t="inlineStr">
         <is>
           <t>Participants received 3 emails every "2" weeks</t>
         </is>
       </c>
-      <c r="U63" s="3" t="n"/>
-      <c r="V63" s="3" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+      <c r="U71" s="4" t="n"/>
+      <c r="V71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>BCIO:008570</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>z) interval (remove)</t>
         </is>
       </c>
-      <c r="C64" s="3" t="n"/>
-      <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
-      <c r="F64" s="3" t="n"/>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="C72" s="4" t="n"/>
+      <c r="D72" s="4" t="n"/>
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="n"/>
+      <c r="G72" s="4" t="inlineStr">
         <is>
           <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr">
+      <c r="H72" s="4" t="inlineStr">
         <is>
           <t>This is not annotated but included due to relationship with duration of interval</t>
         </is>
       </c>
-      <c r="I64" s="3" t="inlineStr">
+      <c r="I72" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J64" s="3" t="n"/>
-      <c r="K64" s="3" t="n"/>
-      <c r="L64" s="3" t="n"/>
-      <c r="M64" s="3" t="n"/>
-      <c r="N64" s="3" t="n"/>
-      <c r="O64" s="3" t="inlineStr">
+      <c r="J72" s="4" t="n"/>
+      <c r="K72" s="4" t="n"/>
+      <c r="L72" s="4" t="n"/>
+      <c r="M72" s="4" t="n"/>
+      <c r="N72" s="4" t="n"/>
+      <c r="O72" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P64" s="3" t="n"/>
-      <c r="Q64" s="3" t="n"/>
-      <c r="R64" s="3" t="n"/>
-      <c r="S64" s="3" t="inlineStr">
+      <c r="P72" s="4" t="n"/>
+      <c r="Q72" s="4" t="n"/>
+      <c r="R72" s="4" t="n"/>
+      <c r="S72" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>
       </c>
-      <c r="T64" s="3" t="n"/>
-      <c r="U64" s="3" t="n"/>
-      <c r="V64" s="3" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="T72" s="4" t="n"/>
+      <c r="U72" s="4" t="n"/>
+      <c r="V72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>BCIO:008520</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>z) intervention temporal part frequency</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
         </is>
       </c>
-      <c r="D65" s="3" t="n"/>
-      <c r="E65" s="3" t="inlineStr">
+      <c r="D73" s="4" t="n"/>
+      <c r="E73" s="4" t="inlineStr">
         <is>
           <t>process attribute</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr">
+      <c r="F73" s="4" t="inlineStr">
         <is>
           <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
         </is>
       </c>
-      <c r="G65" s="3" t="n"/>
-      <c r="H65" s="3" t="inlineStr">
+      <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="inlineStr">
         <is>
           <t>This is used to capture descriptions of the frequency of contact events within a part. 
 Example annotation (in context)
 intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks"</t>
         </is>
       </c>
-      <c r="I65" s="3" t="inlineStr">
+      <c r="I73" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="J65" s="3" t="n"/>
-      <c r="K65" s="3" t="n"/>
-      <c r="L65" s="3" t="inlineStr">
+      <c r="J73" s="4" t="n"/>
+      <c r="K73" s="4" t="n"/>
+      <c r="L73" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M65" s="3" t="n"/>
-      <c r="N65" s="3" t="n"/>
-      <c r="O65" s="3" t="inlineStr">
+      <c r="M73" s="4" t="n"/>
+      <c r="N73" s="4" t="n"/>
+      <c r="O73" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P65" s="3" t="n"/>
-      <c r="Q65" s="3" t="inlineStr">
+      <c r="P73" s="4" t="n"/>
+      <c r="Q73" s="4" t="inlineStr">
         <is>
           <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
         </is>
       </c>
-      <c r="R65" s="3" t="inlineStr">
+      <c r="R73" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S65" s="3" t="inlineStr">
+      <c r="S73" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>
       </c>
-      <c r="T65" s="3" t="n"/>
-      <c r="U65" s="3" t="n"/>
-      <c r="V65" s="3" t="n"/>
+      <c r="T73" s="4" t="n"/>
+      <c r="U73" s="4" t="n"/>
+      <c r="V73" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added class "intervention temporal part"
Added the class "intervention temporal part" to be an intervention level equivalent of the "BCI temporal" part class. Discussed in April 2026 Beh Sci meeting
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micas\OneDrive\Documentos\GitHub\ontologies\Schedule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A52A82-8FB4-4ED1-99E3-1FF519D69D53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191D85E7-B3C3-46C7-B98F-5992FED53AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$V$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$V$74</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="329">
   <si>
     <t>ID</t>
   </si>
@@ -1033,6 +1033,9 @@
   </si>
   <si>
     <t>An &lt;intervention contact event frequency&gt; about the number times a BCI contact event occurs per unit of time.</t>
+  </si>
+  <si>
+    <t>A &lt;planned process&gt; that is a part of an intervention.</t>
   </si>
 </sst>
 </file>
@@ -1088,12 +1091,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1396,8 +1400,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V73"/>
+  <dimension ref="A1:V74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="32.59765625" customWidth="1"/>
+    <col min="10" max="10" width="24.59765625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
@@ -4365,7 +4373,20 @@
       <c r="U73" s="4"/>
       <c r="V73" s="4"/>
     </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="B74" t="s">
+        <v>308</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E74" t="s">
+        <v>58</v>
+      </c>
+      <c r="I74" s="5"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:V74" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add intervention contact event to BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V74"/>
+  <dimension ref="A1:V75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1272,217 +1272,205 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>BCIO:051009</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr"/>
+      <c r="S14" s="3" t="inlineStr"/>
+      <c r="T14" s="3" t="inlineStr"/>
+      <c r="U14" s="3" t="inlineStr"/>
+      <c r="V14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>BCIO:051000</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>intervention contact event duration</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="inlineStr">
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
+      <c r="N15" s="3" t="n"/>
+      <c r="O15" s="3" t="n"/>
+      <c r="P15" s="3" t="n"/>
+      <c r="Q15" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3" t="n"/>
-      <c r="T14" s="3" t="n"/>
-      <c r="U14" s="3" t="n"/>
-      <c r="V14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="R15" s="3" t="n"/>
+      <c r="S15" s="3" t="n"/>
+      <c r="T15" s="3" t="n"/>
+      <c r="U15" s="3" t="n"/>
+      <c r="V15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>BCIO:050505</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>intervention contact event duration statistic</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of intervention contact event durations.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>BCI contact event duration</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="n"/>
-      <c r="O15" s="2" t="n"/>
-      <c r="P15" s="2" t="n"/>
-      <c r="Q15" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R15" s="2" t="n"/>
-      <c r="S15" s="2" t="n"/>
-      <c r="T15" s="2" t="n"/>
-      <c r="U15" s="2" t="n"/>
-      <c r="V15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="n"/>
+      <c r="S16" s="2" t="n"/>
+      <c r="T16" s="2" t="n"/>
+      <c r="U16" s="2" t="n"/>
+      <c r="V16" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>BCIO:051001</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>intervention contact event frequency</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="3" t="n"/>
-      <c r="Q16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="n"/>
+      <c r="P17" s="3" t="n"/>
+      <c r="Q17" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R16" s="3" t="n"/>
-      <c r="S16" s="3" t="n"/>
-      <c r="T16" s="3" t="n"/>
-      <c r="U16" s="3" t="n"/>
-      <c r="V16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050903</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event frequency statistic</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event frequency</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="n"/>
-      <c r="Q17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R17" s="2" t="n"/>
-      <c r="S17" s="2" t="n"/>
-      <c r="T17" s="2" t="n"/>
-      <c r="U17" s="2" t="n"/>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="R17" s="3" t="n"/>
+      <c r="S17" s="3" t="n"/>
+      <c r="T17" s="3" t="n"/>
+      <c r="U17" s="3" t="n"/>
+      <c r="V17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050904</t>
+          <t>BCIO:050903</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -1503,7 +1491,7 @@
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M18" s="2" t="n"/>
@@ -1526,134 +1514,142 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050904</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>intervention contact event number statistic</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>number of BCI contact events</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="n"/>
+      <c r="S19" s="2" t="n"/>
+      <c r="T19" s="2" t="n"/>
+      <c r="U19" s="2" t="n"/>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>BCIO:051002</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>intervention duration</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3" t="n"/>
-      <c r="O19" s="3" t="n"/>
-      <c r="P19" s="3" t="n"/>
-      <c r="Q19" s="3" t="inlineStr">
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="3" t="n"/>
+      <c r="N20" s="3" t="n"/>
+      <c r="O20" s="3" t="n"/>
+      <c r="P20" s="3" t="n"/>
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R19" s="3" t="n"/>
-      <c r="S19" s="3" t="n"/>
-      <c r="T19" s="3" t="n"/>
-      <c r="U19" s="3" t="n"/>
-      <c r="V19" s="3" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050905</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>intervention duration statistic</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>BCI duration</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R20" s="2" t="n"/>
-      <c r="S20" s="2" t="n"/>
-      <c r="T20" s="2" t="n"/>
-      <c r="U20" s="2" t="n"/>
-      <c r="V20" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="R20" s="3" t="n"/>
+      <c r="S20" s="3" t="n"/>
+      <c r="T20" s="3" t="n"/>
+      <c r="U20" s="3" t="n"/>
+      <c r="V20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>BCIO:051008</t>
+          <t>BCIO:050905</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>A &lt;planned process&gt; that is a part of an intervention.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="n"/>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>BCI duration</t>
+        </is>
+      </c>
       <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
@@ -1667,254 +1663,241 @@
       <c r="S21" s="2" t="n"/>
       <c r="T21" s="2" t="n"/>
       <c r="U21" s="2" t="n"/>
-      <c r="V21" s="2" t="n"/>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:051008</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;planned process&gt; that is a part of an intervention.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2" t="n"/>
+      <c r="P22" s="2" t="n"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="n"/>
+      <c r="S22" s="2" t="n"/>
+      <c r="T22" s="2" t="n"/>
+      <c r="U22" s="2" t="n"/>
+      <c r="V22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>BCIO:051003</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>intervention temporal part duration</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; between the start and end of an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="n"/>
-      <c r="Q22" s="3" t="inlineStr">
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="n"/>
+      <c r="O23" s="3" t="n"/>
+      <c r="P23" s="3" t="n"/>
+      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R22" s="3" t="n"/>
-      <c r="S22" s="3" t="n"/>
-      <c r="T22" s="3" t="n"/>
-      <c r="U22" s="3" t="n"/>
-      <c r="V22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="R23" s="3" t="n"/>
+      <c r="S23" s="3" t="n"/>
+      <c r="T23" s="3" t="n"/>
+      <c r="U23" s="3" t="n"/>
+      <c r="V23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>BCIO:050506</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part duration statistic</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of intervention temporal part durations.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>BCI temporal part duration</t>
         </is>
       </c>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R23" s="2" t="n"/>
-      <c r="S23" s="2" t="n"/>
-      <c r="T23" s="2" t="n"/>
-      <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="inlineStr">
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
+      <c r="O24" s="2" t="n"/>
+      <c r="P24" s="2" t="n"/>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="n"/>
+      <c r="S24" s="2" t="n"/>
+      <c r="T24" s="2" t="n"/>
+      <c r="U24" s="2" t="n"/>
+      <c r="V24" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>BCIO:051004</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>intervention temporal part frequency</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is how often intervention temporal parts occur within an intervention.</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">This is useful when grouping contact events together to the schedule of an intervention. For example, authors may describe participants as taking part in 90 minutes of physical activity weekly. These 90 minutes could be split across several contact events, however together these contact events form an intervention part which occurs weekly. </t>
         </is>
       </c>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
-      <c r="O24" s="3" t="n"/>
-      <c r="P24" s="3" t="n"/>
-      <c r="Q24" s="3" t="inlineStr">
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+      <c r="N25" s="3" t="n"/>
+      <c r="O25" s="3" t="n"/>
+      <c r="P25" s="3" t="n"/>
+      <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R24" s="3" t="n"/>
-      <c r="S24" s="3" t="n"/>
-      <c r="T24" s="3" t="n"/>
-      <c r="U24" s="3" t="n"/>
-      <c r="V24" s="3" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050516</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>intervention temporal part frequency statistic</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention temporal part frequencies.</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>BCI temporal part frequency</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="n"/>
-      <c r="Q25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R25" s="2" t="n"/>
-      <c r="S25" s="2" t="n"/>
-      <c r="T25" s="2" t="n"/>
-      <c r="U25" s="2" t="n"/>
-      <c r="V25" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="R25" s="3" t="n"/>
+      <c r="S25" s="3" t="n"/>
+      <c r="T25" s="3" t="n"/>
+      <c r="U25" s="3" t="n"/>
+      <c r="V25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008540</t>
+          <t>BCIO:050516</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>irregular intervention schedule</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or BCI.  </t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
-        </is>
-      </c>
+          <t>A &lt;data item&gt; that is about a collection of intervention temporal part frequencies.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="n"/>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
-Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks" </t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
-        </is>
-      </c>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>BCI temporal part frequency</t>
+        </is>
+      </c>
       <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
@@ -1925,60 +1908,57 @@
         </is>
       </c>
       <c r="R26" s="2" t="n"/>
-      <c r="S26" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T26" s="2" t="inlineStr">
-        <is>
-          <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
-        </is>
-      </c>
+      <c r="S26" s="2" t="n"/>
+      <c r="T26" s="2" t="n"/>
       <c r="U26" s="2" t="n"/>
       <c r="V26" s="2" t="inlineStr">
         <is>
-          <t>CM; JH; PS</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050507</t>
+          <t>BCIO:008540</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event duration</t>
+          <t>irregular intervention schedule</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="n"/>
+          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or BCI.  </t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
+          <t>BCI schedule of delivery</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
+Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks" </t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event duration</t>
-        </is>
-      </c>
+      <c r="L27" s="2" t="n"/>
       <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
@@ -1989,35 +1969,43 @@
         </is>
       </c>
       <c r="R27" s="2" t="n"/>
-      <c r="S27" s="2" t="n"/>
-      <c r="T27" s="2" t="n"/>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
+        </is>
+      </c>
       <c r="U27" s="2" t="n"/>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050906</t>
+          <t>BCIO:050507</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event frequency</t>
+          <t>maximum intervention contact event duration</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2032,7 +2020,7 @@
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M28" s="2" t="n"/>
@@ -2057,23 +2045,23 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050907</t>
+          <t>BCIO:050906</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event number</t>
+          <t>maximum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2088,7 +2076,7 @@
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M29" s="2" t="n"/>
@@ -2113,23 +2101,23 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050908</t>
+          <t>BCIO:050907</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention duration</t>
+          <t>maximum intervention contact event number</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2144,7 +2132,7 @@
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M30" s="2" t="n"/>
@@ -2169,23 +2157,23 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050508</t>
+          <t>BCIO:050908</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part duration</t>
+          <t>maximum intervention duration</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2200,7 +2188,7 @@
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M31" s="2" t="n"/>
@@ -2225,23 +2213,23 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050517</t>
+          <t>BCIO:050508</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part frequency statistic</t>
+          <t>maximum intervention temporal part duration</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2256,7 +2244,7 @@
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M32" s="2" t="n"/>
@@ -2281,23 +2269,23 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050910</t>
+          <t>BCIO:050517</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>maximum total intervention contact event duration</t>
+          <t>maximum intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2312,7 +2300,7 @@
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M33" s="2" t="n"/>
@@ -2337,23 +2325,23 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050509</t>
+          <t>BCIO:050910</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event duration</t>
+          <t>maximum total intervention contact event duration</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2368,7 +2356,7 @@
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M34" s="2" t="n"/>
@@ -2393,23 +2381,23 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050911</t>
+          <t>BCIO:050509</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event frequency</t>
+          <t>mean intervention contact event duration</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2424,7 +2412,7 @@
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M35" s="2" t="n"/>
@@ -2449,23 +2437,23 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050912</t>
+          <t>BCIO:050911</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event number</t>
+          <t>mean intervention contact event frequency</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2480,7 +2468,7 @@
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M36" s="2" t="n"/>
@@ -2505,23 +2493,23 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050909</t>
+          <t>BCIO:050912</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>mean intervention duration</t>
+          <t>mean intervention contact event number</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2536,7 +2524,7 @@
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M37" s="2" t="n"/>
@@ -2561,23 +2549,23 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050510</t>
+          <t>BCIO:050909</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part duration</t>
+          <t>mean intervention duration</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2592,7 +2580,7 @@
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M38" s="2" t="n"/>
@@ -2617,23 +2605,23 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050518</t>
+          <t>BCIO:050510</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part frequency statistic</t>
+          <t>mean intervention temporal part duration</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2648,7 +2636,7 @@
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M39" s="2" t="n"/>
@@ -2673,23 +2661,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050495</t>
+          <t>BCIO:050518</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>mean total intervention contact event duration</t>
+          <t>mean intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2704,7 +2692,7 @@
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M40" s="2" t="n"/>
@@ -2729,23 +2717,23 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050511</t>
+          <t>BCIO:050495</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event duration</t>
+          <t>mean total intervention contact event duration</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2760,7 +2748,7 @@
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M41" s="2" t="n"/>
@@ -2785,23 +2773,23 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050496</t>
+          <t>BCIO:050511</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event frequency</t>
+          <t>median intervention contact event duration</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2816,7 +2804,7 @@
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M42" s="2" t="n"/>
@@ -2841,23 +2829,23 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050497</t>
+          <t>BCIO:050496</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event number</t>
+          <t>median intervention contact event frequency</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2872,7 +2860,7 @@
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M43" s="2" t="n"/>
@@ -2897,23 +2885,23 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050498</t>
+          <t>BCIO:050497</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>median intervention duration</t>
+          <t>median intervention contact event number</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2928,7 +2916,7 @@
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M44" s="2" t="n"/>
@@ -2953,23 +2941,23 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050512</t>
+          <t>BCIO:050498</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part duration</t>
+          <t>median intervention duration</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2984,7 +2972,7 @@
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M45" s="2" t="n"/>
@@ -3009,23 +2997,23 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050519</t>
+          <t>BCIO:050512</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part frequency statistic</t>
+          <t>median intervention temporal part duration</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3040,7 +3028,7 @@
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M46" s="2" t="n"/>
@@ -3065,23 +3053,23 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050499</t>
+          <t>BCIO:050519</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>median total intervention contact event duration</t>
+          <t>median intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3096,7 +3084,7 @@
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M47" s="2" t="n"/>
@@ -3121,23 +3109,23 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050513</t>
+          <t>BCIO:050499</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event duration</t>
+          <t>median total intervention contact event duration</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3152,7 +3140,7 @@
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M48" s="2" t="n"/>
@@ -3177,23 +3165,23 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050500</t>
+          <t>BCIO:050513</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event frequency</t>
+          <t>minimum intervention contact event duration</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3208,7 +3196,7 @@
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M49" s="2" t="n"/>
@@ -3233,23 +3221,23 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050502</t>
+          <t>BCIO:050500</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event number</t>
+          <t>minimum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3264,7 +3252,7 @@
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M50" s="2" t="n"/>
@@ -3289,23 +3277,23 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050501</t>
+          <t>BCIO:050502</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention duration</t>
+          <t>minimum intervention contact event number</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3320,7 +3308,7 @@
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M51" s="2" t="n"/>
@@ -3345,23 +3333,23 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050514</t>
+          <t>BCIO:050501</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part duration</t>
+          <t>minimum intervention duration</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3376,7 +3364,7 @@
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M52" s="2" t="n"/>
@@ -3401,23 +3389,23 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050520</t>
+          <t>BCIO:050514</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part frequency statistic</t>
+          <t>minimum intervention temporal part duration</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3432,7 +3420,7 @@
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M53" s="2" t="n"/>
@@ -3457,23 +3445,23 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050503</t>
+          <t>BCIO:050520</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>minimum total intervention contact event duration</t>
+          <t>minimum intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3488,7 +3476,7 @@
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M54" s="2" t="n"/>
@@ -3513,48 +3501,38 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008515</t>
+          <t>BCIO:050503</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>minimum total intervention contact event duration</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
-        </is>
-      </c>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>number of intervention contact events</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="n"/>
+          <t>total intervention contact event duration statistic</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G55" s="2" t="n"/>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
-Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
-This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>one; 6; 12; twenty</t>
-        </is>
-      </c>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="n"/>
       <c r="J55" s="2" t="n"/>
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M55" s="2" t="n"/>
@@ -3566,98 +3544,164 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="R55" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S55" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
+      <c r="R55" s="2" t="n"/>
+      <c r="S55" s="2" t="n"/>
       <c r="T55" s="2" t="n"/>
       <c r="U55" s="2" t="n"/>
       <c r="V55" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008515</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>number of BCI contact events</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>number of intervention contact events</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
+Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
+This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>one; 6; 12; twenty</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="n"/>
+      <c r="N56" s="2" t="n"/>
+      <c r="O56" s="2" t="n"/>
+      <c r="P56" s="2" t="n"/>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="n"/>
+      <c r="U56" s="2" t="n"/>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>BCIO:051005</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>number of intervention contact events</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="D57" s="3" t="n"/>
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F56" s="3" t="n"/>
-      <c r="G56" s="3" t="n"/>
-      <c r="H56" s="3" t="n"/>
-      <c r="I56" s="3" t="n"/>
-      <c r="J56" s="3" t="n"/>
-      <c r="K56" s="3" t="n"/>
-      <c r="L56" s="3" t="n"/>
-      <c r="M56" s="3" t="n"/>
-      <c r="N56" s="3" t="n"/>
-      <c r="O56" s="3" t="n"/>
-      <c r="P56" s="3" t="n"/>
-      <c r="Q56" s="3" t="inlineStr">
+      <c r="F57" s="3" t="n"/>
+      <c r="G57" s="3" t="n"/>
+      <c r="H57" s="3" t="n"/>
+      <c r="I57" s="3" t="n"/>
+      <c r="J57" s="3" t="n"/>
+      <c r="K57" s="3" t="n"/>
+      <c r="L57" s="3" t="n"/>
+      <c r="M57" s="3" t="n"/>
+      <c r="N57" s="3" t="n"/>
+      <c r="O57" s="3" t="n"/>
+      <c r="P57" s="3" t="n"/>
+      <c r="Q57" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R56" s="3" t="n"/>
-      <c r="S56" s="3" t="n"/>
-      <c r="T56" s="3" t="n"/>
-      <c r="U56" s="3" t="n"/>
-      <c r="V56" s="3" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="R57" s="3" t="n"/>
+      <c r="S57" s="3" t="n"/>
+      <c r="T57" s="3" t="n"/>
+      <c r="U57" s="3" t="n"/>
+      <c r="V57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>BCIO:008580</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">order of BCI temporal parts </t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>A &lt;BCI attribute&gt; that is the  temporal positioning of BCI temporal parts.</t>
         </is>
       </c>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>BCI attribute</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n"/>
-      <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>This is annotated as an open code when any aspect of order is described</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>"After questionnaires were completed, feedback was selected
 out of a database with messages for each possible combination
@@ -3666,102 +3710,50 @@
 levels to the PA guidelines."</t>
         </is>
       </c>
-      <c r="J57" s="2" t="n"/>
-      <c r="K57" s="2" t="n"/>
-      <c r="L57" s="2" t="n"/>
-      <c r="M57" s="2" t="inlineStr">
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="n"/>
+      <c r="M58" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="N57" s="2" t="n"/>
-      <c r="O57" s="2" t="n"/>
-      <c r="P57" s="2" t="n"/>
-      <c r="Q57" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R57" s="2" t="n"/>
-      <c r="S57" s="2" t="inlineStr">
+      <c r="N58" s="2" t="n"/>
+      <c r="O58" s="2" t="n"/>
+      <c r="P58" s="2" t="n"/>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="n"/>
+      <c r="S58" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T57" s="2" t="n"/>
-      <c r="U57" s="2" t="n"/>
-      <c r="V57" s="2" t="inlineStr">
+      <c r="T58" s="2" t="n"/>
+      <c r="U58" s="2" t="n"/>
+      <c r="V58" s="2" t="inlineStr">
         <is>
           <t>CM; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008595</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>q) same time (remove - this is a relation like before and after)</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated</t>
-        </is>
-      </c>
-      <c r="I58" s="4" t="n"/>
-      <c r="J58" s="4" t="n"/>
-      <c r="K58" s="4" t="n"/>
-      <c r="L58" s="4" t="n"/>
-      <c r="M58" s="4" t="n"/>
-      <c r="N58" s="4" t="n"/>
-      <c r="O58" s="4" t="n"/>
-      <c r="P58" s="4" t="n"/>
-      <c r="Q58" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R58" s="4" t="n"/>
-      <c r="S58" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T58" s="4" t="n"/>
-      <c r="U58" s="4" t="n"/>
-      <c r="V58" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008585</t>
+          <t>BCIO:008595</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>r) before (to be removed and added to list of relations)</t>
+          <t>q) same time (remove - this is a relation like before and after)</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
         </is>
       </c>
       <c r="D59" s="4" t="n"/>
@@ -3770,7 +3762,7 @@
       <c r="G59" s="4" t="n"/>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is not annotated </t>
+          <t>This is not annotated</t>
         </is>
       </c>
       <c r="I59" s="4" t="n"/>
@@ -3796,222 +3788,226 @@
       <c r="U59" s="4" t="n"/>
       <c r="V59" s="4" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008585</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>r) before (to be removed and added to list of relations)</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="n"/>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is not annotated </t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="n"/>
+      <c r="J60" s="4" t="n"/>
+      <c r="K60" s="4" t="n"/>
+      <c r="L60" s="4" t="n"/>
+      <c r="M60" s="4" t="n"/>
+      <c r="N60" s="4" t="n"/>
+      <c r="O60" s="4" t="n"/>
+      <c r="P60" s="4" t="n"/>
+      <c r="Q60" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R60" s="4" t="n"/>
+      <c r="S60" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T60" s="4" t="n"/>
+      <c r="U60" s="4" t="n"/>
+      <c r="V60" s="4" t="inlineStr">
+        <is>
           <t>CM; RW</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>BCIO:008535</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>regular intervention schedule</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of a BCI or BCI part.  </t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="F60" s="2" t="n"/>
-      <c r="G60" s="2" t="n"/>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention" </t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
         </is>
       </c>
-      <c r="J60" s="2" t="n"/>
-      <c r="K60" s="2" t="n"/>
-      <c r="L60" s="2" t="n"/>
-      <c r="M60" s="2" t="n"/>
-      <c r="N60" s="2" t="n"/>
-      <c r="O60" s="2" t="n"/>
-      <c r="P60" s="2" t="n"/>
-      <c r="Q60" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R60" s="2" t="n"/>
-      <c r="S60" s="2" t="inlineStr">
+      <c r="J61" s="2" t="n"/>
+      <c r="K61" s="2" t="n"/>
+      <c r="L61" s="2" t="n"/>
+      <c r="M61" s="2" t="n"/>
+      <c r="N61" s="2" t="n"/>
+      <c r="O61" s="2" t="n"/>
+      <c r="P61" s="2" t="n"/>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="n"/>
+      <c r="S61" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T60" s="2" t="n"/>
-      <c r="U60" s="2" t="n"/>
-      <c r="V60" s="2" t="inlineStr">
+      <c r="T61" s="2" t="n"/>
+      <c r="U61" s="2" t="n"/>
+      <c r="V61" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>BCIO:008590</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>s) after (to be removed and added to list of relations)</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>A part of a BCI schedule which is the relation a specified temporal part is in when it starts following the end of another temporal part or timepoint</t>
         </is>
       </c>
-      <c r="D61" s="4" t="n"/>
-      <c r="E61" s="4" t="n"/>
-      <c r="F61" s="4" t="n"/>
-      <c r="G61" s="4" t="n"/>
-      <c r="H61" s="4" t="inlineStr">
+      <c r="D62" s="4" t="n"/>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="inlineStr">
         <is>
           <t>This is not annotated</t>
         </is>
       </c>
-      <c r="I61" s="4" t="n"/>
-      <c r="J61" s="4" t="n"/>
-      <c r="K61" s="4" t="n"/>
-      <c r="L61" s="4" t="n"/>
-      <c r="M61" s="4" t="n"/>
-      <c r="N61" s="4" t="n"/>
-      <c r="O61" s="4" t="n"/>
-      <c r="P61" s="4" t="n"/>
-      <c r="Q61" s="4" t="inlineStr">
+      <c r="I62" s="4" t="n"/>
+      <c r="J62" s="4" t="n"/>
+      <c r="K62" s="4" t="n"/>
+      <c r="L62" s="4" t="n"/>
+      <c r="M62" s="4" t="n"/>
+      <c r="N62" s="4" t="n"/>
+      <c r="O62" s="4" t="n"/>
+      <c r="P62" s="4" t="n"/>
+      <c r="Q62" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R61" s="4" t="n"/>
-      <c r="S61" s="4" t="inlineStr">
+      <c r="R62" s="4" t="n"/>
+      <c r="S62" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T61" s="4" t="n"/>
-      <c r="U61" s="4" t="n"/>
-      <c r="V61" s="4" t="inlineStr">
+      <c r="T62" s="4" t="n"/>
+      <c r="U62" s="4" t="n"/>
+      <c r="V62" s="4" t="inlineStr">
         <is>
           <t>CM; RW</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>BFO:0000038</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>A one-dimensional temporal region is a temporal region that is extended.</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr">
+      <c r="Q63" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V62" t="inlineStr">
+      <c r="V63" t="inlineStr">
         <is>
           <t>JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>BCIO:050312</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">A temporal interval is a one-dimensional temporal region, namely that is self-connected (is without gaps or breaks).
 </t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="n"/>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>one-dimensional temporal region</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
-      <c r="H63" s="4" t="n"/>
-      <c r="I63" s="4" t="n"/>
-      <c r="J63" s="4" t="n"/>
-      <c r="K63" s="4" t="n"/>
-      <c r="L63" s="4" t="n"/>
-      <c r="M63" s="4" t="n"/>
-      <c r="N63" s="4" t="n"/>
-      <c r="O63" s="4" t="n"/>
-      <c r="P63" s="4" t="n"/>
-      <c r="Q63" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R63" s="4" t="n"/>
-      <c r="S63" s="4" t="n"/>
-      <c r="T63" s="4" t="n"/>
-      <c r="U63" s="4" t="n"/>
-      <c r="V63" s="4" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050515</t>
-        </is>
-      </c>
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>temporal part</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>A data item between the start and end of an intervention temporal part.</t>
         </is>
       </c>
       <c r="D64" s="4" t="n"/>
@@ -4023,11 +4019,7 @@
       <c r="F64" s="4" t="n"/>
       <c r="G64" s="4" t="n"/>
       <c r="H64" s="4" t="n"/>
-      <c r="I64" s="4" t="inlineStr">
-        <is>
-          <t>6 weeks; 2 weeks</t>
-        </is>
-      </c>
+      <c r="I64" s="4" t="n"/>
       <c r="J64" s="4" t="n"/>
       <c r="K64" s="4" t="n"/>
       <c r="L64" s="4" t="n"/>
@@ -4046,113 +4038,165 @@
       <c r="U64" s="4" t="n"/>
       <c r="V64" s="4" t="inlineStr">
         <is>
+          <t>JH</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050515</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>temporal part</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>A data item between the start and end of an intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="n"/>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n"/>
+      <c r="G65" s="4" t="n"/>
+      <c r="H65" s="4" t="n"/>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>6 weeks; 2 weeks</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="n"/>
+      <c r="K65" s="4" t="n"/>
+      <c r="L65" s="4" t="n"/>
+      <c r="M65" s="4" t="n"/>
+      <c r="N65" s="4" t="n"/>
+      <c r="O65" s="4" t="n"/>
+      <c r="P65" s="4" t="n"/>
+      <c r="Q65" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R65" s="4" t="n"/>
+      <c r="S65" s="4" t="n"/>
+      <c r="T65" s="4" t="n"/>
+      <c r="U65" s="4" t="n"/>
+      <c r="V65" s="4" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>BCIO:008530</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>temporal reference associated with the intervention</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>A &lt;temporal region&gt; against which a BCI  temporal part is referenced.</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>temporal region</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Temporal references are used by authors when there is a behaviourally relevant event which structures the schedule of a BCI. This can include things like quit dates, childbirth, medical operations etc.
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="n"/>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="n"/>
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
 Example annotation in context: "A feedback call was scheduled to be delivered around 6 months after the birth of the baby".  </t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="K65" s="2" t="n"/>
-      <c r="L65" s="2" t="n"/>
-      <c r="M65" s="2" t="n"/>
-      <c r="N65" s="2" t="n"/>
-      <c r="O65" s="2" t="n"/>
-      <c r="P65" s="2" t="n"/>
-      <c r="Q65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R65" s="2" t="n"/>
-      <c r="S65" s="2" t="inlineStr">
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" s="2" t="n"/>
+      <c r="M66" s="2" t="n"/>
+      <c r="N66" s="2" t="n"/>
+      <c r="O66" s="2" t="n"/>
+      <c r="P66" s="2" t="n"/>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="n"/>
+      <c r="S66" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T65" s="2" t="n"/>
-      <c r="U65" s="2" t="n"/>
-      <c r="V65" s="2" t="inlineStr">
+      <c r="T66" s="2" t="n"/>
+      <c r="U66" s="2" t="n"/>
+      <c r="V66" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>BCIO:008545</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>A &lt;total intervention contact event duration&gt; that is the total of intervention temporal parts within a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>The planned total duration of all sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
 When there is only one session, the total duration of contact events and the duration of a single contact event are technically the same. As a convention, we would annotate this using duration of contact event instead of total duration of contact event. 
@@ -4160,253 +4204,181 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>150 minutes; 12 hours</t>
         </is>
       </c>
-      <c r="J66" s="2" t="n"/>
-      <c r="K66" s="2" t="n"/>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>BCI contact event</t>
         </is>
       </c>
-      <c r="M66" s="2" t="n"/>
-      <c r="N66" s="2" t="n"/>
-      <c r="O66" s="2" t="inlineStr">
+      <c r="M67" s="2" t="n"/>
+      <c r="N67" s="2" t="n"/>
+      <c r="O67" s="2" t="inlineStr">
         <is>
           <t>"is about" contact events or "is about" duration of contact events?</t>
         </is>
       </c>
-      <c r="P66" s="2" t="n"/>
-      <c r="Q66" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R66" s="2" t="inlineStr">
+      <c r="P67" s="2" t="n"/>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S66" s="2" t="inlineStr">
+      <c r="S67" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T66" s="2" t="inlineStr">
+      <c r="T67" s="2" t="inlineStr">
         <is>
           <t>what type of data item is this? (CM)</t>
         </is>
       </c>
-      <c r="U66" s="2" t="n"/>
-      <c r="V66" s="2" t="inlineStr">
+      <c r="U67" s="2" t="n"/>
+      <c r="V67" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>BCIO:051006</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
         </is>
       </c>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="inlineStr">
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F67" s="3" t="n"/>
-      <c r="G67" s="3" t="n"/>
-      <c r="H67" s="3" t="n"/>
-      <c r="I67" s="3" t="n"/>
-      <c r="J67" s="3" t="n"/>
-      <c r="K67" s="3" t="n"/>
-      <c r="L67" s="3" t="n"/>
-      <c r="M67" s="3" t="n"/>
-      <c r="N67" s="3" t="n"/>
-      <c r="O67" s="3" t="n"/>
-      <c r="P67" s="3" t="n"/>
-      <c r="Q67" s="3" t="inlineStr">
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="n"/>
+      <c r="I68" s="3" t="n"/>
+      <c r="J68" s="3" t="n"/>
+      <c r="K68" s="3" t="n"/>
+      <c r="L68" s="3" t="n"/>
+      <c r="M68" s="3" t="n"/>
+      <c r="N68" s="3" t="n"/>
+      <c r="O68" s="3" t="n"/>
+      <c r="P68" s="3" t="n"/>
+      <c r="Q68" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R67" s="3" t="n"/>
-      <c r="S67" s="3" t="n"/>
-      <c r="T67" s="3" t="n"/>
-      <c r="U67" s="3" t="n"/>
-      <c r="V67" s="3" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="R68" s="3" t="n"/>
+      <c r="S68" s="3" t="n"/>
+      <c r="T68" s="3" t="n"/>
+      <c r="U68" s="3" t="n"/>
+      <c r="V68" s="3" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>BCIO:050504</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="n"/>
-      <c r="I68" s="2" t="n"/>
-      <c r="J68" s="2" t="n"/>
-      <c r="K68" s="2" t="n"/>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="M68" s="2" t="n"/>
-      <c r="N68" s="2" t="n"/>
-      <c r="O68" s="2" t="n"/>
-      <c r="P68" s="2" t="n"/>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R68" s="2" t="n"/>
-      <c r="S68" s="2" t="n"/>
-      <c r="T68" s="2" t="n"/>
-      <c r="U68" s="2" t="n"/>
-      <c r="V68" s="2" t="inlineStr">
+      <c r="M69" s="2" t="n"/>
+      <c r="N69" s="2" t="n"/>
+      <c r="O69" s="2" t="n"/>
+      <c r="P69" s="2" t="n"/>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="n"/>
+      <c r="S69" s="2" t="n"/>
+      <c r="T69" s="2" t="n"/>
+      <c r="U69" s="2" t="n"/>
+      <c r="V69" s="2" t="inlineStr">
         <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008605</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="n"/>
-      <c r="E69" s="4" t="n"/>
-      <c r="F69" s="4" t="n"/>
-      <c r="G69" s="4" t="n"/>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
-        </is>
-      </c>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>Participants received "3" emails every 2 weeks</t>
-        </is>
-      </c>
-      <c r="J69" s="4" t="n"/>
-      <c r="K69" s="4" t="n"/>
-      <c r="L69" s="4" t="inlineStr">
-        <is>
-          <t>contact event</t>
-        </is>
-      </c>
-      <c r="M69" s="4" t="n"/>
-      <c r="N69" s="4" t="n"/>
-      <c r="O69" s="4" t="n"/>
-      <c r="P69" s="4" t="n"/>
-      <c r="Q69" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R69" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S69" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T69" s="4" t="inlineStr">
-        <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
-        </is>
-      </c>
-      <c r="U69" s="4" t="n"/>
-      <c r="V69" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008550</t>
+          <t>BCIO:008605</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration (still to confirm inclusion)</t>
+          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
+          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
         </is>
       </c>
       <c r="D70" s="4" t="n"/>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
       <c r="G70" s="4" t="n"/>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in "90" minutes of PA weekly</t>
+          <t>Participants received "3" emails every 2 weeks</t>
         </is>
       </c>
       <c r="J70" s="4" t="n"/>
@@ -4418,11 +4390,7 @@
       </c>
       <c r="M70" s="4" t="n"/>
       <c r="N70" s="4" t="n"/>
-      <c r="O70" s="4" t="inlineStr">
-        <is>
-          <t>is about contact events or is about duration of contact events?</t>
-        </is>
-      </c>
+      <c r="O70" s="4" t="n"/>
       <c r="P70" s="4" t="n"/>
       <c r="Q70" s="4" t="inlineStr">
         <is>
@@ -4441,7 +4409,7 @@
       </c>
       <c r="T70" s="4" t="inlineStr">
         <is>
-          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
         </is>
       </c>
       <c r="U70" s="4" t="n"/>
@@ -4454,17 +4422,17 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008555</t>
+          <t>BCIO:008550</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
+          <t>z) contact event sum duration (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
+          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
         </is>
       </c>
       <c r="D71" s="4" t="n"/>
@@ -4482,7 +4450,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in 90 minutes of PA "weekly"</t>
+          <t>The participants took part in "90" minutes of PA weekly</t>
         </is>
       </c>
       <c r="J71" s="4" t="n"/>
@@ -4530,43 +4498,51 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008600</t>
+          <t>BCIO:008555</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>z) frequency period</t>
+          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
         </is>
       </c>
       <c r="D72" s="4" t="n"/>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
-      <c r="H72" s="4" t="n"/>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>Participants received 3 emails every "2" weeks</t>
+          <t>The participants took part in 90 minutes of PA "weekly"</t>
         </is>
       </c>
       <c r="J72" s="4" t="n"/>
       <c r="K72" s="4" t="n"/>
       <c r="L72" s="4" t="inlineStr">
         <is>
-          <t>intervention temporal part</t>
+          <t>contact event</t>
         </is>
       </c>
       <c r="M72" s="4" t="n"/>
       <c r="N72" s="4" t="n"/>
-      <c r="O72" s="4" t="n"/>
+      <c r="O72" s="4" t="inlineStr">
+        <is>
+          <t>is about contact events or is about duration of contact events?</t>
+        </is>
+      </c>
       <c r="P72" s="4" t="n"/>
       <c r="Q72" s="4" t="inlineStr">
         <is>
@@ -4585,7 +4561,7 @@
       </c>
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
       <c r="U72" s="4" t="n"/>
@@ -4598,48 +4574,64 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008570</t>
+          <t>BCIO:008600</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>z) interval (remove)</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="n"/>
+          <t>z) frequency period</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+        </is>
+      </c>
       <c r="D73" s="4" t="n"/>
-      <c r="E73" s="4" t="n"/>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+        </is>
+      </c>
       <c r="F73" s="4" t="n"/>
       <c r="G73" s="4" t="n"/>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated but included due to relationship with duration of interval</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>Participants received 3 emails every "2" weeks</t>
+        </is>
+      </c>
       <c r="J73" s="4" t="n"/>
       <c r="K73" s="4" t="n"/>
-      <c r="L73" s="4" t="n"/>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
       <c r="M73" s="4" t="n"/>
       <c r="N73" s="4" t="n"/>
-      <c r="O73" s="4" t="inlineStr">
-        <is>
-          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
-        </is>
-      </c>
+      <c r="O73" s="4" t="n"/>
       <c r="P73" s="4" t="n"/>
       <c r="Q73" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R73" s="4" t="n"/>
+      <c r="R73" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="S73" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T73" s="4" t="n"/>
+      <c r="T73" s="4" t="inlineStr">
+        <is>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+        </is>
+      </c>
       <c r="U73" s="4" t="n"/>
       <c r="V73" s="4" t="inlineStr">
         <is>
@@ -4650,72 +4642,124 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008520</t>
+          <t>BCIO:008570</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>z) intervention temporal part frequency</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
-        </is>
-      </c>
+          <t>z) interval (remove)</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="n"/>
       <c r="D74" s="4" t="n"/>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
-        <is>
-          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
-        </is>
-      </c>
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="n"/>
       <c r="G74" s="4" t="n"/>
       <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>This is not annotated but included due to relationship with duration of interval</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="n"/>
+      <c r="J74" s="4" t="n"/>
+      <c r="K74" s="4" t="n"/>
+      <c r="L74" s="4" t="n"/>
+      <c r="M74" s="4" t="n"/>
+      <c r="N74" s="4" t="n"/>
+      <c r="O74" s="4" t="inlineStr">
+        <is>
+          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+        </is>
+      </c>
+      <c r="P74" s="4" t="n"/>
+      <c r="Q74" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R74" s="4" t="n"/>
+      <c r="S74" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T74" s="4" t="n"/>
+      <c r="U74" s="4" t="n"/>
+      <c r="V74" s="4" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008520</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>z) intervention temporal part frequency</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="n"/>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="inlineStr">
         <is>
           <t>This is used to capture descriptions of the frequency of contact events within a part. 
 Example annotation (in context)
 intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks"</t>
         </is>
       </c>
-      <c r="I74" s="4" t="n"/>
-      <c r="J74" s="4" t="n"/>
-      <c r="K74" s="4" t="n"/>
-      <c r="L74" s="4" t="inlineStr">
+      <c r="I75" s="4" t="n"/>
+      <c r="J75" s="4" t="n"/>
+      <c r="K75" s="4" t="n"/>
+      <c r="L75" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M74" s="4" t="n"/>
-      <c r="N74" s="4" t="n"/>
-      <c r="O74" s="4" t="n"/>
-      <c r="P74" s="4" t="n"/>
-      <c r="Q74" s="4" t="inlineStr">
+      <c r="M75" s="4" t="n"/>
+      <c r="N75" s="4" t="n"/>
+      <c r="O75" s="4" t="n"/>
+      <c r="P75" s="4" t="n"/>
+      <c r="Q75" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R74" s="4" t="inlineStr">
+      <c r="R75" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S74" s="4" t="inlineStr">
+      <c r="S75" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T74" s="4" t="inlineStr">
+      <c r="T75" s="4" t="inlineStr">
         <is>
           <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
         </is>
       </c>
-      <c r="U74" s="4" t="n"/>
-      <c r="V74" s="4" t="inlineStr">
+      <c r="U75" s="4" t="n"/>
+      <c r="V75" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>

</xml_diff>

<commit_message>
Update BCI contact event in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -564,13 +564,13 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A &lt;BCI temporal part&gt; that is an occasion in which a member of a BCI population comes into contact with a BCI.  </t>
+          <t xml:space="preserve">An &lt;intervention contact event&gt; that is an occasion in which a member of a BCI population comes into contact with a BCI.  </t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part</t>
+          <t>intervention contact event</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1285,33 +1285,33 @@
           <t>An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>intervention temporal part</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
-      <c r="N14" s="3" t="inlineStr"/>
-      <c r="O14" s="3" t="inlineStr"/>
-      <c r="P14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
+      <c r="N14" s="3" t="n"/>
+      <c r="O14" s="3" t="n"/>
+      <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr"/>
-      <c r="S14" s="3" t="inlineStr"/>
-      <c r="T14" s="3" t="inlineStr"/>
-      <c r="U14" s="3" t="inlineStr"/>
-      <c r="V14" s="3" t="inlineStr"/>
+      <c r="R14" s="3" t="n"/>
+      <c r="S14" s="3" t="n"/>
+      <c r="T14" s="3" t="n"/>
+      <c r="U14" s="3" t="n"/>
+      <c r="V14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add intervention schedule of delivery to BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V76"/>
+  <dimension ref="A1:V77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1714,295 +1714,278 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051011</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>An &lt;intervention attribute&gt; that is its temporal organisation.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr"/>
+      <c r="N23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="inlineStr"/>
+      <c r="S23" s="3" t="inlineStr"/>
+      <c r="T23" s="3" t="inlineStr"/>
+      <c r="U23" s="3" t="inlineStr"/>
+      <c r="V23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>BCIO:051008</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>A &lt;planned process&gt; that is a part of an intervention.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R23" s="2" t="n"/>
-      <c r="S23" s="2" t="n"/>
-      <c r="T23" s="2" t="n"/>
-      <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
+      <c r="O24" s="2" t="n"/>
+      <c r="P24" s="2" t="n"/>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="n"/>
+      <c r="S24" s="2" t="n"/>
+      <c r="T24" s="2" t="n"/>
+      <c r="U24" s="2" t="n"/>
+      <c r="V24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>BCIO:051003</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>intervention temporal part duration</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; between the start and end of an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
-      <c r="O24" s="3" t="n"/>
-      <c r="P24" s="3" t="n"/>
-      <c r="Q24" s="3" t="inlineStr">
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+      <c r="N25" s="3" t="n"/>
+      <c r="O25" s="3" t="n"/>
+      <c r="P25" s="3" t="n"/>
+      <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R24" s="3" t="n"/>
-      <c r="S24" s="3" t="n"/>
-      <c r="T24" s="3" t="n"/>
-      <c r="U24" s="3" t="n"/>
-      <c r="V24" s="3" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="R25" s="3" t="n"/>
+      <c r="S25" s="3" t="n"/>
+      <c r="T25" s="3" t="n"/>
+      <c r="U25" s="3" t="n"/>
+      <c r="V25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>BCIO:050506</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part duration statistic</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of intervention temporal part durations.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>BCI temporal part duration</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="n"/>
-      <c r="Q25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R25" s="2" t="n"/>
-      <c r="S25" s="2" t="n"/>
-      <c r="T25" s="2" t="n"/>
-      <c r="U25" s="2" t="n"/>
-      <c r="V25" s="2" t="inlineStr">
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="n"/>
+      <c r="O26" s="2" t="n"/>
+      <c r="P26" s="2" t="n"/>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="n"/>
+      <c r="S26" s="2" t="n"/>
+      <c r="T26" s="2" t="n"/>
+      <c r="U26" s="2" t="n"/>
+      <c r="V26" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>BCIO:051004</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>intervention temporal part frequency</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is how often intervention temporal parts occur within an intervention.</t>
         </is>
       </c>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">This is useful when grouping contact events together to the schedule of an intervention. For example, authors may describe participants as taking part in 90 minutes of physical activity weekly. These 90 minutes could be split across several contact events, however together these contact events form an intervention part which occurs weekly. </t>
         </is>
       </c>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="inlineStr">
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n"/>
+      <c r="M27" s="3" t="n"/>
+      <c r="N27" s="3" t="n"/>
+      <c r="O27" s="3" t="n"/>
+      <c r="P27" s="3" t="n"/>
+      <c r="Q27" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R26" s="3" t="n"/>
-      <c r="S26" s="3" t="n"/>
-      <c r="T26" s="3" t="n"/>
-      <c r="U26" s="3" t="n"/>
-      <c r="V26" s="3" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050516</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>intervention temporal part frequency statistic</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention temporal part frequencies.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
-      <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>BCI temporal part frequency</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n"/>
-      <c r="N27" s="2" t="n"/>
-      <c r="O27" s="2" t="n"/>
-      <c r="P27" s="2" t="n"/>
-      <c r="Q27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R27" s="2" t="n"/>
-      <c r="S27" s="2" t="n"/>
-      <c r="T27" s="2" t="n"/>
-      <c r="U27" s="2" t="n"/>
-      <c r="V27" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="R27" s="3" t="n"/>
+      <c r="S27" s="3" t="n"/>
+      <c r="T27" s="3" t="n"/>
+      <c r="U27" s="3" t="n"/>
+      <c r="V27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008540</t>
+          <t>BCIO:050516</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>irregular intervention schedule</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or BCI.  </t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
-        </is>
-      </c>
+          <t>A &lt;data item&gt; that is about a collection of intervention temporal part frequencies.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="n"/>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
-Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks" </t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
-        </is>
-      </c>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>BCI temporal part frequency</t>
+        </is>
+      </c>
       <c r="M28" s="2" t="n"/>
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="n"/>
@@ -2013,60 +1996,57 @@
         </is>
       </c>
       <c r="R28" s="2" t="n"/>
-      <c r="S28" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T28" s="2" t="inlineStr">
-        <is>
-          <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
-        </is>
-      </c>
+      <c r="S28" s="2" t="n"/>
+      <c r="T28" s="2" t="n"/>
       <c r="U28" s="2" t="n"/>
       <c r="V28" s="2" t="inlineStr">
         <is>
-          <t>CM; JH; PS</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050507</t>
+          <t>BCIO:008540</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event duration</t>
+          <t>irregular intervention schedule</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="n"/>
+          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or BCI.  </t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
+        </is>
+      </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
+          <t>BCI schedule of delivery</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
+Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks" </t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event duration</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n"/>
@@ -2077,35 +2057,43 @@
         </is>
       </c>
       <c r="R29" s="2" t="n"/>
-      <c r="S29" s="2" t="n"/>
-      <c r="T29" s="2" t="n"/>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
+        </is>
+      </c>
       <c r="U29" s="2" t="n"/>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050906</t>
+          <t>BCIO:050507</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event frequency</t>
+          <t>maximum intervention contact event duration</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2120,7 +2108,7 @@
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M30" s="2" t="n"/>
@@ -2145,23 +2133,23 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050907</t>
+          <t>BCIO:050906</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event number</t>
+          <t>maximum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2176,7 +2164,7 @@
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M31" s="2" t="n"/>
@@ -2201,23 +2189,23 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050908</t>
+          <t>BCIO:050907</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention duration</t>
+          <t>maximum intervention contact event number</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2232,7 +2220,7 @@
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M32" s="2" t="n"/>
@@ -2257,23 +2245,23 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050508</t>
+          <t>BCIO:050908</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part duration</t>
+          <t>maximum intervention duration</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2288,7 +2276,7 @@
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M33" s="2" t="n"/>
@@ -2313,23 +2301,23 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050517</t>
+          <t>BCIO:050508</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part frequency statistic</t>
+          <t>maximum intervention temporal part duration</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2344,7 +2332,7 @@
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M34" s="2" t="n"/>
@@ -2369,23 +2357,23 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050910</t>
+          <t>BCIO:050517</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>maximum total intervention contact event duration</t>
+          <t>maximum intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2400,7 +2388,7 @@
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M35" s="2" t="n"/>
@@ -2425,23 +2413,23 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050509</t>
+          <t>BCIO:050910</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event duration</t>
+          <t>maximum total intervention contact event duration</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2456,7 +2444,7 @@
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M36" s="2" t="n"/>
@@ -2481,23 +2469,23 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050911</t>
+          <t>BCIO:050509</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event frequency</t>
+          <t>mean intervention contact event duration</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2512,7 +2500,7 @@
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M37" s="2" t="n"/>
@@ -2537,23 +2525,23 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050912</t>
+          <t>BCIO:050911</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event number</t>
+          <t>mean intervention contact event frequency</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2568,7 +2556,7 @@
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M38" s="2" t="n"/>
@@ -2593,23 +2581,23 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050909</t>
+          <t>BCIO:050912</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>mean intervention duration</t>
+          <t>mean intervention contact event number</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2624,7 +2612,7 @@
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M39" s="2" t="n"/>
@@ -2649,23 +2637,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050510</t>
+          <t>BCIO:050909</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part duration</t>
+          <t>mean intervention duration</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2680,7 +2668,7 @@
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M40" s="2" t="n"/>
@@ -2705,23 +2693,23 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050518</t>
+          <t>BCIO:050510</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part frequency statistic</t>
+          <t>mean intervention temporal part duration</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2736,7 +2724,7 @@
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M41" s="2" t="n"/>
@@ -2761,23 +2749,23 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050495</t>
+          <t>BCIO:050518</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>mean total intervention contact event duration</t>
+          <t>mean intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2792,7 +2780,7 @@
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M42" s="2" t="n"/>
@@ -2817,23 +2805,23 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050511</t>
+          <t>BCIO:050495</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event duration</t>
+          <t>mean total intervention contact event duration</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2848,7 +2836,7 @@
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M43" s="2" t="n"/>
@@ -2873,23 +2861,23 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050496</t>
+          <t>BCIO:050511</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event frequency</t>
+          <t>median intervention contact event duration</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2904,7 +2892,7 @@
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M44" s="2" t="n"/>
@@ -2929,23 +2917,23 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050497</t>
+          <t>BCIO:050496</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event number</t>
+          <t>median intervention contact event frequency</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2960,7 +2948,7 @@
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M45" s="2" t="n"/>
@@ -2985,23 +2973,23 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050498</t>
+          <t>BCIO:050497</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>median intervention duration</t>
+          <t>median intervention contact event number</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3016,7 +3004,7 @@
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M46" s="2" t="n"/>
@@ -3041,23 +3029,23 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050512</t>
+          <t>BCIO:050498</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part duration</t>
+          <t>median intervention duration</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3072,7 +3060,7 @@
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M47" s="2" t="n"/>
@@ -3097,23 +3085,23 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050519</t>
+          <t>BCIO:050512</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part frequency statistic</t>
+          <t>median intervention temporal part duration</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3128,7 +3116,7 @@
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M48" s="2" t="n"/>
@@ -3153,23 +3141,23 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050499</t>
+          <t>BCIO:050519</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>median total intervention contact event duration</t>
+          <t>median intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3184,7 +3172,7 @@
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M49" s="2" t="n"/>
@@ -3209,23 +3197,23 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050513</t>
+          <t>BCIO:050499</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event duration</t>
+          <t>median total intervention contact event duration</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3240,7 +3228,7 @@
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M50" s="2" t="n"/>
@@ -3265,23 +3253,23 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050500</t>
+          <t>BCIO:050513</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event frequency</t>
+          <t>minimum intervention contact event duration</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3296,7 +3284,7 @@
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M51" s="2" t="n"/>
@@ -3321,23 +3309,23 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050502</t>
+          <t>BCIO:050500</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event number</t>
+          <t>minimum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3352,7 +3340,7 @@
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M52" s="2" t="n"/>
@@ -3377,23 +3365,23 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050501</t>
+          <t>BCIO:050502</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention duration</t>
+          <t>minimum intervention contact event number</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3408,7 +3396,7 @@
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M53" s="2" t="n"/>
@@ -3433,23 +3421,23 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050514</t>
+          <t>BCIO:050501</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part duration</t>
+          <t>minimum intervention duration</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3464,7 +3452,7 @@
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M54" s="2" t="n"/>
@@ -3489,23 +3477,23 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050520</t>
+          <t>BCIO:050514</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part frequency statistic</t>
+          <t>minimum intervention temporal part duration</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -3520,7 +3508,7 @@
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M55" s="2" t="n"/>
@@ -3545,23 +3533,23 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050503</t>
+          <t>BCIO:050520</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>minimum total intervention contact event duration</t>
+          <t>minimum intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3576,7 +3564,7 @@
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M56" s="2" t="n"/>
@@ -3601,48 +3589,38 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008515</t>
+          <t>BCIO:050503</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>minimum total intervention contact event duration</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
-        </is>
-      </c>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>number of intervention contact events</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="n"/>
+          <t>total intervention contact event duration statistic</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
-Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
-This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
-        </is>
-      </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>one; 6; 12; twenty</t>
-        </is>
-      </c>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
       <c r="J57" s="2" t="n"/>
       <c r="K57" s="2" t="n"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M57" s="2" t="n"/>
@@ -3654,98 +3632,164 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="R57" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S57" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
+      <c r="R57" s="2" t="n"/>
+      <c r="S57" s="2" t="n"/>
       <c r="T57" s="2" t="n"/>
       <c r="U57" s="2" t="n"/>
       <c r="V57" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008515</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>number of BCI contact events</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>number of intervention contact events</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
+Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
+This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>one; 6; 12; twenty</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="n"/>
+      <c r="N58" s="2" t="n"/>
+      <c r="O58" s="2" t="n"/>
+      <c r="P58" s="2" t="n"/>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="n"/>
+      <c r="U58" s="2" t="n"/>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>BCIO:051005</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>number of intervention contact events</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D58" s="3" t="n"/>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="D59" s="3" t="n"/>
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F58" s="3" t="n"/>
-      <c r="G58" s="3" t="n"/>
-      <c r="H58" s="3" t="n"/>
-      <c r="I58" s="3" t="n"/>
-      <c r="J58" s="3" t="n"/>
-      <c r="K58" s="3" t="n"/>
-      <c r="L58" s="3" t="n"/>
-      <c r="M58" s="3" t="n"/>
-      <c r="N58" s="3" t="n"/>
-      <c r="O58" s="3" t="n"/>
-      <c r="P58" s="3" t="n"/>
-      <c r="Q58" s="3" t="inlineStr">
+      <c r="F59" s="3" t="n"/>
+      <c r="G59" s="3" t="n"/>
+      <c r="H59" s="3" t="n"/>
+      <c r="I59" s="3" t="n"/>
+      <c r="J59" s="3" t="n"/>
+      <c r="K59" s="3" t="n"/>
+      <c r="L59" s="3" t="n"/>
+      <c r="M59" s="3" t="n"/>
+      <c r="N59" s="3" t="n"/>
+      <c r="O59" s="3" t="n"/>
+      <c r="P59" s="3" t="n"/>
+      <c r="Q59" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R58" s="3" t="n"/>
-      <c r="S58" s="3" t="n"/>
-      <c r="T58" s="3" t="n"/>
-      <c r="U58" s="3" t="n"/>
-      <c r="V58" s="3" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="R59" s="3" t="n"/>
+      <c r="S59" s="3" t="n"/>
+      <c r="T59" s="3" t="n"/>
+      <c r="U59" s="3" t="n"/>
+      <c r="V59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>BCIO:008580</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">order of BCI temporal parts </t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>A &lt;BCI attribute&gt; that is the  temporal positioning of BCI temporal parts.</t>
         </is>
       </c>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>BCI attribute</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n"/>
-      <c r="G59" s="2" t="n"/>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="n"/>
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>This is annotated as an open code when any aspect of order is described</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>"After questionnaires were completed, feedback was selected
 out of a database with messages for each possible combination
@@ -3754,102 +3798,50 @@
 levels to the PA guidelines."</t>
         </is>
       </c>
-      <c r="J59" s="2" t="n"/>
-      <c r="K59" s="2" t="n"/>
-      <c r="L59" s="2" t="n"/>
-      <c r="M59" s="2" t="inlineStr">
+      <c r="J60" s="2" t="n"/>
+      <c r="K60" s="2" t="n"/>
+      <c r="L60" s="2" t="n"/>
+      <c r="M60" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="N59" s="2" t="n"/>
-      <c r="O59" s="2" t="n"/>
-      <c r="P59" s="2" t="n"/>
-      <c r="Q59" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R59" s="2" t="n"/>
-      <c r="S59" s="2" t="inlineStr">
+      <c r="N60" s="2" t="n"/>
+      <c r="O60" s="2" t="n"/>
+      <c r="P60" s="2" t="n"/>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="n"/>
+      <c r="S60" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T59" s="2" t="n"/>
-      <c r="U59" s="2" t="n"/>
-      <c r="V59" s="2" t="inlineStr">
+      <c r="T60" s="2" t="n"/>
+      <c r="U60" s="2" t="n"/>
+      <c r="V60" s="2" t="inlineStr">
         <is>
           <t>CM; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008595</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>q) same time (remove - this is a relation like before and after)</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="n"/>
-      <c r="E60" s="4" t="n"/>
-      <c r="F60" s="4" t="n"/>
-      <c r="G60" s="4" t="n"/>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated</t>
-        </is>
-      </c>
-      <c r="I60" s="4" t="n"/>
-      <c r="J60" s="4" t="n"/>
-      <c r="K60" s="4" t="n"/>
-      <c r="L60" s="4" t="n"/>
-      <c r="M60" s="4" t="n"/>
-      <c r="N60" s="4" t="n"/>
-      <c r="O60" s="4" t="n"/>
-      <c r="P60" s="4" t="n"/>
-      <c r="Q60" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R60" s="4" t="n"/>
-      <c r="S60" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T60" s="4" t="n"/>
-      <c r="U60" s="4" t="n"/>
-      <c r="V60" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008585</t>
+          <t>BCIO:008595</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>r) before (to be removed and added to list of relations)</t>
+          <t>q) same time (remove - this is a relation like before and after)</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
         </is>
       </c>
       <c r="D61" s="4" t="n"/>
@@ -3858,7 +3850,7 @@
       <c r="G61" s="4" t="n"/>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is not annotated </t>
+          <t>This is not annotated</t>
         </is>
       </c>
       <c r="I61" s="4" t="n"/>
@@ -3884,222 +3876,226 @@
       <c r="U61" s="4" t="n"/>
       <c r="V61" s="4" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008585</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>r) before (to be removed and added to list of relations)</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n"/>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is not annotated </t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="n"/>
+      <c r="J62" s="4" t="n"/>
+      <c r="K62" s="4" t="n"/>
+      <c r="L62" s="4" t="n"/>
+      <c r="M62" s="4" t="n"/>
+      <c r="N62" s="4" t="n"/>
+      <c r="O62" s="4" t="n"/>
+      <c r="P62" s="4" t="n"/>
+      <c r="Q62" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R62" s="4" t="n"/>
+      <c r="S62" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T62" s="4" t="n"/>
+      <c r="U62" s="4" t="n"/>
+      <c r="V62" s="4" t="inlineStr">
+        <is>
           <t>CM; RW</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>BCIO:008535</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>regular intervention schedule</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of a BCI or BCI part.  </t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="F62" s="2" t="n"/>
-      <c r="G62" s="2" t="n"/>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="n"/>
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention" </t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr">
         <is>
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
         </is>
       </c>
-      <c r="J62" s="2" t="n"/>
-      <c r="K62" s="2" t="n"/>
-      <c r="L62" s="2" t="n"/>
-      <c r="M62" s="2" t="n"/>
-      <c r="N62" s="2" t="n"/>
-      <c r="O62" s="2" t="n"/>
-      <c r="P62" s="2" t="n"/>
-      <c r="Q62" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R62" s="2" t="n"/>
-      <c r="S62" s="2" t="inlineStr">
+      <c r="J63" s="2" t="n"/>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
+      <c r="M63" s="2" t="n"/>
+      <c r="N63" s="2" t="n"/>
+      <c r="O63" s="2" t="n"/>
+      <c r="P63" s="2" t="n"/>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="n"/>
+      <c r="S63" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T62" s="2" t="n"/>
-      <c r="U62" s="2" t="n"/>
-      <c r="V62" s="2" t="inlineStr">
+      <c r="T63" s="2" t="n"/>
+      <c r="U63" s="2" t="n"/>
+      <c r="V63" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>BCIO:008590</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>s) after (to be removed and added to list of relations)</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>A part of a BCI schedule which is the relation a specified temporal part is in when it starts following the end of another temporal part or timepoint</t>
         </is>
       </c>
-      <c r="D63" s="4" t="n"/>
-      <c r="E63" s="4" t="n"/>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
-      <c r="H63" s="4" t="inlineStr">
+      <c r="D64" s="4" t="n"/>
+      <c r="E64" s="4" t="n"/>
+      <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>This is not annotated</t>
         </is>
       </c>
-      <c r="I63" s="4" t="n"/>
-      <c r="J63" s="4" t="n"/>
-      <c r="K63" s="4" t="n"/>
-      <c r="L63" s="4" t="n"/>
-      <c r="M63" s="4" t="n"/>
-      <c r="N63" s="4" t="n"/>
-      <c r="O63" s="4" t="n"/>
-      <c r="P63" s="4" t="n"/>
-      <c r="Q63" s="4" t="inlineStr">
+      <c r="I64" s="4" t="n"/>
+      <c r="J64" s="4" t="n"/>
+      <c r="K64" s="4" t="n"/>
+      <c r="L64" s="4" t="n"/>
+      <c r="M64" s="4" t="n"/>
+      <c r="N64" s="4" t="n"/>
+      <c r="O64" s="4" t="n"/>
+      <c r="P64" s="4" t="n"/>
+      <c r="Q64" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R63" s="4" t="n"/>
-      <c r="S63" s="4" t="inlineStr">
+      <c r="R64" s="4" t="n"/>
+      <c r="S64" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T63" s="4" t="n"/>
-      <c r="U63" s="4" t="n"/>
-      <c r="V63" s="4" t="inlineStr">
+      <c r="T64" s="4" t="n"/>
+      <c r="U64" s="4" t="n"/>
+      <c r="V64" s="4" t="inlineStr">
         <is>
           <t>CM; RW</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>BFO:0000038</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>A one-dimensional temporal region is a temporal region that is extended.</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="Q64" t="inlineStr">
+      <c r="Q65" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V64" t="inlineStr">
+      <c r="V65" t="inlineStr">
         <is>
           <t>JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>BCIO:050312</t>
         </is>
       </c>
-      <c r="B65" s="4" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">A temporal interval is a one-dimensional temporal region, namely that is self-connected (is without gaps or breaks).
 </t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="n"/>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>one-dimensional temporal region</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="n"/>
-      <c r="G65" s="4" t="n"/>
-      <c r="H65" s="4" t="n"/>
-      <c r="I65" s="4" t="n"/>
-      <c r="J65" s="4" t="n"/>
-      <c r="K65" s="4" t="n"/>
-      <c r="L65" s="4" t="n"/>
-      <c r="M65" s="4" t="n"/>
-      <c r="N65" s="4" t="n"/>
-      <c r="O65" s="4" t="n"/>
-      <c r="P65" s="4" t="n"/>
-      <c r="Q65" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R65" s="4" t="n"/>
-      <c r="S65" s="4" t="n"/>
-      <c r="T65" s="4" t="n"/>
-      <c r="U65" s="4" t="n"/>
-      <c r="V65" s="4" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050515</t>
-        </is>
-      </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>temporal part</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>A data item between the start and end of an intervention temporal part.</t>
         </is>
       </c>
       <c r="D66" s="4" t="n"/>
@@ -4111,11 +4107,7 @@
       <c r="F66" s="4" t="n"/>
       <c r="G66" s="4" t="n"/>
       <c r="H66" s="4" t="n"/>
-      <c r="I66" s="4" t="inlineStr">
-        <is>
-          <t>6 weeks; 2 weeks</t>
-        </is>
-      </c>
+      <c r="I66" s="4" t="n"/>
       <c r="J66" s="4" t="n"/>
       <c r="K66" s="4" t="n"/>
       <c r="L66" s="4" t="n"/>
@@ -4134,113 +4126,165 @@
       <c r="U66" s="4" t="n"/>
       <c r="V66" s="4" t="inlineStr">
         <is>
+          <t>JH</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050515</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>temporal part</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>A data item between the start and end of an intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="n"/>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n"/>
+      <c r="G67" s="4" t="n"/>
+      <c r="H67" s="4" t="n"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>6 weeks; 2 weeks</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="n"/>
+      <c r="K67" s="4" t="n"/>
+      <c r="L67" s="4" t="n"/>
+      <c r="M67" s="4" t="n"/>
+      <c r="N67" s="4" t="n"/>
+      <c r="O67" s="4" t="n"/>
+      <c r="P67" s="4" t="n"/>
+      <c r="Q67" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R67" s="4" t="n"/>
+      <c r="S67" s="4" t="n"/>
+      <c r="T67" s="4" t="n"/>
+      <c r="U67" s="4" t="n"/>
+      <c r="V67" s="4" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>BCIO:008530</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>temporal reference associated with the intervention</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>A &lt;temporal region&gt; against which a BCI  temporal part is referenced.</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>temporal region</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>Temporal references are used by authors when there is a behaviourally relevant event which structures the schedule of a BCI. This can include things like quit dates, childbirth, medical operations etc.
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="n"/>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
 Example annotation in context: "A feedback call was scheduled to be delivered around 6 months after the birth of the baby".  </t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr">
         <is>
           <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
+      <c r="J68" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="K67" s="2" t="n"/>
-      <c r="L67" s="2" t="n"/>
-      <c r="M67" s="2" t="n"/>
-      <c r="N67" s="2" t="n"/>
-      <c r="O67" s="2" t="n"/>
-      <c r="P67" s="2" t="n"/>
-      <c r="Q67" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R67" s="2" t="n"/>
-      <c r="S67" s="2" t="inlineStr">
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
+      <c r="M68" s="2" t="n"/>
+      <c r="N68" s="2" t="n"/>
+      <c r="O68" s="2" t="n"/>
+      <c r="P68" s="2" t="n"/>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="n"/>
+      <c r="S68" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T67" s="2" t="n"/>
-      <c r="U67" s="2" t="n"/>
-      <c r="V67" s="2" t="inlineStr">
+      <c r="T68" s="2" t="n"/>
+      <c r="U68" s="2" t="n"/>
+      <c r="V68" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>BCIO:008545</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>A &lt;total intervention contact event duration&gt; that is the total of intervention temporal parts within a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>The planned total duration of all sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="F68" s="2" t="n"/>
-      <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
 When there is only one session, the total duration of contact events and the duration of a single contact event are technically the same. As a convention, we would annotate this using duration of contact event instead of total duration of contact event. 
@@ -4248,253 +4292,181 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>150 minutes; 12 hours</t>
         </is>
       </c>
-      <c r="J68" s="2" t="n"/>
-      <c r="K68" s="2" t="n"/>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>BCI contact event</t>
         </is>
       </c>
-      <c r="M68" s="2" t="n"/>
-      <c r="N68" s="2" t="n"/>
-      <c r="O68" s="2" t="inlineStr">
+      <c r="M69" s="2" t="n"/>
+      <c r="N69" s="2" t="n"/>
+      <c r="O69" s="2" t="inlineStr">
         <is>
           <t>"is about" contact events or "is about" duration of contact events?</t>
         </is>
       </c>
-      <c r="P68" s="2" t="n"/>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R68" s="2" t="inlineStr">
+      <c r="P69" s="2" t="n"/>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S68" s="2" t="inlineStr">
+      <c r="S69" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T68" s="2" t="inlineStr">
+      <c r="T69" s="2" t="inlineStr">
         <is>
           <t>what type of data item is this? (CM)</t>
         </is>
       </c>
-      <c r="U68" s="2" t="n"/>
-      <c r="V68" s="2" t="inlineStr">
+      <c r="U69" s="2" t="n"/>
+      <c r="V69" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>BCIO:051006</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
         </is>
       </c>
-      <c r="D69" s="3" t="n"/>
-      <c r="E69" s="3" t="inlineStr">
+      <c r="D70" s="3" t="n"/>
+      <c r="E70" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F69" s="3" t="n"/>
-      <c r="G69" s="3" t="n"/>
-      <c r="H69" s="3" t="n"/>
-      <c r="I69" s="3" t="n"/>
-      <c r="J69" s="3" t="n"/>
-      <c r="K69" s="3" t="n"/>
-      <c r="L69" s="3" t="n"/>
-      <c r="M69" s="3" t="n"/>
-      <c r="N69" s="3" t="n"/>
-      <c r="O69" s="3" t="n"/>
-      <c r="P69" s="3" t="n"/>
-      <c r="Q69" s="3" t="inlineStr">
+      <c r="F70" s="3" t="n"/>
+      <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
+      <c r="I70" s="3" t="n"/>
+      <c r="J70" s="3" t="n"/>
+      <c r="K70" s="3" t="n"/>
+      <c r="L70" s="3" t="n"/>
+      <c r="M70" s="3" t="n"/>
+      <c r="N70" s="3" t="n"/>
+      <c r="O70" s="3" t="n"/>
+      <c r="P70" s="3" t="n"/>
+      <c r="Q70" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R69" s="3" t="n"/>
-      <c r="S69" s="3" t="n"/>
-      <c r="T69" s="3" t="n"/>
-      <c r="U69" s="3" t="n"/>
-      <c r="V69" s="3" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="R70" s="3" t="n"/>
+      <c r="S70" s="3" t="n"/>
+      <c r="T70" s="3" t="n"/>
+      <c r="U70" s="3" t="n"/>
+      <c r="V70" s="3" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>BCIO:050504</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G70" s="2" t="n"/>
-      <c r="H70" s="2" t="n"/>
-      <c r="I70" s="2" t="n"/>
-      <c r="J70" s="2" t="n"/>
-      <c r="K70" s="2" t="n"/>
-      <c r="L70" s="2" t="inlineStr">
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="n"/>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="n"/>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="M70" s="2" t="n"/>
-      <c r="N70" s="2" t="n"/>
-      <c r="O70" s="2" t="n"/>
-      <c r="P70" s="2" t="n"/>
-      <c r="Q70" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R70" s="2" t="n"/>
-      <c r="S70" s="2" t="n"/>
-      <c r="T70" s="2" t="n"/>
-      <c r="U70" s="2" t="n"/>
-      <c r="V70" s="2" t="inlineStr">
+      <c r="M71" s="2" t="n"/>
+      <c r="N71" s="2" t="n"/>
+      <c r="O71" s="2" t="n"/>
+      <c r="P71" s="2" t="n"/>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="n"/>
+      <c r="S71" s="2" t="n"/>
+      <c r="T71" s="2" t="n"/>
+      <c r="U71" s="2" t="n"/>
+      <c r="V71" s="2" t="inlineStr">
         <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008605</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="n"/>
-      <c r="E71" s="4" t="n"/>
-      <c r="F71" s="4" t="n"/>
-      <c r="G71" s="4" t="n"/>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
-        </is>
-      </c>
-      <c r="I71" s="4" t="inlineStr">
-        <is>
-          <t>Participants received "3" emails every 2 weeks</t>
-        </is>
-      </c>
-      <c r="J71" s="4" t="n"/>
-      <c r="K71" s="4" t="n"/>
-      <c r="L71" s="4" t="inlineStr">
-        <is>
-          <t>contact event</t>
-        </is>
-      </c>
-      <c r="M71" s="4" t="n"/>
-      <c r="N71" s="4" t="n"/>
-      <c r="O71" s="4" t="n"/>
-      <c r="P71" s="4" t="n"/>
-      <c r="Q71" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R71" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S71" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T71" s="4" t="inlineStr">
-        <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
-        </is>
-      </c>
-      <c r="U71" s="4" t="n"/>
-      <c r="V71" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008550</t>
+          <t>BCIO:008605</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration (still to confirm inclusion)</t>
+          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
+          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
         </is>
       </c>
       <c r="D72" s="4" t="n"/>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in "90" minutes of PA weekly</t>
+          <t>Participants received "3" emails every 2 weeks</t>
         </is>
       </c>
       <c r="J72" s="4" t="n"/>
@@ -4506,11 +4478,7 @@
       </c>
       <c r="M72" s="4" t="n"/>
       <c r="N72" s="4" t="n"/>
-      <c r="O72" s="4" t="inlineStr">
-        <is>
-          <t>is about contact events or is about duration of contact events?</t>
-        </is>
-      </c>
+      <c r="O72" s="4" t="n"/>
       <c r="P72" s="4" t="n"/>
       <c r="Q72" s="4" t="inlineStr">
         <is>
@@ -4529,7 +4497,7 @@
       </c>
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
         </is>
       </c>
       <c r="U72" s="4" t="n"/>
@@ -4542,17 +4510,17 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008555</t>
+          <t>BCIO:008550</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
+          <t>z) contact event sum duration (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
+          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
         </is>
       </c>
       <c r="D73" s="4" t="n"/>
@@ -4570,7 +4538,7 @@
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in 90 minutes of PA "weekly"</t>
+          <t>The participants took part in "90" minutes of PA weekly</t>
         </is>
       </c>
       <c r="J73" s="4" t="n"/>
@@ -4618,43 +4586,51 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008600</t>
+          <t>BCIO:008555</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>z) frequency period</t>
+          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
         </is>
       </c>
       <c r="D74" s="4" t="n"/>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F74" s="4" t="n"/>
       <c r="G74" s="4" t="n"/>
-      <c r="H74" s="4" t="n"/>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>Participants received 3 emails every "2" weeks</t>
+          <t>The participants took part in 90 minutes of PA "weekly"</t>
         </is>
       </c>
       <c r="J74" s="4" t="n"/>
       <c r="K74" s="4" t="n"/>
       <c r="L74" s="4" t="inlineStr">
         <is>
-          <t>intervention temporal part</t>
+          <t>contact event</t>
         </is>
       </c>
       <c r="M74" s="4" t="n"/>
       <c r="N74" s="4" t="n"/>
-      <c r="O74" s="4" t="n"/>
+      <c r="O74" s="4" t="inlineStr">
+        <is>
+          <t>is about contact events or is about duration of contact events?</t>
+        </is>
+      </c>
       <c r="P74" s="4" t="n"/>
       <c r="Q74" s="4" t="inlineStr">
         <is>
@@ -4673,7 +4649,7 @@
       </c>
       <c r="T74" s="4" t="inlineStr">
         <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
       <c r="U74" s="4" t="n"/>
@@ -4686,48 +4662,64 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008570</t>
+          <t>BCIO:008600</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>z) interval (remove)</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="n"/>
+          <t>z) frequency period</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+        </is>
+      </c>
       <c r="D75" s="4" t="n"/>
-      <c r="E75" s="4" t="n"/>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+        </is>
+      </c>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated but included due to relationship with duration of interval</t>
-        </is>
-      </c>
-      <c r="I75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>Participants received 3 emails every "2" weeks</t>
+        </is>
+      </c>
       <c r="J75" s="4" t="n"/>
       <c r="K75" s="4" t="n"/>
-      <c r="L75" s="4" t="n"/>
+      <c r="L75" s="4" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
       <c r="M75" s="4" t="n"/>
       <c r="N75" s="4" t="n"/>
-      <c r="O75" s="4" t="inlineStr">
-        <is>
-          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
-        </is>
-      </c>
+      <c r="O75" s="4" t="n"/>
       <c r="P75" s="4" t="n"/>
       <c r="Q75" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R75" s="4" t="n"/>
+      <c r="R75" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="S75" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T75" s="4" t="n"/>
+      <c r="T75" s="4" t="inlineStr">
+        <is>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+        </is>
+      </c>
       <c r="U75" s="4" t="n"/>
       <c r="V75" s="4" t="inlineStr">
         <is>
@@ -4738,72 +4730,124 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008520</t>
+          <t>BCIO:008570</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>z) intervention temporal part frequency</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
-        </is>
-      </c>
+          <t>z) interval (remove)</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="n"/>
       <c r="D76" s="4" t="n"/>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
-        </is>
-      </c>
+      <c r="E76" s="4" t="n"/>
+      <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
       <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>This is not annotated but included due to relationship with duration of interval</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="n"/>
+      <c r="J76" s="4" t="n"/>
+      <c r="K76" s="4" t="n"/>
+      <c r="L76" s="4" t="n"/>
+      <c r="M76" s="4" t="n"/>
+      <c r="N76" s="4" t="n"/>
+      <c r="O76" s="4" t="inlineStr">
+        <is>
+          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+        </is>
+      </c>
+      <c r="P76" s="4" t="n"/>
+      <c r="Q76" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R76" s="4" t="n"/>
+      <c r="S76" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T76" s="4" t="n"/>
+      <c r="U76" s="4" t="n"/>
+      <c r="V76" s="4" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008520</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>z) intervention temporal part frequency</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="n"/>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="n"/>
+      <c r="H77" s="4" t="inlineStr">
         <is>
           <t>This is used to capture descriptions of the frequency of contact events within a part. 
 Example annotation (in context)
 intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks"</t>
         </is>
       </c>
-      <c r="I76" s="4" t="n"/>
-      <c r="J76" s="4" t="n"/>
-      <c r="K76" s="4" t="n"/>
-      <c r="L76" s="4" t="inlineStr">
+      <c r="I77" s="4" t="n"/>
+      <c r="J77" s="4" t="n"/>
+      <c r="K77" s="4" t="n"/>
+      <c r="L77" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M76" s="4" t="n"/>
-      <c r="N76" s="4" t="n"/>
-      <c r="O76" s="4" t="n"/>
-      <c r="P76" s="4" t="n"/>
-      <c r="Q76" s="4" t="inlineStr">
+      <c r="M77" s="4" t="n"/>
+      <c r="N77" s="4" t="n"/>
+      <c r="O77" s="4" t="n"/>
+      <c r="P77" s="4" t="n"/>
+      <c r="Q77" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R76" s="4" t="inlineStr">
+      <c r="R77" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S76" s="4" t="inlineStr">
+      <c r="S77" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T76" s="4" t="inlineStr">
+      <c r="T77" s="4" t="inlineStr">
         <is>
           <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
         </is>
       </c>
-      <c r="U76" s="4" t="n"/>
-      <c r="V76" s="4" t="inlineStr">
+      <c r="U77" s="4" t="n"/>
+      <c r="V77" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>

</xml_diff>

<commit_message>
Update irregular intervention schedule in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -1729,33 +1729,33 @@
           <t>An &lt;intervention attribute&gt; that is its temporal organisation.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
-      <c r="N23" s="3" t="inlineStr"/>
-      <c r="O23" s="3" t="inlineStr"/>
-      <c r="P23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="n"/>
+      <c r="O23" s="3" t="n"/>
+      <c r="P23" s="3" t="n"/>
       <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R23" s="3" t="inlineStr"/>
-      <c r="S23" s="3" t="inlineStr"/>
-      <c r="T23" s="3" t="inlineStr"/>
-      <c r="U23" s="3" t="inlineStr"/>
-      <c r="V23" s="3" t="inlineStr"/>
+      <c r="R23" s="3" t="n"/>
+      <c r="S23" s="3" t="n"/>
+      <c r="T23" s="3" t="n"/>
+      <c r="U23" s="3" t="n"/>
+      <c r="V23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or BCI.  </t>
+          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or intervention.  </t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
+          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="F29" s="2" t="n"/>

</xml_diff>

<commit_message>
Update regular intervention schedule in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -3945,7 +3945,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A &lt;BCI schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of a BCI or BCI part.  </t>
+          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
+          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="F63" s="2" t="n"/>

</xml_diff>

<commit_message>
Add order of intervention temporal parts to BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V77"/>
+  <dimension ref="A1:V78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3829,71 +3829,63 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008595</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>q) same time (remove - this is a relation like before and after)</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="n"/>
-      <c r="E61" s="4" t="n"/>
-      <c r="F61" s="4" t="n"/>
-      <c r="G61" s="4" t="n"/>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated</t>
-        </is>
-      </c>
-      <c r="I61" s="4" t="n"/>
-      <c r="J61" s="4" t="n"/>
-      <c r="K61" s="4" t="n"/>
-      <c r="L61" s="4" t="n"/>
-      <c r="M61" s="4" t="n"/>
-      <c r="N61" s="4" t="n"/>
-      <c r="O61" s="4" t="n"/>
-      <c r="P61" s="4" t="n"/>
-      <c r="Q61" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R61" s="4" t="n"/>
-      <c r="S61" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T61" s="4" t="n"/>
-      <c r="U61" s="4" t="n"/>
-      <c r="V61" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
-        </is>
-      </c>
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051012</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>order of intervention temporal parts</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>An &lt;intervention attribute&gt; that is the  temporal positioning of intervention temporal parts.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr"/>
+      <c r="G61" s="3" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr"/>
+      <c r="J61" s="3" t="inlineStr"/>
+      <c r="K61" s="3" t="inlineStr"/>
+      <c r="L61" s="3" t="inlineStr"/>
+      <c r="M61" s="3" t="inlineStr"/>
+      <c r="N61" s="3" t="inlineStr"/>
+      <c r="O61" s="3" t="inlineStr"/>
+      <c r="P61" s="3" t="inlineStr"/>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr"/>
+      <c r="S61" s="3" t="inlineStr"/>
+      <c r="T61" s="3" t="inlineStr"/>
+      <c r="U61" s="3" t="inlineStr"/>
+      <c r="V61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008585</t>
+          <t>BCIO:008595</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>r) before (to be removed and added to list of relations)</t>
+          <t>q) same time (remove - this is a relation like before and after)</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
         </is>
       </c>
       <c r="D62" s="4" t="n"/>
@@ -3902,7 +3894,7 @@
       <c r="G62" s="4" t="n"/>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is not annotated </t>
+          <t>This is not annotated</t>
         </is>
       </c>
       <c r="I62" s="4" t="n"/>
@@ -3928,222 +3920,226 @@
       <c r="U62" s="4" t="n"/>
       <c r="V62" s="4" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008585</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>r) before (to be removed and added to list of relations)</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="n"/>
+      <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is not annotated </t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="n"/>
+      <c r="J63" s="4" t="n"/>
+      <c r="K63" s="4" t="n"/>
+      <c r="L63" s="4" t="n"/>
+      <c r="M63" s="4" t="n"/>
+      <c r="N63" s="4" t="n"/>
+      <c r="O63" s="4" t="n"/>
+      <c r="P63" s="4" t="n"/>
+      <c r="Q63" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R63" s="4" t="n"/>
+      <c r="S63" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T63" s="4" t="n"/>
+      <c r="U63" s="4" t="n"/>
+      <c r="V63" s="4" t="inlineStr">
+        <is>
           <t>CM; RW</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>BCIO:008535</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>regular intervention schedule</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="F63" s="2" t="n"/>
-      <c r="G63" s="2" t="n"/>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention" </t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
         </is>
       </c>
-      <c r="J63" s="2" t="n"/>
-      <c r="K63" s="2" t="n"/>
-      <c r="L63" s="2" t="n"/>
-      <c r="M63" s="2" t="n"/>
-      <c r="N63" s="2" t="n"/>
-      <c r="O63" s="2" t="n"/>
-      <c r="P63" s="2" t="n"/>
-      <c r="Q63" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R63" s="2" t="n"/>
-      <c r="S63" s="2" t="inlineStr">
+      <c r="J64" s="2" t="n"/>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
+      <c r="M64" s="2" t="n"/>
+      <c r="N64" s="2" t="n"/>
+      <c r="O64" s="2" t="n"/>
+      <c r="P64" s="2" t="n"/>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="n"/>
+      <c r="S64" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T63" s="2" t="n"/>
-      <c r="U63" s="2" t="n"/>
-      <c r="V63" s="2" t="inlineStr">
+      <c r="T64" s="2" t="n"/>
+      <c r="U64" s="2" t="n"/>
+      <c r="V64" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>BCIO:008590</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>s) after (to be removed and added to list of relations)</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>A part of a BCI schedule which is the relation a specified temporal part is in when it starts following the end of another temporal part or timepoint</t>
         </is>
       </c>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="4" t="n"/>
-      <c r="H64" s="4" t="inlineStr">
+      <c r="D65" s="4" t="n"/>
+      <c r="E65" s="4" t="n"/>
+      <c r="F65" s="4" t="n"/>
+      <c r="G65" s="4" t="n"/>
+      <c r="H65" s="4" t="inlineStr">
         <is>
           <t>This is not annotated</t>
         </is>
       </c>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="n"/>
-      <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="n"/>
-      <c r="M64" s="4" t="n"/>
-      <c r="N64" s="4" t="n"/>
-      <c r="O64" s="4" t="n"/>
-      <c r="P64" s="4" t="n"/>
-      <c r="Q64" s="4" t="inlineStr">
+      <c r="I65" s="4" t="n"/>
+      <c r="J65" s="4" t="n"/>
+      <c r="K65" s="4" t="n"/>
+      <c r="L65" s="4" t="n"/>
+      <c r="M65" s="4" t="n"/>
+      <c r="N65" s="4" t="n"/>
+      <c r="O65" s="4" t="n"/>
+      <c r="P65" s="4" t="n"/>
+      <c r="Q65" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R64" s="4" t="n"/>
-      <c r="S64" s="4" t="inlineStr">
+      <c r="R65" s="4" t="n"/>
+      <c r="S65" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T64" s="4" t="n"/>
-      <c r="U64" s="4" t="n"/>
-      <c r="V64" s="4" t="inlineStr">
+      <c r="T65" s="4" t="n"/>
+      <c r="U65" s="4" t="n"/>
+      <c r="V65" s="4" t="inlineStr">
         <is>
           <t>CM; RW</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>BFO:0000038</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>A one-dimensional temporal region is a temporal region that is extended.</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="Q65" t="inlineStr">
+      <c r="Q66" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V65" t="inlineStr">
+      <c r="V66" t="inlineStr">
         <is>
           <t>JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>BCIO:050312</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">A temporal interval is a one-dimensional temporal region, namely that is self-connected (is without gaps or breaks).
 </t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="n"/>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>one-dimensional temporal region</t>
-        </is>
-      </c>
-      <c r="F66" s="4" t="n"/>
-      <c r="G66" s="4" t="n"/>
-      <c r="H66" s="4" t="n"/>
-      <c r="I66" s="4" t="n"/>
-      <c r="J66" s="4" t="n"/>
-      <c r="K66" s="4" t="n"/>
-      <c r="L66" s="4" t="n"/>
-      <c r="M66" s="4" t="n"/>
-      <c r="N66" s="4" t="n"/>
-      <c r="O66" s="4" t="n"/>
-      <c r="P66" s="4" t="n"/>
-      <c r="Q66" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R66" s="4" t="n"/>
-      <c r="S66" s="4" t="n"/>
-      <c r="T66" s="4" t="n"/>
-      <c r="U66" s="4" t="n"/>
-      <c r="V66" s="4" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050515</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>temporal part</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>A data item between the start and end of an intervention temporal part.</t>
         </is>
       </c>
       <c r="D67" s="4" t="n"/>
@@ -4155,11 +4151,7 @@
       <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="n"/>
       <c r="H67" s="4" t="n"/>
-      <c r="I67" s="4" t="inlineStr">
-        <is>
-          <t>6 weeks; 2 weeks</t>
-        </is>
-      </c>
+      <c r="I67" s="4" t="n"/>
       <c r="J67" s="4" t="n"/>
       <c r="K67" s="4" t="n"/>
       <c r="L67" s="4" t="n"/>
@@ -4178,113 +4170,165 @@
       <c r="U67" s="4" t="n"/>
       <c r="V67" s="4" t="inlineStr">
         <is>
+          <t>JH</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050515</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>temporal part</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>A data item between the start and end of an intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="n"/>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n"/>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>6 weeks; 2 weeks</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="n"/>
+      <c r="K68" s="4" t="n"/>
+      <c r="L68" s="4" t="n"/>
+      <c r="M68" s="4" t="n"/>
+      <c r="N68" s="4" t="n"/>
+      <c r="O68" s="4" t="n"/>
+      <c r="P68" s="4" t="n"/>
+      <c r="Q68" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R68" s="4" t="n"/>
+      <c r="S68" s="4" t="n"/>
+      <c r="T68" s="4" t="n"/>
+      <c r="U68" s="4" t="n"/>
+      <c r="V68" s="4" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>BCIO:008530</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>temporal reference associated with the intervention</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>A &lt;temporal region&gt; against which a BCI  temporal part is referenced.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>temporal region</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>Temporal references are used by authors when there is a behaviourally relevant event which structures the schedule of a BCI. This can include things like quit dates, childbirth, medical operations etc.
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
 Example annotation in context: "A feedback call was scheduled to be delivered around 6 months after the birth of the baby".  </t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
+      <c r="J69" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="K68" s="2" t="n"/>
-      <c r="L68" s="2" t="n"/>
-      <c r="M68" s="2" t="n"/>
-      <c r="N68" s="2" t="n"/>
-      <c r="O68" s="2" t="n"/>
-      <c r="P68" s="2" t="n"/>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R68" s="2" t="n"/>
-      <c r="S68" s="2" t="inlineStr">
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
+      <c r="M69" s="2" t="n"/>
+      <c r="N69" s="2" t="n"/>
+      <c r="O69" s="2" t="n"/>
+      <c r="P69" s="2" t="n"/>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="n"/>
+      <c r="S69" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T68" s="2" t="n"/>
-      <c r="U68" s="2" t="n"/>
-      <c r="V68" s="2" t="inlineStr">
+      <c r="T69" s="2" t="n"/>
+      <c r="U69" s="2" t="n"/>
+      <c r="V69" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>BCIO:008545</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>A &lt;total intervention contact event duration&gt; that is the total of intervention temporal parts within a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>The planned total duration of all sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="F69" s="2" t="n"/>
-      <c r="G69" s="2" t="n"/>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
 When there is only one session, the total duration of contact events and the duration of a single contact event are technically the same. As a convention, we would annotate this using duration of contact event instead of total duration of contact event. 
@@ -4292,253 +4336,181 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>150 minutes; 12 hours</t>
         </is>
       </c>
-      <c r="J69" s="2" t="n"/>
-      <c r="K69" s="2" t="n"/>
-      <c r="L69" s="2" t="inlineStr">
+      <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>BCI contact event</t>
         </is>
       </c>
-      <c r="M69" s="2" t="n"/>
-      <c r="N69" s="2" t="n"/>
-      <c r="O69" s="2" t="inlineStr">
+      <c r="M70" s="2" t="n"/>
+      <c r="N70" s="2" t="n"/>
+      <c r="O70" s="2" t="inlineStr">
         <is>
           <t>"is about" contact events or "is about" duration of contact events?</t>
         </is>
       </c>
-      <c r="P69" s="2" t="n"/>
-      <c r="Q69" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R69" s="2" t="inlineStr">
+      <c r="P70" s="2" t="n"/>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S69" s="2" t="inlineStr">
+      <c r="S70" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T69" s="2" t="inlineStr">
+      <c r="T70" s="2" t="inlineStr">
         <is>
           <t>what type of data item is this? (CM)</t>
         </is>
       </c>
-      <c r="U69" s="2" t="n"/>
-      <c r="V69" s="2" t="inlineStr">
+      <c r="U70" s="2" t="n"/>
+      <c r="V70" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>BCIO:051006</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
         </is>
       </c>
-      <c r="D70" s="3" t="n"/>
-      <c r="E70" s="3" t="inlineStr">
+      <c r="D71" s="3" t="n"/>
+      <c r="E71" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F70" s="3" t="n"/>
-      <c r="G70" s="3" t="n"/>
-      <c r="H70" s="3" t="n"/>
-      <c r="I70" s="3" t="n"/>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="3" t="n"/>
-      <c r="L70" s="3" t="n"/>
-      <c r="M70" s="3" t="n"/>
-      <c r="N70" s="3" t="n"/>
-      <c r="O70" s="3" t="n"/>
-      <c r="P70" s="3" t="n"/>
-      <c r="Q70" s="3" t="inlineStr">
+      <c r="F71" s="3" t="n"/>
+      <c r="G71" s="3" t="n"/>
+      <c r="H71" s="3" t="n"/>
+      <c r="I71" s="3" t="n"/>
+      <c r="J71" s="3" t="n"/>
+      <c r="K71" s="3" t="n"/>
+      <c r="L71" s="3" t="n"/>
+      <c r="M71" s="3" t="n"/>
+      <c r="N71" s="3" t="n"/>
+      <c r="O71" s="3" t="n"/>
+      <c r="P71" s="3" t="n"/>
+      <c r="Q71" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R70" s="3" t="n"/>
-      <c r="S70" s="3" t="n"/>
-      <c r="T70" s="3" t="n"/>
-      <c r="U70" s="3" t="n"/>
-      <c r="V70" s="3" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="R71" s="3" t="n"/>
+      <c r="S71" s="3" t="n"/>
+      <c r="T71" s="3" t="n"/>
+      <c r="U71" s="3" t="n"/>
+      <c r="V71" s="3" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>BCIO:050504</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D71" s="2" t="n"/>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G71" s="2" t="n"/>
-      <c r="H71" s="2" t="n"/>
-      <c r="I71" s="2" t="n"/>
-      <c r="J71" s="2" t="n"/>
-      <c r="K71" s="2" t="n"/>
-      <c r="L71" s="2" t="inlineStr">
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="n"/>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="n"/>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="M71" s="2" t="n"/>
-      <c r="N71" s="2" t="n"/>
-      <c r="O71" s="2" t="n"/>
-      <c r="P71" s="2" t="n"/>
-      <c r="Q71" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R71" s="2" t="n"/>
-      <c r="S71" s="2" t="n"/>
-      <c r="T71" s="2" t="n"/>
-      <c r="U71" s="2" t="n"/>
-      <c r="V71" s="2" t="inlineStr">
+      <c r="M72" s="2" t="n"/>
+      <c r="N72" s="2" t="n"/>
+      <c r="O72" s="2" t="n"/>
+      <c r="P72" s="2" t="n"/>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="n"/>
+      <c r="S72" s="2" t="n"/>
+      <c r="T72" s="2" t="n"/>
+      <c r="U72" s="2" t="n"/>
+      <c r="V72" s="2" t="inlineStr">
         <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008605</t>
-        </is>
-      </c>
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="n"/>
-      <c r="E72" s="4" t="n"/>
-      <c r="F72" s="4" t="n"/>
-      <c r="G72" s="4" t="n"/>
-      <c r="H72" s="4" t="inlineStr">
-        <is>
-          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
-        </is>
-      </c>
-      <c r="I72" s="4" t="inlineStr">
-        <is>
-          <t>Participants received "3" emails every 2 weeks</t>
-        </is>
-      </c>
-      <c r="J72" s="4" t="n"/>
-      <c r="K72" s="4" t="n"/>
-      <c r="L72" s="4" t="inlineStr">
-        <is>
-          <t>contact event</t>
-        </is>
-      </c>
-      <c r="M72" s="4" t="n"/>
-      <c r="N72" s="4" t="n"/>
-      <c r="O72" s="4" t="n"/>
-      <c r="P72" s="4" t="n"/>
-      <c r="Q72" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R72" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S72" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T72" s="4" t="inlineStr">
-        <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
-        </is>
-      </c>
-      <c r="U72" s="4" t="n"/>
-      <c r="V72" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008550</t>
+          <t>BCIO:008605</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration (still to confirm inclusion)</t>
+          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
+          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
         </is>
       </c>
       <c r="D73" s="4" t="n"/>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="n"/>
       <c r="G73" s="4" t="n"/>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in "90" minutes of PA weekly</t>
+          <t>Participants received "3" emails every 2 weeks</t>
         </is>
       </c>
       <c r="J73" s="4" t="n"/>
@@ -4550,11 +4522,7 @@
       </c>
       <c r="M73" s="4" t="n"/>
       <c r="N73" s="4" t="n"/>
-      <c r="O73" s="4" t="inlineStr">
-        <is>
-          <t>is about contact events or is about duration of contact events?</t>
-        </is>
-      </c>
+      <c r="O73" s="4" t="n"/>
       <c r="P73" s="4" t="n"/>
       <c r="Q73" s="4" t="inlineStr">
         <is>
@@ -4573,7 +4541,7 @@
       </c>
       <c r="T73" s="4" t="inlineStr">
         <is>
-          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
         </is>
       </c>
       <c r="U73" s="4" t="n"/>
@@ -4586,17 +4554,17 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008555</t>
+          <t>BCIO:008550</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
+          <t>z) contact event sum duration (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
+          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
         </is>
       </c>
       <c r="D74" s="4" t="n"/>
@@ -4614,7 +4582,7 @@
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in 90 minutes of PA "weekly"</t>
+          <t>The participants took part in "90" minutes of PA weekly</t>
         </is>
       </c>
       <c r="J74" s="4" t="n"/>
@@ -4662,43 +4630,51 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008600</t>
+          <t>BCIO:008555</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>z) frequency period</t>
+          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
         </is>
       </c>
       <c r="D75" s="4" t="n"/>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
-      <c r="H75" s="4" t="n"/>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>Participants received 3 emails every "2" weeks</t>
+          <t>The participants took part in 90 minutes of PA "weekly"</t>
         </is>
       </c>
       <c r="J75" s="4" t="n"/>
       <c r="K75" s="4" t="n"/>
       <c r="L75" s="4" t="inlineStr">
         <is>
-          <t>intervention temporal part</t>
+          <t>contact event</t>
         </is>
       </c>
       <c r="M75" s="4" t="n"/>
       <c r="N75" s="4" t="n"/>
-      <c r="O75" s="4" t="n"/>
+      <c r="O75" s="4" t="inlineStr">
+        <is>
+          <t>is about contact events or is about duration of contact events?</t>
+        </is>
+      </c>
       <c r="P75" s="4" t="n"/>
       <c r="Q75" s="4" t="inlineStr">
         <is>
@@ -4717,7 +4693,7 @@
       </c>
       <c r="T75" s="4" t="inlineStr">
         <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
       <c r="U75" s="4" t="n"/>
@@ -4730,48 +4706,64 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008570</t>
+          <t>BCIO:008600</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>z) interval (remove)</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="n"/>
+          <t>z) frequency period</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+        </is>
+      </c>
       <c r="D76" s="4" t="n"/>
-      <c r="E76" s="4" t="n"/>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+        </is>
+      </c>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
-      <c r="H76" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated but included due to relationship with duration of interval</t>
-        </is>
-      </c>
-      <c r="I76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>Participants received 3 emails every "2" weeks</t>
+        </is>
+      </c>
       <c r="J76" s="4" t="n"/>
       <c r="K76" s="4" t="n"/>
-      <c r="L76" s="4" t="n"/>
+      <c r="L76" s="4" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
       <c r="M76" s="4" t="n"/>
       <c r="N76" s="4" t="n"/>
-      <c r="O76" s="4" t="inlineStr">
-        <is>
-          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
-        </is>
-      </c>
+      <c r="O76" s="4" t="n"/>
       <c r="P76" s="4" t="n"/>
       <c r="Q76" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R76" s="4" t="n"/>
+      <c r="R76" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="S76" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T76" s="4" t="n"/>
+      <c r="T76" s="4" t="inlineStr">
+        <is>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+        </is>
+      </c>
       <c r="U76" s="4" t="n"/>
       <c r="V76" s="4" t="inlineStr">
         <is>
@@ -4782,72 +4774,124 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008520</t>
+          <t>BCIO:008570</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>z) intervention temporal part frequency</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
-        </is>
-      </c>
+          <t>z) interval (remove)</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="n"/>
       <c r="D77" s="4" t="n"/>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
-        </is>
-      </c>
+      <c r="E77" s="4" t="n"/>
+      <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="n"/>
       <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>This is not annotated but included due to relationship with duration of interval</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="n"/>
+      <c r="J77" s="4" t="n"/>
+      <c r="K77" s="4" t="n"/>
+      <c r="L77" s="4" t="n"/>
+      <c r="M77" s="4" t="n"/>
+      <c r="N77" s="4" t="n"/>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+        </is>
+      </c>
+      <c r="P77" s="4" t="n"/>
+      <c r="Q77" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R77" s="4" t="n"/>
+      <c r="S77" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T77" s="4" t="n"/>
+      <c r="U77" s="4" t="n"/>
+      <c r="V77" s="4" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008520</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>z) intervention temporal part frequency</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="n"/>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="inlineStr">
         <is>
           <t>This is used to capture descriptions of the frequency of contact events within a part. 
 Example annotation (in context)
 intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks"</t>
         </is>
       </c>
-      <c r="I77" s="4" t="n"/>
-      <c r="J77" s="4" t="n"/>
-      <c r="K77" s="4" t="n"/>
-      <c r="L77" s="4" t="inlineStr">
+      <c r="I78" s="4" t="n"/>
+      <c r="J78" s="4" t="n"/>
+      <c r="K78" s="4" t="n"/>
+      <c r="L78" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M77" s="4" t="n"/>
-      <c r="N77" s="4" t="n"/>
-      <c r="O77" s="4" t="n"/>
-      <c r="P77" s="4" t="n"/>
-      <c r="Q77" s="4" t="inlineStr">
+      <c r="M78" s="4" t="n"/>
+      <c r="N78" s="4" t="n"/>
+      <c r="O78" s="4" t="n"/>
+      <c r="P78" s="4" t="n"/>
+      <c r="Q78" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R77" s="4" t="inlineStr">
+      <c r="R78" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S77" s="4" t="inlineStr">
+      <c r="S78" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T77" s="4" t="inlineStr">
+      <c r="T78" s="4" t="inlineStr">
         <is>
           <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
         </is>
       </c>
-      <c r="U77" s="4" t="n"/>
-      <c r="V77" s="4" t="inlineStr">
+      <c r="U78" s="4" t="n"/>
+      <c r="V78" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>

</xml_diff>

<commit_message>
Update order of BCI temporal parts  in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -3773,13 +3773,13 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>A &lt;BCI attribute&gt; that is the  temporal positioning of BCI temporal parts.</t>
+          <t>An &lt;order of intervention temporal parts&gt; that is the  temporal positioning of BCI temporal parts.</t>
         </is>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
+          <t>order of intervention temporal parts</t>
         </is>
       </c>
       <c r="F60" s="2" t="n"/>
@@ -3844,33 +3844,33 @@
           <t>An &lt;intervention attribute&gt; that is the  temporal positioning of intervention temporal parts.</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="n"/>
       <c r="E61" s="3" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="F61" s="3" t="inlineStr"/>
-      <c r="G61" s="3" t="inlineStr"/>
-      <c r="H61" s="3" t="inlineStr"/>
-      <c r="I61" s="3" t="inlineStr"/>
-      <c r="J61" s="3" t="inlineStr"/>
-      <c r="K61" s="3" t="inlineStr"/>
-      <c r="L61" s="3" t="inlineStr"/>
-      <c r="M61" s="3" t="inlineStr"/>
-      <c r="N61" s="3" t="inlineStr"/>
-      <c r="O61" s="3" t="inlineStr"/>
-      <c r="P61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
+      <c r="I61" s="3" t="n"/>
+      <c r="J61" s="3" t="n"/>
+      <c r="K61" s="3" t="n"/>
+      <c r="L61" s="3" t="n"/>
+      <c r="M61" s="3" t="n"/>
+      <c r="N61" s="3" t="n"/>
+      <c r="O61" s="3" t="n"/>
+      <c r="P61" s="3" t="n"/>
       <c r="Q61" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R61" s="3" t="inlineStr"/>
-      <c r="S61" s="3" t="inlineStr"/>
-      <c r="T61" s="3" t="inlineStr"/>
-      <c r="U61" s="3" t="inlineStr"/>
-      <c r="V61" s="3" t="inlineStr"/>
+      <c r="R61" s="3" t="n"/>
+      <c r="S61" s="3" t="n"/>
+      <c r="T61" s="3" t="n"/>
+      <c r="U61" s="3" t="n"/>
+      <c r="V61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Edit BCIO_Schedule.xlsx: update 2, add 2
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V78"/>
+  <dimension ref="A1:V80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2013,22 +2013,22 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
+          <t>irregular BCI schedule</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An &lt;irregular intervention schedule&gt; in which the frequency and duration of contact events change over the course of a temporal part or intervention.  </t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
           <t>irregular intervention schedule</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or intervention.  </t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="F29" s="2" t="n"/>
@@ -2075,81 +2075,82 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050507</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>maximum intervention contact event duration</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event duration statistic</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event duration</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n"/>
-      <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="n"/>
-      <c r="P30" s="2" t="n"/>
-      <c r="Q30" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R30" s="2" t="n"/>
-      <c r="S30" s="2" t="n"/>
-      <c r="T30" s="2" t="n"/>
-      <c r="U30" s="2" t="n"/>
-      <c r="V30" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051013</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>irregular intervention schedule</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or intervention.  </t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
+Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks"  </t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="3" t="inlineStr"/>
+      <c r="N30" s="3" t="inlineStr"/>
+      <c r="O30" s="3" t="inlineStr"/>
+      <c r="P30" s="3" t="inlineStr"/>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr"/>
+      <c r="S30" s="3" t="inlineStr"/>
+      <c r="T30" s="3" t="inlineStr"/>
+      <c r="U30" s="3" t="inlineStr"/>
+      <c r="V30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050906</t>
+          <t>BCIO:050507</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event frequency</t>
+          <t>maximum intervention contact event duration</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2164,7 +2165,7 @@
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M31" s="2" t="n"/>
@@ -2189,23 +2190,23 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050907</t>
+          <t>BCIO:050906</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention contact event number</t>
+          <t>maximum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2220,7 +2221,7 @@
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M32" s="2" t="n"/>
@@ -2245,23 +2246,23 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050908</t>
+          <t>BCIO:050907</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention duration</t>
+          <t>maximum intervention contact event number</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2276,7 +2277,7 @@
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M33" s="2" t="n"/>
@@ -2301,23 +2302,23 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050508</t>
+          <t>BCIO:050908</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part duration</t>
+          <t>maximum intervention duration</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2332,7 +2333,7 @@
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M34" s="2" t="n"/>
@@ -2357,23 +2358,23 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050517</t>
+          <t>BCIO:050508</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>maximum intervention temporal part frequency statistic</t>
+          <t>maximum intervention temporal part duration</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2388,7 +2389,7 @@
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M35" s="2" t="n"/>
@@ -2413,23 +2414,23 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050910</t>
+          <t>BCIO:050517</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>maximum total intervention contact event duration</t>
+          <t>maximum intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2444,7 +2445,7 @@
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M36" s="2" t="n"/>
@@ -2469,23 +2470,23 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050509</t>
+          <t>BCIO:050910</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event duration</t>
+          <t>maximum total intervention contact event duration</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2500,7 +2501,7 @@
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M37" s="2" t="n"/>
@@ -2525,23 +2526,23 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050911</t>
+          <t>BCIO:050509</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event frequency</t>
+          <t>mean intervention contact event duration</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2556,7 +2557,7 @@
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M38" s="2" t="n"/>
@@ -2581,23 +2582,23 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050912</t>
+          <t>BCIO:050911</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>mean intervention contact event number</t>
+          <t>mean intervention contact event frequency</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2612,7 +2613,7 @@
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M39" s="2" t="n"/>
@@ -2637,23 +2638,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050909</t>
+          <t>BCIO:050912</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>mean intervention duration</t>
+          <t>mean intervention contact event number</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2668,7 +2669,7 @@
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M40" s="2" t="n"/>
@@ -2693,23 +2694,23 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050510</t>
+          <t>BCIO:050909</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part duration</t>
+          <t>mean intervention duration</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2724,7 +2725,7 @@
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M41" s="2" t="n"/>
@@ -2749,23 +2750,23 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050518</t>
+          <t>BCIO:050510</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>mean intervention temporal part frequency statistic</t>
+          <t>mean intervention temporal part duration</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2780,7 +2781,7 @@
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M42" s="2" t="n"/>
@@ -2805,23 +2806,23 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050495</t>
+          <t>BCIO:050518</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>mean total intervention contact event duration</t>
+          <t>mean intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2836,7 +2837,7 @@
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M43" s="2" t="n"/>
@@ -2861,23 +2862,23 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050511</t>
+          <t>BCIO:050495</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event duration</t>
+          <t>mean total intervention contact event duration</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
         </is>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2892,7 +2893,7 @@
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M44" s="2" t="n"/>
@@ -2917,23 +2918,23 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050496</t>
+          <t>BCIO:050511</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event frequency</t>
+          <t>median intervention contact event duration</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2948,7 +2949,7 @@
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M45" s="2" t="n"/>
@@ -2973,23 +2974,23 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050497</t>
+          <t>BCIO:050496</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>median intervention contact event number</t>
+          <t>median intervention contact event frequency</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3004,7 +3005,7 @@
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M46" s="2" t="n"/>
@@ -3029,23 +3030,23 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050498</t>
+          <t>BCIO:050497</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>median intervention duration</t>
+          <t>median intervention contact event number</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3060,7 +3061,7 @@
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M47" s="2" t="n"/>
@@ -3085,23 +3086,23 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050512</t>
+          <t>BCIO:050498</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part duration</t>
+          <t>median intervention duration</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3116,7 +3117,7 @@
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M48" s="2" t="n"/>
@@ -3141,23 +3142,23 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050519</t>
+          <t>BCIO:050512</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>median intervention temporal part frequency statistic</t>
+          <t>median intervention temporal part duration</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3172,7 +3173,7 @@
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M49" s="2" t="n"/>
@@ -3197,23 +3198,23 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050499</t>
+          <t>BCIO:050519</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>median total intervention contact event duration</t>
+          <t>median intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3228,7 +3229,7 @@
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M50" s="2" t="n"/>
@@ -3253,23 +3254,23 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050513</t>
+          <t>BCIO:050499</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event duration</t>
+          <t>median total intervention contact event duration</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>total intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3284,7 +3285,7 @@
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M51" s="2" t="n"/>
@@ -3309,23 +3310,23 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050500</t>
+          <t>BCIO:050513</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event frequency</t>
+          <t>minimum intervention contact event duration</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
+          <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event duration statistic</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3340,7 +3341,7 @@
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>BCI contact event duration</t>
         </is>
       </c>
       <c r="M52" s="2" t="n"/>
@@ -3365,23 +3366,23 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050502</t>
+          <t>BCIO:050500</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention contact event number</t>
+          <t>minimum intervention contact event frequency</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
+          <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention contact event frequency statistic</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3396,7 +3397,7 @@
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>BCI contact event frequency</t>
         </is>
       </c>
       <c r="M53" s="2" t="n"/>
@@ -3421,23 +3422,23 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050501</t>
+          <t>BCIO:050502</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention duration</t>
+          <t>minimum intervention contact event number</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
+          <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3452,7 +3453,7 @@
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>BCI duration</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M54" s="2" t="n"/>
@@ -3477,23 +3478,23 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050514</t>
+          <t>BCIO:050501</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part duration</t>
+          <t>minimum intervention duration</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
+          <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
         </is>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration statistic</t>
+          <t>intervention duration statistic</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -3508,7 +3509,7 @@
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI duration</t>
         </is>
       </c>
       <c r="M55" s="2" t="n"/>
@@ -3533,23 +3534,23 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050520</t>
+          <t>BCIO:050514</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>minimum intervention temporal part frequency statistic</t>
+          <t>minimum intervention temporal part duration</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
+          <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part frequency statistic</t>
+          <t>intervention temporal part duration statistic</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3564,7 +3565,7 @@
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="M56" s="2" t="n"/>
@@ -3589,23 +3590,23 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050503</t>
+          <t>BCIO:050520</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>minimum total intervention contact event duration</t>
+          <t>minimum intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+          <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>total intervention contact event duration statistic</t>
+          <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3620,7 +3621,7 @@
       <c r="K57" s="2" t="n"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="M57" s="2" t="n"/>
@@ -3645,48 +3646,38 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008515</t>
+          <t>BCIO:050503</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>minimum total intervention contact event duration</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
-        </is>
-      </c>
+          <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>number of intervention contact events</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="n"/>
+          <t>total intervention contact event duration statistic</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G58" s="2" t="n"/>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
-Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
-This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>one; 6; 12; twenty</t>
-        </is>
-      </c>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="n"/>
       <c r="J58" s="2" t="n"/>
       <c r="K58" s="2" t="n"/>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event</t>
+          <t>total BCI contact event duration</t>
         </is>
       </c>
       <c r="M58" s="2" t="n"/>
@@ -3698,98 +3689,164 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="R58" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S58" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
+      <c r="R58" s="2" t="n"/>
+      <c r="S58" s="2" t="n"/>
       <c r="T58" s="2" t="n"/>
       <c r="U58" s="2" t="n"/>
       <c r="V58" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008515</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>number of BCI contact events</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>number of intervention contact events</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
+Example annotations (in context): participants attended "a" gp visit ; at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes 
+This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>one; 6; 12; twenty</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="n"/>
+      <c r="N59" s="2" t="n"/>
+      <c r="O59" s="2" t="n"/>
+      <c r="P59" s="2" t="n"/>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="n"/>
+      <c r="U59" s="2" t="n"/>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>BCIO:051005</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>number of intervention contact events</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D59" s="3" t="n"/>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="D60" s="3" t="n"/>
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F59" s="3" t="n"/>
-      <c r="G59" s="3" t="n"/>
-      <c r="H59" s="3" t="n"/>
-      <c r="I59" s="3" t="n"/>
-      <c r="J59" s="3" t="n"/>
-      <c r="K59" s="3" t="n"/>
-      <c r="L59" s="3" t="n"/>
-      <c r="M59" s="3" t="n"/>
-      <c r="N59" s="3" t="n"/>
-      <c r="O59" s="3" t="n"/>
-      <c r="P59" s="3" t="n"/>
-      <c r="Q59" s="3" t="inlineStr">
+      <c r="F60" s="3" t="n"/>
+      <c r="G60" s="3" t="n"/>
+      <c r="H60" s="3" t="n"/>
+      <c r="I60" s="3" t="n"/>
+      <c r="J60" s="3" t="n"/>
+      <c r="K60" s="3" t="n"/>
+      <c r="L60" s="3" t="n"/>
+      <c r="M60" s="3" t="n"/>
+      <c r="N60" s="3" t="n"/>
+      <c r="O60" s="3" t="n"/>
+      <c r="P60" s="3" t="n"/>
+      <c r="Q60" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R59" s="3" t="n"/>
-      <c r="S59" s="3" t="n"/>
-      <c r="T59" s="3" t="n"/>
-      <c r="U59" s="3" t="n"/>
-      <c r="V59" s="3" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="R60" s="3" t="n"/>
+      <c r="S60" s="3" t="n"/>
+      <c r="T60" s="3" t="n"/>
+      <c r="U60" s="3" t="n"/>
+      <c r="V60" s="3" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>BCIO:008580</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">order of BCI temporal parts </t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>An &lt;order of intervention temporal parts&gt; that is the  temporal positioning of BCI temporal parts.</t>
         </is>
       </c>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>order of intervention temporal parts</t>
         </is>
       </c>
-      <c r="F60" s="2" t="n"/>
-      <c r="G60" s="2" t="n"/>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>This is annotated as an open code when any aspect of order is described</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>"After questionnaires were completed, feedback was selected
 out of a database with messages for each possible combination
@@ -3798,146 +3855,94 @@
 levels to the PA guidelines."</t>
         </is>
       </c>
-      <c r="J60" s="2" t="n"/>
-      <c r="K60" s="2" t="n"/>
-      <c r="L60" s="2" t="n"/>
-      <c r="M60" s="2" t="inlineStr">
+      <c r="J61" s="2" t="n"/>
+      <c r="K61" s="2" t="n"/>
+      <c r="L61" s="2" t="n"/>
+      <c r="M61" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="N60" s="2" t="n"/>
-      <c r="O60" s="2" t="n"/>
-      <c r="P60" s="2" t="n"/>
-      <c r="Q60" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R60" s="2" t="n"/>
-      <c r="S60" s="2" t="inlineStr">
+      <c r="N61" s="2" t="n"/>
+      <c r="O61" s="2" t="n"/>
+      <c r="P61" s="2" t="n"/>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="n"/>
+      <c r="S61" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T60" s="2" t="n"/>
-      <c r="U60" s="2" t="n"/>
-      <c r="V60" s="2" t="inlineStr">
+      <c r="T61" s="2" t="n"/>
+      <c r="U61" s="2" t="n"/>
+      <c r="V61" s="2" t="inlineStr">
         <is>
           <t>CM; PS</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>BCIO:051012</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>order of intervention temporal parts</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>An &lt;intervention attribute&gt; that is the  temporal positioning of intervention temporal parts.</t>
         </is>
       </c>
-      <c r="D61" s="3" t="n"/>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="D62" s="3" t="n"/>
+      <c r="E62" s="3" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="F61" s="3" t="n"/>
-      <c r="G61" s="3" t="n"/>
-      <c r="H61" s="3" t="n"/>
-      <c r="I61" s="3" t="n"/>
-      <c r="J61" s="3" t="n"/>
-      <c r="K61" s="3" t="n"/>
-      <c r="L61" s="3" t="n"/>
-      <c r="M61" s="3" t="n"/>
-      <c r="N61" s="3" t="n"/>
-      <c r="O61" s="3" t="n"/>
-      <c r="P61" s="3" t="n"/>
-      <c r="Q61" s="3" t="inlineStr">
+      <c r="F62" s="3" t="n"/>
+      <c r="G62" s="3" t="n"/>
+      <c r="H62" s="3" t="n"/>
+      <c r="I62" s="3" t="n"/>
+      <c r="J62" s="3" t="n"/>
+      <c r="K62" s="3" t="n"/>
+      <c r="L62" s="3" t="n"/>
+      <c r="M62" s="3" t="n"/>
+      <c r="N62" s="3" t="n"/>
+      <c r="O62" s="3" t="n"/>
+      <c r="P62" s="3" t="n"/>
+      <c r="Q62" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R61" s="3" t="n"/>
-      <c r="S61" s="3" t="n"/>
-      <c r="T61" s="3" t="n"/>
-      <c r="U61" s="3" t="n"/>
-      <c r="V61" s="3" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008595</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>q) same time (remove - this is a relation like before and after)</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="n"/>
-      <c r="E62" s="4" t="n"/>
-      <c r="F62" s="4" t="n"/>
-      <c r="G62" s="4" t="n"/>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated</t>
-        </is>
-      </c>
-      <c r="I62" s="4" t="n"/>
-      <c r="J62" s="4" t="n"/>
-      <c r="K62" s="4" t="n"/>
-      <c r="L62" s="4" t="n"/>
-      <c r="M62" s="4" t="n"/>
-      <c r="N62" s="4" t="n"/>
-      <c r="O62" s="4" t="n"/>
-      <c r="P62" s="4" t="n"/>
-      <c r="Q62" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R62" s="4" t="n"/>
-      <c r="S62" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T62" s="4" t="n"/>
-      <c r="U62" s="4" t="n"/>
-      <c r="V62" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
-        </is>
-      </c>
+      <c r="R62" s="3" t="n"/>
+      <c r="S62" s="3" t="n"/>
+      <c r="T62" s="3" t="n"/>
+      <c r="U62" s="3" t="n"/>
+      <c r="V62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008585</t>
+          <t>BCIO:008595</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>r) before (to be removed and added to list of relations)</t>
+          <t>q) same time (remove - this is a relation like before and after)</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it occurs whilst another temporal part or timepoint occurs</t>
         </is>
       </c>
       <c r="D63" s="4" t="n"/>
@@ -3946,7 +3951,7 @@
       <c r="G63" s="4" t="n"/>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is not annotated </t>
+          <t>This is not annotated</t>
         </is>
       </c>
       <c r="I63" s="4" t="n"/>
@@ -3972,185 +3977,209 @@
       <c r="U63" s="4" t="n"/>
       <c r="V63" s="4" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008585</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>r) before (to be removed and added to list of relations)</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it ends prior to the beginning of another temporal part or timepoint</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="n"/>
+      <c r="E64" s="4" t="n"/>
+      <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is not annotated </t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="n"/>
+      <c r="J64" s="4" t="n"/>
+      <c r="K64" s="4" t="n"/>
+      <c r="L64" s="4" t="n"/>
+      <c r="M64" s="4" t="n"/>
+      <c r="N64" s="4" t="n"/>
+      <c r="O64" s="4" t="n"/>
+      <c r="P64" s="4" t="n"/>
+      <c r="Q64" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R64" s="4" t="n"/>
+      <c r="S64" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T64" s="4" t="n"/>
+      <c r="U64" s="4" t="n"/>
+      <c r="V64" s="4" t="inlineStr">
+        <is>
           <t>CM; RW</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>BCIO:008535</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>regular BCI schedule</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A &lt;regular intervention schedule&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>regular intervention schedule</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>intervention schedule of delivery</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="n"/>
-      <c r="G64" s="2" t="n"/>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention" </t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr">
         <is>
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
         </is>
       </c>
-      <c r="J64" s="2" t="n"/>
-      <c r="K64" s="2" t="n"/>
-      <c r="L64" s="2" t="n"/>
-      <c r="M64" s="2" t="n"/>
-      <c r="N64" s="2" t="n"/>
-      <c r="O64" s="2" t="n"/>
-      <c r="P64" s="2" t="n"/>
-      <c r="Q64" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R64" s="2" t="n"/>
-      <c r="S64" s="2" t="inlineStr">
+      <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
+      <c r="M65" s="2" t="n"/>
+      <c r="N65" s="2" t="n"/>
+      <c r="O65" s="2" t="n"/>
+      <c r="P65" s="2" t="n"/>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R65" s="2" t="n"/>
+      <c r="S65" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T64" s="2" t="n"/>
-      <c r="U64" s="2" t="n"/>
-      <c r="V64" s="2" t="inlineStr">
+      <c r="T65" s="2" t="n"/>
+      <c r="U65" s="2" t="n"/>
+      <c r="V65" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008590</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>s) after (to be removed and added to list of relations)</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it starts following the end of another temporal part or timepoint</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="n"/>
-      <c r="E65" s="4" t="n"/>
-      <c r="F65" s="4" t="n"/>
-      <c r="G65" s="4" t="n"/>
-      <c r="H65" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated</t>
-        </is>
-      </c>
-      <c r="I65" s="4" t="n"/>
-      <c r="J65" s="4" t="n"/>
-      <c r="K65" s="4" t="n"/>
-      <c r="L65" s="4" t="n"/>
-      <c r="M65" s="4" t="n"/>
-      <c r="N65" s="4" t="n"/>
-      <c r="O65" s="4" t="n"/>
-      <c r="P65" s="4" t="n"/>
-      <c r="Q65" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R65" s="4" t="n"/>
-      <c r="S65" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T65" s="4" t="n"/>
-      <c r="U65" s="4" t="n"/>
-      <c r="V65" s="4" t="inlineStr">
-        <is>
-          <t>CM; RW</t>
-        </is>
-      </c>
-    </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>BFO:0000038</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>A one-dimensional temporal region is a temporal region that is extended.</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>occurrent</t>
-        </is>
-      </c>
-      <c r="Q66" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="V66" t="inlineStr">
-        <is>
-          <t>JH; PS</t>
-        </is>
-      </c>
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051014</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>regular intervention schedule</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr"/>
+      <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
+Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention"</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr"/>
+      <c r="N66" s="3" t="inlineStr"/>
+      <c r="O66" s="3" t="inlineStr"/>
+      <c r="P66" s="3" t="inlineStr"/>
+      <c r="Q66" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="R66" s="3" t="inlineStr"/>
+      <c r="S66" s="3" t="inlineStr"/>
+      <c r="T66" s="3" t="inlineStr"/>
+      <c r="U66" s="3" t="inlineStr"/>
+      <c r="V66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050312</t>
+          <t>BCIO:008590</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>temporal interval</t>
+          <t>s) after (to be removed and added to list of relations)</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">A temporal interval is a one-dimensional temporal region, namely that is self-connected (is without gaps or breaks).
-</t>
+          <t>A part of a BCI schedule which is the relation a specified temporal part is in when it starts following the end of another temporal part or timepoint</t>
         </is>
       </c>
       <c r="D67" s="4" t="n"/>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>one-dimensional temporal region</t>
-        </is>
-      </c>
+      <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="n"/>
-      <c r="H67" s="4" t="n"/>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>This is not annotated</t>
+        </is>
+      </c>
       <c r="I67" s="4" t="n"/>
       <c r="J67" s="4" t="n"/>
       <c r="K67" s="4" t="n"/>
@@ -4165,170 +4194,255 @@
         </is>
       </c>
       <c r="R67" s="4" t="n"/>
-      <c r="S67" s="4" t="n"/>
+      <c r="S67" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="T67" s="4" t="n"/>
       <c r="U67" s="4" t="n"/>
       <c r="V67" s="4" t="inlineStr">
         <is>
+          <t>CM; RW</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BFO:0000038</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>A one-dimensional temporal region is a temporal region that is extended.</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>JH; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050312</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A temporal interval is a one-dimensional temporal region, namely that is self-connected (is without gaps or breaks).
+</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="n"/>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n"/>
+      <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="n"/>
+      <c r="I69" s="4" t="n"/>
+      <c r="J69" s="4" t="n"/>
+      <c r="K69" s="4" t="n"/>
+      <c r="L69" s="4" t="n"/>
+      <c r="M69" s="4" t="n"/>
+      <c r="N69" s="4" t="n"/>
+      <c r="O69" s="4" t="n"/>
+      <c r="P69" s="4" t="n"/>
+      <c r="Q69" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R69" s="4" t="n"/>
+      <c r="S69" s="4" t="n"/>
+      <c r="T69" s="4" t="n"/>
+      <c r="U69" s="4" t="n"/>
+      <c r="V69" s="4" t="inlineStr">
+        <is>
           <t>JH</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>BCIO:050515</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>temporal part</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>A data item between the start and end of an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D68" s="4" t="n"/>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="D70" s="4" t="n"/>
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="F68" s="4" t="n"/>
-      <c r="G68" s="4" t="n"/>
-      <c r="H68" s="4" t="n"/>
-      <c r="I68" s="4" t="inlineStr">
+      <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n"/>
+      <c r="I70" s="4" t="inlineStr">
         <is>
           <t>6 weeks; 2 weeks</t>
         </is>
       </c>
-      <c r="J68" s="4" t="n"/>
-      <c r="K68" s="4" t="n"/>
-      <c r="L68" s="4" t="n"/>
-      <c r="M68" s="4" t="n"/>
-      <c r="N68" s="4" t="n"/>
-      <c r="O68" s="4" t="n"/>
-      <c r="P68" s="4" t="n"/>
-      <c r="Q68" s="4" t="inlineStr">
+      <c r="J70" s="4" t="n"/>
+      <c r="K70" s="4" t="n"/>
+      <c r="L70" s="4" t="n"/>
+      <c r="M70" s="4" t="n"/>
+      <c r="N70" s="4" t="n"/>
+      <c r="O70" s="4" t="n"/>
+      <c r="P70" s="4" t="n"/>
+      <c r="Q70" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R68" s="4" t="n"/>
-      <c r="S68" s="4" t="n"/>
-      <c r="T68" s="4" t="n"/>
-      <c r="U68" s="4" t="n"/>
-      <c r="V68" s="4" t="inlineStr">
+      <c r="R70" s="4" t="n"/>
+      <c r="S70" s="4" t="n"/>
+      <c r="T70" s="4" t="n"/>
+      <c r="U70" s="4" t="n"/>
+      <c r="V70" s="4" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>BCIO:008530</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>temporal reference associated with the intervention</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>A &lt;temporal region&gt; against which a BCI  temporal part is referenced.</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>temporal region</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>Temporal references are used by authors when there is a behaviourally relevant event which structures the schedule of a BCI. This can include things like quit dates, childbirth, medical operations etc.
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="n"/>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
 Example annotation in context: "A feedback call was scheduled to be delivered around 6 months after the birth of the baby".  </t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="I71" s="2" t="inlineStr">
         <is>
           <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
+      <c r="J71" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="K69" s="2" t="n"/>
-      <c r="L69" s="2" t="n"/>
-      <c r="M69" s="2" t="n"/>
-      <c r="N69" s="2" t="n"/>
-      <c r="O69" s="2" t="n"/>
-      <c r="P69" s="2" t="n"/>
-      <c r="Q69" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R69" s="2" t="n"/>
-      <c r="S69" s="2" t="inlineStr">
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
+      <c r="M71" s="2" t="n"/>
+      <c r="N71" s="2" t="n"/>
+      <c r="O71" s="2" t="n"/>
+      <c r="P71" s="2" t="n"/>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="n"/>
+      <c r="S71" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T69" s="2" t="n"/>
-      <c r="U69" s="2" t="n"/>
-      <c r="V69" s="2" t="inlineStr">
+      <c r="T71" s="2" t="n"/>
+      <c r="U71" s="2" t="n"/>
+      <c r="V71" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>BCIO:008545</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>A &lt;total intervention contact event duration&gt; that is the total of intervention temporal parts within a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>The planned total duration of all sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="F70" s="2" t="n"/>
-      <c r="G70" s="2" t="n"/>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
 When there is only one session, the total duration of contact events and the duration of a single contact event are technically the same. As a convention, we would annotate this using duration of contact event instead of total duration of contact event. 
@@ -4336,329 +4450,181 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>150 minutes; 12 hours</t>
         </is>
       </c>
-      <c r="J70" s="2" t="n"/>
-      <c r="K70" s="2" t="n"/>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event</t>
-        </is>
-      </c>
-      <c r="M70" s="2" t="n"/>
-      <c r="N70" s="2" t="n"/>
-      <c r="O70" s="2" t="inlineStr">
-        <is>
-          <t>"is about" contact events or "is about" duration of contact events?</t>
-        </is>
-      </c>
-      <c r="P70" s="2" t="n"/>
-      <c r="Q70" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R70" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S70" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T70" s="2" t="inlineStr">
-        <is>
-          <t>what type of data item is this? (CM)</t>
-        </is>
-      </c>
-      <c r="U70" s="2" t="n"/>
-      <c r="V70" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051006</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>total intervention contact event duration</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="n"/>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="n"/>
-      <c r="G71" s="3" t="n"/>
-      <c r="H71" s="3" t="n"/>
-      <c r="I71" s="3" t="n"/>
-      <c r="J71" s="3" t="n"/>
-      <c r="K71" s="3" t="n"/>
-      <c r="L71" s="3" t="n"/>
-      <c r="M71" s="3" t="n"/>
-      <c r="N71" s="3" t="n"/>
-      <c r="O71" s="3" t="n"/>
-      <c r="P71" s="3" t="n"/>
-      <c r="Q71" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="R71" s="3" t="n"/>
-      <c r="S71" s="3" t="n"/>
-      <c r="T71" s="3" t="n"/>
-      <c r="U71" s="3" t="n"/>
-      <c r="V71" s="3" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050504</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>total intervention contact event duration statistic</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="n"/>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="n"/>
-      <c r="H72" s="2" t="n"/>
-      <c r="I72" s="2" t="n"/>
       <c r="J72" s="2" t="n"/>
       <c r="K72" s="2" t="n"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>BCI contact event</t>
         </is>
       </c>
       <c r="M72" s="2" t="n"/>
       <c r="N72" s="2" t="n"/>
-      <c r="O72" s="2" t="n"/>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>"is about" contact events or "is about" duration of contact events?</t>
+        </is>
+      </c>
       <c r="P72" s="2" t="n"/>
       <c r="Q72" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="R72" s="2" t="n"/>
-      <c r="S72" s="2" t="n"/>
-      <c r="T72" s="2" t="n"/>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S72" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T72" s="2" t="inlineStr">
+        <is>
+          <t>what type of data item is this? (CM)</t>
+        </is>
+      </c>
       <c r="U72" s="2" t="n"/>
       <c r="V72" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051006</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>total intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n"/>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n"/>
+      <c r="G73" s="3" t="n"/>
+      <c r="H73" s="3" t="n"/>
+      <c r="I73" s="3" t="n"/>
+      <c r="J73" s="3" t="n"/>
+      <c r="K73" s="3" t="n"/>
+      <c r="L73" s="3" t="n"/>
+      <c r="M73" s="3" t="n"/>
+      <c r="N73" s="3" t="n"/>
+      <c r="O73" s="3" t="n"/>
+      <c r="P73" s="3" t="n"/>
+      <c r="Q73" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="R73" s="3" t="n"/>
+      <c r="S73" s="3" t="n"/>
+      <c r="T73" s="3" t="n"/>
+      <c r="U73" s="3" t="n"/>
+      <c r="V73" s="3" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050504</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>total intervention contact event duration statistic</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n"/>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="n"/>
+      <c r="H74" s="2" t="n"/>
+      <c r="I74" s="2" t="n"/>
+      <c r="J74" s="2" t="n"/>
+      <c r="K74" s="2" t="n"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>total BCI contact event duration</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="n"/>
+      <c r="N74" s="2" t="n"/>
+      <c r="O74" s="2" t="n"/>
+      <c r="P74" s="2" t="n"/>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="n"/>
+      <c r="S74" s="2" t="n"/>
+      <c r="T74" s="2" t="n"/>
+      <c r="U74" s="2" t="n"/>
+      <c r="V74" s="2" t="inlineStr">
+        <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008605</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="n"/>
-      <c r="E73" s="4" t="n"/>
-      <c r="F73" s="4" t="n"/>
-      <c r="G73" s="4" t="n"/>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>Participants received "3" emails every 2 weeks</t>
-        </is>
-      </c>
-      <c r="J73" s="4" t="n"/>
-      <c r="K73" s="4" t="n"/>
-      <c r="L73" s="4" t="inlineStr">
-        <is>
-          <t>contact event</t>
-        </is>
-      </c>
-      <c r="M73" s="4" t="n"/>
-      <c r="N73" s="4" t="n"/>
-      <c r="O73" s="4" t="n"/>
-      <c r="P73" s="4" t="n"/>
-      <c r="Q73" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R73" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S73" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T73" s="4" t="inlineStr">
-        <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
-        </is>
-      </c>
-      <c r="U73" s="4" t="n"/>
-      <c r="V73" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008550</t>
-        </is>
-      </c>
-      <c r="B74" s="4" t="inlineStr">
-        <is>
-          <t>z) contact event sum duration (still to confirm inclusion)</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="n"/>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="n"/>
-      <c r="G74" s="4" t="n"/>
-      <c r="H74" s="4" t="inlineStr">
-        <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
-        </is>
-      </c>
-      <c r="I74" s="4" t="inlineStr">
-        <is>
-          <t>The participants took part in "90" minutes of PA weekly</t>
-        </is>
-      </c>
-      <c r="J74" s="4" t="n"/>
-      <c r="K74" s="4" t="n"/>
-      <c r="L74" s="4" t="inlineStr">
-        <is>
-          <t>contact event</t>
-        </is>
-      </c>
-      <c r="M74" s="4" t="n"/>
-      <c r="N74" s="4" t="n"/>
-      <c r="O74" s="4" t="inlineStr">
-        <is>
-          <t>is about contact events or is about duration of contact events?</t>
-        </is>
-      </c>
-      <c r="P74" s="4" t="n"/>
-      <c r="Q74" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R74" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S74" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T74" s="4" t="inlineStr">
-        <is>
-          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
-        </is>
-      </c>
-      <c r="U74" s="4" t="n"/>
-      <c r="V74" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008555</t>
+          <t>BCIO:008605</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
+          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
+          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
         </is>
       </c>
       <c r="D75" s="4" t="n"/>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in 90 minutes of PA "weekly"</t>
+          <t>Participants received "3" emails every 2 weeks</t>
         </is>
       </c>
       <c r="J75" s="4" t="n"/>
@@ -4670,11 +4636,7 @@
       </c>
       <c r="M75" s="4" t="n"/>
       <c r="N75" s="4" t="n"/>
-      <c r="O75" s="4" t="inlineStr">
-        <is>
-          <t>is about contact events or is about duration of contact events?</t>
-        </is>
-      </c>
+      <c r="O75" s="4" t="n"/>
       <c r="P75" s="4" t="n"/>
       <c r="Q75" s="4" t="inlineStr">
         <is>
@@ -4693,7 +4655,7 @@
       </c>
       <c r="T75" s="4" t="inlineStr">
         <is>
-          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
         </is>
       </c>
       <c r="U75" s="4" t="n"/>
@@ -4706,43 +4668,51 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008600</t>
+          <t>BCIO:008550</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>z) frequency period</t>
+          <t>z) contact event sum duration (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
         </is>
       </c>
       <c r="D76" s="4" t="n"/>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
-      <c r="H76" s="4" t="n"/>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>Participants received 3 emails every "2" weeks</t>
+          <t>The participants took part in "90" minutes of PA weekly</t>
         </is>
       </c>
       <c r="J76" s="4" t="n"/>
       <c r="K76" s="4" t="n"/>
       <c r="L76" s="4" t="inlineStr">
         <is>
-          <t>intervention temporal part</t>
+          <t>contact event</t>
         </is>
       </c>
       <c r="M76" s="4" t="n"/>
       <c r="N76" s="4" t="n"/>
-      <c r="O76" s="4" t="n"/>
+      <c r="O76" s="4" t="inlineStr">
+        <is>
+          <t>is about contact events or is about duration of contact events?</t>
+        </is>
+      </c>
       <c r="P76" s="4" t="n"/>
       <c r="Q76" s="4" t="inlineStr">
         <is>
@@ -4761,7 +4731,7 @@
       </c>
       <c r="T76" s="4" t="inlineStr">
         <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
       <c r="U76" s="4" t="n"/>
@@ -4774,33 +4744,49 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008570</t>
+          <t>BCIO:008555</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>z) interval (remove)</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="n"/>
+          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
+        </is>
+      </c>
       <c r="D77" s="4" t="n"/>
-      <c r="E77" s="4" t="n"/>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="n"/>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>This is not annotated but included due to relationship with duration of interval</t>
-        </is>
-      </c>
-      <c r="I77" s="4" t="n"/>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>The participants took part in 90 minutes of PA "weekly"</t>
+        </is>
+      </c>
       <c r="J77" s="4" t="n"/>
       <c r="K77" s="4" t="n"/>
-      <c r="L77" s="4" t="n"/>
+      <c r="L77" s="4" t="inlineStr">
+        <is>
+          <t>contact event</t>
+        </is>
+      </c>
       <c r="M77" s="4" t="n"/>
       <c r="N77" s="4" t="n"/>
       <c r="O77" s="4" t="inlineStr">
         <is>
-          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+          <t>is about contact events or is about duration of contact events?</t>
         </is>
       </c>
       <c r="P77" s="4" t="n"/>
@@ -4809,13 +4795,21 @@
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R77" s="4" t="n"/>
+      <c r="R77" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="S77" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T77" s="4" t="n"/>
+      <c r="T77" s="4" t="inlineStr">
+        <is>
+          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
+        </is>
+      </c>
       <c r="U77" s="4" t="n"/>
       <c r="V77" s="4" t="inlineStr">
         <is>
@@ -4826,44 +4820,38 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008520</t>
+          <t>BCIO:008600</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>z) intervention temporal part frequency</t>
+          <t>z) frequency period</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
+          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
         </is>
       </c>
       <c r="D78" s="4" t="n"/>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
-        </is>
-      </c>
+          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="n"/>
-      <c r="H78" s="4" t="inlineStr">
-        <is>
-          <t>This is used to capture descriptions of the frequency of contact events within a part. 
-Example annotation (in context)
-intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks"</t>
-        </is>
-      </c>
-      <c r="I78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>Participants received 3 emails every "2" weeks</t>
+        </is>
+      </c>
       <c r="J78" s="4" t="n"/>
       <c r="K78" s="4" t="n"/>
       <c r="L78" s="4" t="inlineStr">
         <is>
-          <t>contact event</t>
+          <t>intervention temporal part</t>
         </is>
       </c>
       <c r="M78" s="4" t="n"/>
@@ -4887,11 +4875,137 @@
       </c>
       <c r="T78" s="4" t="inlineStr">
         <is>
-          <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
         </is>
       </c>
       <c r="U78" s="4" t="n"/>
       <c r="V78" s="4" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008570</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>z) interval (remove)</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="n"/>
+      <c r="D79" s="4" t="n"/>
+      <c r="E79" s="4" t="n"/>
+      <c r="F79" s="4" t="n"/>
+      <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>This is not annotated but included due to relationship with duration of interval</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="n"/>
+      <c r="J79" s="4" t="n"/>
+      <c r="K79" s="4" t="n"/>
+      <c r="L79" s="4" t="n"/>
+      <c r="M79" s="4" t="n"/>
+      <c r="N79" s="4" t="n"/>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+        </is>
+      </c>
+      <c r="P79" s="4" t="n"/>
+      <c r="Q79" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R79" s="4" t="n"/>
+      <c r="S79" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T79" s="4" t="n"/>
+      <c r="U79" s="4" t="n"/>
+      <c r="V79" s="4" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008520</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>z) intervention temporal part frequency</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="n"/>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>This is used to capture descriptions of the frequency of contact events within a part. 
+Example annotation (in context)
+intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks"</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="n"/>
+      <c r="J80" s="4" t="n"/>
+      <c r="K80" s="4" t="n"/>
+      <c r="L80" s="4" t="inlineStr">
+        <is>
+          <t>contact event</t>
+        </is>
+      </c>
+      <c r="M80" s="4" t="n"/>
+      <c r="N80" s="4" t="n"/>
+      <c r="O80" s="4" t="n"/>
+      <c r="P80" s="4" t="n"/>
+      <c r="Q80" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R80" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S80" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T80" s="4" t="inlineStr">
+        <is>
+          <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
+        </is>
+      </c>
+      <c r="U80" s="4" t="n"/>
+      <c r="V80" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>

</xml_diff>

<commit_message>
Edit BCIO_Schedule.xlsx: update 1, add 1
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V80"/>
+  <dimension ref="A1:V81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2100,8 +2100,8 @@
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
@@ -2113,23 +2113,23 @@
           <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr"/>
-      <c r="N30" s="3" t="inlineStr"/>
-      <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="n"/>
+      <c r="N30" s="3" t="n"/>
+      <c r="O30" s="3" t="n"/>
+      <c r="P30" s="3" t="n"/>
       <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R30" s="3" t="inlineStr"/>
-      <c r="S30" s="3" t="inlineStr"/>
-      <c r="T30" s="3" t="inlineStr"/>
-      <c r="U30" s="3" t="inlineStr"/>
-      <c r="V30" s="3" t="inlineStr"/>
+      <c r="R30" s="3" t="n"/>
+      <c r="S30" s="3" t="n"/>
+      <c r="T30" s="3" t="n"/>
+      <c r="U30" s="3" t="n"/>
+      <c r="V30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4124,8 +4124,8 @@
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr"/>
-      <c r="G66" s="3" t="inlineStr"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="n"/>
       <c r="H66" s="3" t="inlineStr">
         <is>
           <t>This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
@@ -4137,23 +4137,23 @@
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
         </is>
       </c>
-      <c r="J66" s="3" t="inlineStr"/>
-      <c r="K66" s="3" t="inlineStr"/>
-      <c r="L66" s="3" t="inlineStr"/>
-      <c r="M66" s="3" t="inlineStr"/>
-      <c r="N66" s="3" t="inlineStr"/>
-      <c r="O66" s="3" t="inlineStr"/>
-      <c r="P66" s="3" t="inlineStr"/>
+      <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="n"/>
+      <c r="L66" s="3" t="n"/>
+      <c r="M66" s="3" t="n"/>
+      <c r="N66" s="3" t="n"/>
+      <c r="O66" s="3" t="n"/>
+      <c r="P66" s="3" t="n"/>
       <c r="Q66" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R66" s="3" t="inlineStr"/>
-      <c r="S66" s="3" t="inlineStr"/>
-      <c r="T66" s="3" t="inlineStr"/>
-      <c r="U66" s="3" t="inlineStr"/>
-      <c r="V66" s="3" t="inlineStr"/>
+      <c r="R66" s="3" t="n"/>
+      <c r="S66" s="3" t="n"/>
+      <c r="T66" s="3" t="n"/>
+      <c r="U66" s="3" t="n"/>
+      <c r="V66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -4348,22 +4348,22 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
+          <t>temporal reference associated with the BCI</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;temporal reference associated with the intervention&gt; against which a BCI  temporal part is referenced.</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
           <t>temporal reference associated with the intervention</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;temporal region&gt; against which a BCI  temporal part is referenced.</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>temporal region</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -4415,34 +4415,96 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051015</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>temporal reference associated with the intervention</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal region&gt; against which an intervention  temporal part is referenced.</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Temporal references are used by authors when there is a behaviourally relevant event which structures the schedule of a BCI. This can include things like quit dates, childbirth, medical operations etc.
+We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr"/>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
+Example annotation in context: "A feedback call was scheduled to be delivered around 6 months after the birth of the baby".</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="inlineStr"/>
+      <c r="M72" s="3" t="inlineStr"/>
+      <c r="N72" s="3" t="inlineStr"/>
+      <c r="O72" s="3" t="inlineStr"/>
+      <c r="P72" s="3" t="inlineStr"/>
+      <c r="Q72" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="R72" s="3" t="inlineStr"/>
+      <c r="S72" s="3" t="inlineStr"/>
+      <c r="T72" s="3" t="inlineStr"/>
+      <c r="U72" s="3" t="inlineStr"/>
+      <c r="V72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>BCIO:008545</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>A &lt;total intervention contact event duration&gt; that is the total of intervention temporal parts within a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>The planned total duration of all sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="F72" s="2" t="n"/>
-      <c r="G72" s="2" t="n"/>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="n"/>
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
 When there is only one session, the total duration of contact events and the duration of a single contact event are technically the same. As a convention, we would annotate this using duration of contact event instead of total duration of contact event. 
@@ -4450,253 +4512,181 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>150 minutes; 12 hours</t>
         </is>
       </c>
-      <c r="J72" s="2" t="n"/>
-      <c r="K72" s="2" t="n"/>
-      <c r="L72" s="2" t="inlineStr">
+      <c r="J73" s="2" t="n"/>
+      <c r="K73" s="2" t="n"/>
+      <c r="L73" s="2" t="inlineStr">
         <is>
           <t>BCI contact event</t>
         </is>
       </c>
-      <c r="M72" s="2" t="n"/>
-      <c r="N72" s="2" t="n"/>
-      <c r="O72" s="2" t="inlineStr">
+      <c r="M73" s="2" t="n"/>
+      <c r="N73" s="2" t="n"/>
+      <c r="O73" s="2" t="inlineStr">
         <is>
           <t>"is about" contact events or "is about" duration of contact events?</t>
         </is>
       </c>
-      <c r="P72" s="2" t="n"/>
-      <c r="Q72" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R72" s="2" t="inlineStr">
+      <c r="P73" s="2" t="n"/>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S72" s="2" t="inlineStr">
+      <c r="S73" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T72" s="2" t="inlineStr">
+      <c r="T73" s="2" t="inlineStr">
         <is>
           <t>what type of data item is this? (CM)</t>
         </is>
       </c>
-      <c r="U72" s="2" t="n"/>
-      <c r="V72" s="2" t="inlineStr">
+      <c r="U73" s="2" t="n"/>
+      <c r="V73" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="3" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>BCIO:051006</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>total intervention contact event duration</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
         </is>
       </c>
-      <c r="D73" s="3" t="n"/>
-      <c r="E73" s="3" t="inlineStr">
+      <c r="D74" s="3" t="n"/>
+      <c r="E74" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="F73" s="3" t="n"/>
-      <c r="G73" s="3" t="n"/>
-      <c r="H73" s="3" t="n"/>
-      <c r="I73" s="3" t="n"/>
-      <c r="J73" s="3" t="n"/>
-      <c r="K73" s="3" t="n"/>
-      <c r="L73" s="3" t="n"/>
-      <c r="M73" s="3" t="n"/>
-      <c r="N73" s="3" t="n"/>
-      <c r="O73" s="3" t="n"/>
-      <c r="P73" s="3" t="n"/>
-      <c r="Q73" s="3" t="inlineStr">
+      <c r="F74" s="3" t="n"/>
+      <c r="G74" s="3" t="n"/>
+      <c r="H74" s="3" t="n"/>
+      <c r="I74" s="3" t="n"/>
+      <c r="J74" s="3" t="n"/>
+      <c r="K74" s="3" t="n"/>
+      <c r="L74" s="3" t="n"/>
+      <c r="M74" s="3" t="n"/>
+      <c r="N74" s="3" t="n"/>
+      <c r="O74" s="3" t="n"/>
+      <c r="P74" s="3" t="n"/>
+      <c r="Q74" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R73" s="3" t="n"/>
-      <c r="S73" s="3" t="n"/>
-      <c r="T73" s="3" t="n"/>
-      <c r="U73" s="3" t="n"/>
-      <c r="V73" s="3" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="R74" s="3" t="n"/>
+      <c r="S74" s="3" t="n"/>
+      <c r="T74" s="3" t="n"/>
+      <c r="U74" s="3" t="n"/>
+      <c r="V74" s="3" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>BCIO:050504</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D74" s="2" t="n"/>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="D75" s="2" t="n"/>
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G74" s="2" t="n"/>
-      <c r="H74" s="2" t="n"/>
-      <c r="I74" s="2" t="n"/>
-      <c r="J74" s="2" t="n"/>
-      <c r="K74" s="2" t="n"/>
-      <c r="L74" s="2" t="inlineStr">
+      <c r="G75" s="2" t="n"/>
+      <c r="H75" s="2" t="n"/>
+      <c r="I75" s="2" t="n"/>
+      <c r="J75" s="2" t="n"/>
+      <c r="K75" s="2" t="n"/>
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>total BCI contact event duration</t>
         </is>
       </c>
-      <c r="M74" s="2" t="n"/>
-      <c r="N74" s="2" t="n"/>
-      <c r="O74" s="2" t="n"/>
-      <c r="P74" s="2" t="n"/>
-      <c r="Q74" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R74" s="2" t="n"/>
-      <c r="S74" s="2" t="n"/>
-      <c r="T74" s="2" t="n"/>
-      <c r="U74" s="2" t="n"/>
-      <c r="V74" s="2" t="inlineStr">
+      <c r="M75" s="2" t="n"/>
+      <c r="N75" s="2" t="n"/>
+      <c r="O75" s="2" t="n"/>
+      <c r="P75" s="2" t="n"/>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="n"/>
+      <c r="S75" s="2" t="n"/>
+      <c r="T75" s="2" t="n"/>
+      <c r="U75" s="2" t="n"/>
+      <c r="V75" s="2" t="inlineStr">
         <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:008605</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="n"/>
-      <c r="E75" s="4" t="n"/>
-      <c r="F75" s="4" t="n"/>
-      <c r="G75" s="4" t="n"/>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
-        </is>
-      </c>
-      <c r="I75" s="4" t="inlineStr">
-        <is>
-          <t>Participants received "3" emails every 2 weeks</t>
-        </is>
-      </c>
-      <c r="J75" s="4" t="n"/>
-      <c r="K75" s="4" t="n"/>
-      <c r="L75" s="4" t="inlineStr">
-        <is>
-          <t>contact event</t>
-        </is>
-      </c>
-      <c r="M75" s="4" t="n"/>
-      <c r="N75" s="4" t="n"/>
-      <c r="O75" s="4" t="n"/>
-      <c r="P75" s="4" t="n"/>
-      <c r="Q75" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R75" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S75" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T75" s="4" t="inlineStr">
-        <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
-        </is>
-      </c>
-      <c r="U75" s="4" t="n"/>
-      <c r="V75" s="4" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008550</t>
+          <t>BCIO:008605</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration (still to confirm inclusion)</t>
+          <t>z) (removed as equivalent to number of contact events) number of repetitions</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
+          <t>A data item that is the number of repetitions of contact events within a temporal part or BCI for which the frequency is described</t>
         </is>
       </c>
       <c r="D76" s="4" t="n"/>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+          <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in "90" minutes of PA weekly</t>
+          <t>Participants received "3" emails every 2 weeks</t>
         </is>
       </c>
       <c r="J76" s="4" t="n"/>
@@ -4708,11 +4698,7 @@
       </c>
       <c r="M76" s="4" t="n"/>
       <c r="N76" s="4" t="n"/>
-      <c r="O76" s="4" t="inlineStr">
-        <is>
-          <t>is about contact events or is about duration of contact events?</t>
-        </is>
-      </c>
+      <c r="O76" s="4" t="n"/>
       <c r="P76" s="4" t="n"/>
       <c r="Q76" s="4" t="inlineStr">
         <is>
@@ -4731,7 +4717,7 @@
       </c>
       <c r="T76" s="4" t="inlineStr">
         <is>
-          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
         </is>
       </c>
       <c r="U76" s="4" t="n"/>
@@ -4744,17 +4730,17 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008555</t>
+          <t>BCIO:008550</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
+          <t>z) contact event sum duration (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
+          <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
         </is>
       </c>
       <c r="D77" s="4" t="n"/>
@@ -4772,7 +4758,7 @@
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>The participants took part in 90 minutes of PA "weekly"</t>
+          <t>The participants took part in "90" minutes of PA weekly</t>
         </is>
       </c>
       <c r="J77" s="4" t="n"/>
@@ -4820,43 +4806,51 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008600</t>
+          <t>BCIO:008555</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>z) frequency period</t>
+          <t>z) contact event sum duration frequency (still to confirm inclusion)</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+          <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
         </is>
       </c>
       <c r="D78" s="4" t="n"/>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="n"/>
-      <c r="H78" s="4" t="n"/>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
       <c r="I78" s="4" t="inlineStr">
         <is>
-          <t>Participants received 3 emails every "2" weeks</t>
+          <t>The participants took part in 90 minutes of PA "weekly"</t>
         </is>
       </c>
       <c r="J78" s="4" t="n"/>
       <c r="K78" s="4" t="n"/>
       <c r="L78" s="4" t="inlineStr">
         <is>
-          <t>intervention temporal part</t>
+          <t>contact event</t>
         </is>
       </c>
       <c r="M78" s="4" t="n"/>
       <c r="N78" s="4" t="n"/>
-      <c r="O78" s="4" t="n"/>
+      <c r="O78" s="4" t="inlineStr">
+        <is>
+          <t>is about contact events or is about duration of contact events?</t>
+        </is>
+      </c>
       <c r="P78" s="4" t="n"/>
       <c r="Q78" s="4" t="inlineStr">
         <is>
@@ -4875,7 +4869,7 @@
       </c>
       <c r="T78" s="4" t="inlineStr">
         <is>
-          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+          <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
       <c r="U78" s="4" t="n"/>
@@ -4888,48 +4882,64 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008570</t>
+          <t>BCIO:008600</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>z) interval (remove)</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="n"/>
+          <t>z) frequency period</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
+        </is>
+      </c>
       <c r="D79" s="4" t="n"/>
-      <c r="E79" s="4" t="n"/>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
+        </is>
+      </c>
       <c r="F79" s="4" t="n"/>
       <c r="G79" s="4" t="n"/>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated but included due to relationship with duration of interval</t>
-        </is>
-      </c>
-      <c r="I79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>Participants received 3 emails every "2" weeks</t>
+        </is>
+      </c>
       <c r="J79" s="4" t="n"/>
       <c r="K79" s="4" t="n"/>
-      <c r="L79" s="4" t="n"/>
+      <c r="L79" s="4" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
       <c r="M79" s="4" t="n"/>
       <c r="N79" s="4" t="n"/>
-      <c r="O79" s="4" t="inlineStr">
-        <is>
-          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
-        </is>
-      </c>
+      <c r="O79" s="4" t="n"/>
       <c r="P79" s="4" t="n"/>
       <c r="Q79" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R79" s="4" t="n"/>
+      <c r="R79" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="S79" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T79" s="4" t="n"/>
+      <c r="T79" s="4" t="inlineStr">
+        <is>
+          <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
+        </is>
+      </c>
       <c r="U79" s="4" t="n"/>
       <c r="V79" s="4" t="inlineStr">
         <is>
@@ -4940,72 +4950,124 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>BCIO:008520</t>
+          <t>BCIO:008570</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>z) intervention temporal part frequency</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
-        </is>
-      </c>
+          <t>z) interval (remove)</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="n"/>
       <c r="D80" s="4" t="n"/>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
-        </is>
-      </c>
+      <c r="E80" s="4" t="n"/>
+      <c r="F80" s="4" t="n"/>
       <c r="G80" s="4" t="n"/>
       <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>This is not annotated but included due to relationship with duration of interval</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="n"/>
+      <c r="J80" s="4" t="n"/>
+      <c r="K80" s="4" t="n"/>
+      <c r="L80" s="4" t="n"/>
+      <c r="M80" s="4" t="n"/>
+      <c r="N80" s="4" t="n"/>
+      <c r="O80" s="4" t="inlineStr">
+        <is>
+          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+        </is>
+      </c>
+      <c r="P80" s="4" t="n"/>
+      <c r="Q80" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="R80" s="4" t="n"/>
+      <c r="S80" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T80" s="4" t="n"/>
+      <c r="U80" s="4" t="n"/>
+      <c r="V80" s="4" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:008520</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>z) intervention temporal part frequency</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="n"/>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="inlineStr">
         <is>
           <t>This is used to capture descriptions of the frequency of contact events within a part. 
 Example annotation (in context)
 intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks"</t>
         </is>
       </c>
-      <c r="I80" s="4" t="n"/>
-      <c r="J80" s="4" t="n"/>
-      <c r="K80" s="4" t="n"/>
-      <c r="L80" s="4" t="inlineStr">
+      <c r="I81" s="4" t="n"/>
+      <c r="J81" s="4" t="n"/>
+      <c r="K81" s="4" t="n"/>
+      <c r="L81" s="4" t="inlineStr">
         <is>
           <t>contact event</t>
         </is>
       </c>
-      <c r="M80" s="4" t="n"/>
-      <c r="N80" s="4" t="n"/>
-      <c r="O80" s="4" t="n"/>
-      <c r="P80" s="4" t="n"/>
-      <c r="Q80" s="4" t="inlineStr">
+      <c r="M81" s="4" t="n"/>
+      <c r="N81" s="4" t="n"/>
+      <c r="O81" s="4" t="n"/>
+      <c r="P81" s="4" t="n"/>
+      <c r="Q81" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R80" s="4" t="inlineStr">
+      <c r="R81" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S80" s="4" t="inlineStr">
+      <c r="S81" s="4" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T80" s="4" t="inlineStr">
+      <c r="T81" s="4" t="inlineStr">
         <is>
           <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
         </is>
       </c>
-      <c r="U80" s="4" t="n"/>
-      <c r="V80" s="4" t="inlineStr">
+      <c r="U81" s="4" t="n"/>
+      <c r="V81" s="4" t="inlineStr">
         <is>
           <t>CM</t>
         </is>

</xml_diff>

<commit_message>
Update interval between intervention temporal parts in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -472,77 +472,77 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Curator note</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Annotation rules</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'part of'</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has attribute' [RO:0000053]</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'is about' [IAO:0000136]</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'is attribute of' [RO:0000052]</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'occupies temporal region' [BFO:0000155]</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>To be reviewed by</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Definition_Source</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Logical definition</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Annotation rules</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Examples</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'part of'</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has attribute' [RO:0000053]</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'is about' [IAO:0000136]</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'is attribute of' [RO:0000052]</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'occupies temporal region' [BFO:0000155]</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Curator note</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Definition_Source</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Aggregate</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Curation status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Aggregate</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>To be reviewed by</t>
-        </is>
-      </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>Definition_ID</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Definition_ID</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -596,13 +596,13 @@
       </c>
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="inlineStr">
@@ -648,13 +648,13 @@
       <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="n"/>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="n"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="n"/>
       <c r="V3" s="2" t="inlineStr">
@@ -713,13 +713,13 @@
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="n"/>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T4" s="2" t="n"/>
       <c r="U4" s="2" t="n"/>
       <c r="V4" s="2" t="inlineStr">
@@ -773,13 +773,13 @@
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n"/>
-      <c r="O5" s="2" t="n"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
@@ -787,7 +787,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T5" s="2" t="n"/>
@@ -839,13 +839,13 @@
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="n"/>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q6" s="2" t="n"/>
       <c r="R6" s="2" t="n"/>
-      <c r="S6" s="2" t="n"/>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="n"/>
       <c r="V6" s="2" t="inlineStr">
@@ -911,17 +911,17 @@
           <t>BCI temporal part duration</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q7" s="2" t="n"/>
       <c r="R7" s="2" t="n"/>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T7" s="2" t="n"/>
@@ -977,13 +977,13 @@
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
-      <c r="O8" s="2" t="n"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P8" s="2" t="n"/>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
@@ -991,7 +991,7 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T8" s="2" t="n"/>
@@ -1056,13 +1056,13 @@
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="n"/>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q9" s="2" t="n"/>
       <c r="R9" s="2" t="n"/>
-      <c r="S9" s="2" t="n"/>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T9" s="2" t="n"/>
       <c r="U9" s="2" t="n"/>
       <c r="V9" s="2" t="inlineStr">
@@ -1108,13 +1108,13 @@
       </c>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q10" s="2" t="n"/>
       <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="n"/>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T10" s="2" t="n"/>
       <c r="U10" s="2" t="n"/>
       <c r="V10" s="2" t="n"/>
@@ -1140,7 +1140,7 @@
           <t>specifically dependent continuant</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1200,13 +1200,13 @@
       </c>
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
-      <c r="O12" s="2" t="n"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P12" s="2" t="n"/>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q12" s="2" t="n"/>
       <c r="R12" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T12" s="2" t="n"/>
@@ -1228,7 +1228,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050999</t>
+          <t>BCIO:051017</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1258,13 +1258,13 @@
       <c r="N13" s="3" t="n"/>
       <c r="O13" s="3" t="n"/>
       <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="Q13" s="3" t="n"/>
+      <c r="R13" s="3" t="n"/>
+      <c r="S13" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3" t="n"/>
       <c r="T13" s="3" t="n"/>
       <c r="U13" s="3" t="n"/>
       <c r="V13" s="3" t="n"/>
@@ -1302,13 +1302,13 @@
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="n"/>
-      <c r="Q14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q14" s="2" t="n"/>
       <c r="R14" s="2" t="n"/>
-      <c r="S14" s="2" t="n"/>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T14" s="2" t="n"/>
       <c r="U14" s="2" t="n"/>
       <c r="V14" s="2" t="n"/>
@@ -1346,13 +1346,13 @@
       <c r="N15" s="3" t="n"/>
       <c r="O15" s="3" t="n"/>
       <c r="P15" s="3" t="n"/>
-      <c r="Q15" s="3" t="inlineStr">
+      <c r="Q15" s="3" t="n"/>
+      <c r="R15" s="3" t="n"/>
+      <c r="S15" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R15" s="3" t="n"/>
-      <c r="S15" s="3" t="n"/>
       <c r="T15" s="3" t="n"/>
       <c r="U15" s="3" t="n"/>
       <c r="V15" s="3" t="n"/>
@@ -1390,13 +1390,13 @@
       <c r="N16" s="3" t="n"/>
       <c r="O16" s="3" t="n"/>
       <c r="P16" s="3" t="n"/>
-      <c r="Q16" s="3" t="inlineStr">
+      <c r="Q16" s="3" t="n"/>
+      <c r="R16" s="3" t="n"/>
+      <c r="S16" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R16" s="3" t="n"/>
-      <c r="S16" s="3" t="n"/>
       <c r="T16" s="3" t="n"/>
       <c r="U16" s="3" t="n"/>
       <c r="V16" s="3" t="n"/>
@@ -1442,13 +1442,13 @@
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="n"/>
-      <c r="Q17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q17" s="2" t="n"/>
       <c r="R17" s="2" t="n"/>
-      <c r="S17" s="2" t="n"/>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T17" s="2" t="n"/>
       <c r="U17" s="2" t="n"/>
       <c r="V17" s="2" t="inlineStr">
@@ -1490,13 +1490,13 @@
       <c r="N18" s="3" t="n"/>
       <c r="O18" s="3" t="n"/>
       <c r="P18" s="3" t="n"/>
-      <c r="Q18" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="n"/>
+      <c r="R18" s="3" t="n"/>
+      <c r="S18" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R18" s="3" t="n"/>
-      <c r="S18" s="3" t="n"/>
       <c r="T18" s="3" t="n"/>
       <c r="U18" s="3" t="n"/>
       <c r="V18" s="3" t="n"/>
@@ -1542,13 +1542,13 @@
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="n"/>
-      <c r="Q19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q19" s="2" t="n"/>
       <c r="R19" s="2" t="n"/>
-      <c r="S19" s="2" t="n"/>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T19" s="2" t="n"/>
       <c r="U19" s="2" t="n"/>
       <c r="V19" s="2" t="inlineStr">
@@ -1598,13 +1598,13 @@
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q20" s="2" t="n"/>
       <c r="R20" s="2" t="n"/>
-      <c r="S20" s="2" t="n"/>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T20" s="2" t="n"/>
       <c r="U20" s="2" t="n"/>
       <c r="V20" s="2" t="inlineStr">
@@ -1646,13 +1646,13 @@
       <c r="N21" s="3" t="n"/>
       <c r="O21" s="3" t="n"/>
       <c r="P21" s="3" t="n"/>
-      <c r="Q21" s="3" t="inlineStr">
+      <c r="Q21" s="3" t="n"/>
+      <c r="R21" s="3" t="n"/>
+      <c r="S21" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R21" s="3" t="n"/>
-      <c r="S21" s="3" t="n"/>
       <c r="T21" s="3" t="n"/>
       <c r="U21" s="3" t="n"/>
       <c r="V21" s="3" t="n"/>
@@ -1698,13 +1698,13 @@
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="n"/>
-      <c r="Q22" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q22" s="2" t="n"/>
       <c r="R22" s="2" t="n"/>
-      <c r="S22" s="2" t="n"/>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T22" s="2" t="n"/>
       <c r="U22" s="2" t="n"/>
       <c r="V22" s="2" t="inlineStr">
@@ -1746,13 +1746,13 @@
       <c r="N23" s="3" t="n"/>
       <c r="O23" s="3" t="n"/>
       <c r="P23" s="3" t="n"/>
-      <c r="Q23" s="3" t="inlineStr">
+      <c r="Q23" s="3" t="n"/>
+      <c r="R23" s="3" t="n"/>
+      <c r="S23" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R23" s="3" t="n"/>
-      <c r="S23" s="3" t="n"/>
       <c r="T23" s="3" t="n"/>
       <c r="U23" s="3" t="n"/>
       <c r="V23" s="3" t="n"/>
@@ -1790,13 +1790,13 @@
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="n"/>
-      <c r="Q24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q24" s="2" t="n"/>
       <c r="R24" s="2" t="n"/>
-      <c r="S24" s="2" t="n"/>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T24" s="2" t="n"/>
       <c r="U24" s="2" t="n"/>
       <c r="V24" s="2" t="n"/>
@@ -1834,13 +1834,13 @@
       <c r="N25" s="3" t="n"/>
       <c r="O25" s="3" t="n"/>
       <c r="P25" s="3" t="n"/>
-      <c r="Q25" s="3" t="inlineStr">
+      <c r="Q25" s="3" t="n"/>
+      <c r="R25" s="3" t="n"/>
+      <c r="S25" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R25" s="3" t="n"/>
-      <c r="S25" s="3" t="n"/>
       <c r="T25" s="3" t="n"/>
       <c r="U25" s="3" t="n"/>
       <c r="V25" s="3" t="n"/>
@@ -1886,13 +1886,13 @@
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
-      <c r="Q26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
-      <c r="S26" s="2" t="n"/>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T26" s="2" t="n"/>
       <c r="U26" s="2" t="n"/>
       <c r="V26" s="2" t="inlineStr">
@@ -1938,13 +1938,13 @@
       <c r="N27" s="3" t="n"/>
       <c r="O27" s="3" t="n"/>
       <c r="P27" s="3" t="n"/>
-      <c r="Q27" s="3" t="inlineStr">
+      <c r="Q27" s="3" t="n"/>
+      <c r="R27" s="3" t="n"/>
+      <c r="S27" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R27" s="3" t="n"/>
-      <c r="S27" s="3" t="n"/>
       <c r="T27" s="3" t="n"/>
       <c r="U27" s="3" t="n"/>
       <c r="V27" s="3" t="n"/>
@@ -1990,13 +1990,13 @@
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="n"/>
-      <c r="Q28" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q28" s="2" t="n"/>
       <c r="R28" s="2" t="n"/>
-      <c r="S28" s="2" t="n"/>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T28" s="2" t="n"/>
       <c r="U28" s="2" t="n"/>
       <c r="V28" s="2" t="inlineStr">
@@ -2049,25 +2049,25 @@
       <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="n"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P29" s="2" t="n"/>
-      <c r="Q29" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q29" s="2" t="n"/>
       <c r="R29" s="2" t="n"/>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T29" s="2" t="inlineStr">
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="n"/>
+      <c r="U29" s="2" t="inlineStr">
         <is>
           <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
         </is>
       </c>
-      <c r="U29" s="2" t="n"/>
       <c r="V29" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
@@ -2120,13 +2120,13 @@
       <c r="N30" s="3" t="n"/>
       <c r="O30" s="3" t="n"/>
       <c r="P30" s="3" t="n"/>
-      <c r="Q30" s="3" t="inlineStr">
+      <c r="Q30" s="3" t="n"/>
+      <c r="R30" s="3" t="n"/>
+      <c r="S30" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R30" s="3" t="n"/>
-      <c r="S30" s="3" t="n"/>
       <c r="T30" s="3" t="n"/>
       <c r="U30" s="3" t="n"/>
       <c r="V30" s="3" t="n"/>
@@ -2172,13 +2172,13 @@
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q31" s="2" t="n"/>
       <c r="R31" s="2" t="n"/>
-      <c r="S31" s="2" t="n"/>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T31" s="2" t="n"/>
       <c r="U31" s="2" t="n"/>
       <c r="V31" s="2" t="inlineStr">
@@ -2228,13 +2228,13 @@
       <c r="N32" s="2" t="n"/>
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="n"/>
-      <c r="Q32" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q32" s="2" t="n"/>
       <c r="R32" s="2" t="n"/>
-      <c r="S32" s="2" t="n"/>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T32" s="2" t="n"/>
       <c r="U32" s="2" t="n"/>
       <c r="V32" s="2" t="inlineStr">
@@ -2284,13 +2284,13 @@
       <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="n"/>
-      <c r="Q33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q33" s="2" t="n"/>
       <c r="R33" s="2" t="n"/>
-      <c r="S33" s="2" t="n"/>
+      <c r="S33" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T33" s="2" t="n"/>
       <c r="U33" s="2" t="n"/>
       <c r="V33" s="2" t="inlineStr">
@@ -2340,13 +2340,13 @@
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="n"/>
-      <c r="Q34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q34" s="2" t="n"/>
       <c r="R34" s="2" t="n"/>
-      <c r="S34" s="2" t="n"/>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T34" s="2" t="n"/>
       <c r="U34" s="2" t="n"/>
       <c r="V34" s="2" t="inlineStr">
@@ -2396,13 +2396,13 @@
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="n"/>
-      <c r="Q35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q35" s="2" t="n"/>
       <c r="R35" s="2" t="n"/>
-      <c r="S35" s="2" t="n"/>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T35" s="2" t="n"/>
       <c r="U35" s="2" t="n"/>
       <c r="V35" s="2" t="inlineStr">
@@ -2452,13 +2452,13 @@
       <c r="N36" s="2" t="n"/>
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="n"/>
-      <c r="Q36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q36" s="2" t="n"/>
       <c r="R36" s="2" t="n"/>
-      <c r="S36" s="2" t="n"/>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T36" s="2" t="n"/>
       <c r="U36" s="2" t="n"/>
       <c r="V36" s="2" t="inlineStr">
@@ -2508,13 +2508,13 @@
       <c r="N37" s="2" t="n"/>
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="n"/>
-      <c r="Q37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q37" s="2" t="n"/>
       <c r="R37" s="2" t="n"/>
-      <c r="S37" s="2" t="n"/>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T37" s="2" t="n"/>
       <c r="U37" s="2" t="n"/>
       <c r="V37" s="2" t="inlineStr">
@@ -2564,13 +2564,13 @@
       <c r="N38" s="2" t="n"/>
       <c r="O38" s="2" t="n"/>
       <c r="P38" s="2" t="n"/>
-      <c r="Q38" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q38" s="2" t="n"/>
       <c r="R38" s="2" t="n"/>
-      <c r="S38" s="2" t="n"/>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T38" s="2" t="n"/>
       <c r="U38" s="2" t="n"/>
       <c r="V38" s="2" t="inlineStr">
@@ -2620,13 +2620,13 @@
       <c r="N39" s="2" t="n"/>
       <c r="O39" s="2" t="n"/>
       <c r="P39" s="2" t="n"/>
-      <c r="Q39" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q39" s="2" t="n"/>
       <c r="R39" s="2" t="n"/>
-      <c r="S39" s="2" t="n"/>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T39" s="2" t="n"/>
       <c r="U39" s="2" t="n"/>
       <c r="V39" s="2" t="inlineStr">
@@ -2676,13 +2676,13 @@
       <c r="N40" s="2" t="n"/>
       <c r="O40" s="2" t="n"/>
       <c r="P40" s="2" t="n"/>
-      <c r="Q40" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q40" s="2" t="n"/>
       <c r="R40" s="2" t="n"/>
-      <c r="S40" s="2" t="n"/>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T40" s="2" t="n"/>
       <c r="U40" s="2" t="n"/>
       <c r="V40" s="2" t="inlineStr">
@@ -2732,13 +2732,13 @@
       <c r="N41" s="2" t="n"/>
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="n"/>
-      <c r="Q41" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q41" s="2" t="n"/>
       <c r="R41" s="2" t="n"/>
-      <c r="S41" s="2" t="n"/>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T41" s="2" t="n"/>
       <c r="U41" s="2" t="n"/>
       <c r="V41" s="2" t="inlineStr">
@@ -2788,13 +2788,13 @@
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="n"/>
-      <c r="Q42" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q42" s="2" t="n"/>
       <c r="R42" s="2" t="n"/>
-      <c r="S42" s="2" t="n"/>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T42" s="2" t="n"/>
       <c r="U42" s="2" t="n"/>
       <c r="V42" s="2" t="inlineStr">
@@ -2844,13 +2844,13 @@
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="2" t="n"/>
       <c r="P43" s="2" t="n"/>
-      <c r="Q43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q43" s="2" t="n"/>
       <c r="R43" s="2" t="n"/>
-      <c r="S43" s="2" t="n"/>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T43" s="2" t="n"/>
       <c r="U43" s="2" t="n"/>
       <c r="V43" s="2" t="inlineStr">
@@ -2900,13 +2900,13 @@
       <c r="N44" s="2" t="n"/>
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="n"/>
-      <c r="Q44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q44" s="2" t="n"/>
       <c r="R44" s="2" t="n"/>
-      <c r="S44" s="2" t="n"/>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T44" s="2" t="n"/>
       <c r="U44" s="2" t="n"/>
       <c r="V44" s="2" t="inlineStr">
@@ -2956,13 +2956,13 @@
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
       <c r="P45" s="2" t="n"/>
-      <c r="Q45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q45" s="2" t="n"/>
       <c r="R45" s="2" t="n"/>
-      <c r="S45" s="2" t="n"/>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T45" s="2" t="n"/>
       <c r="U45" s="2" t="n"/>
       <c r="V45" s="2" t="inlineStr">
@@ -3012,13 +3012,13 @@
       <c r="N46" s="2" t="n"/>
       <c r="O46" s="2" t="n"/>
       <c r="P46" s="2" t="n"/>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q46" s="2" t="n"/>
       <c r="R46" s="2" t="n"/>
-      <c r="S46" s="2" t="n"/>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T46" s="2" t="n"/>
       <c r="U46" s="2" t="n"/>
       <c r="V46" s="2" t="inlineStr">
@@ -3068,13 +3068,13 @@
       <c r="N47" s="2" t="n"/>
       <c r="O47" s="2" t="n"/>
       <c r="P47" s="2" t="n"/>
-      <c r="Q47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q47" s="2" t="n"/>
       <c r="R47" s="2" t="n"/>
-      <c r="S47" s="2" t="n"/>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T47" s="2" t="n"/>
       <c r="U47" s="2" t="n"/>
       <c r="V47" s="2" t="inlineStr">
@@ -3124,13 +3124,13 @@
       <c r="N48" s="2" t="n"/>
       <c r="O48" s="2" t="n"/>
       <c r="P48" s="2" t="n"/>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q48" s="2" t="n"/>
       <c r="R48" s="2" t="n"/>
-      <c r="S48" s="2" t="n"/>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T48" s="2" t="n"/>
       <c r="U48" s="2" t="n"/>
       <c r="V48" s="2" t="inlineStr">
@@ -3180,13 +3180,13 @@
       <c r="N49" s="2" t="n"/>
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="n"/>
-      <c r="Q49" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q49" s="2" t="n"/>
       <c r="R49" s="2" t="n"/>
-      <c r="S49" s="2" t="n"/>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T49" s="2" t="n"/>
       <c r="U49" s="2" t="n"/>
       <c r="V49" s="2" t="inlineStr">
@@ -3236,13 +3236,13 @@
       <c r="N50" s="2" t="n"/>
       <c r="O50" s="2" t="n"/>
       <c r="P50" s="2" t="n"/>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q50" s="2" t="n"/>
       <c r="R50" s="2" t="n"/>
-      <c r="S50" s="2" t="n"/>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T50" s="2" t="n"/>
       <c r="U50" s="2" t="n"/>
       <c r="V50" s="2" t="inlineStr">
@@ -3292,13 +3292,13 @@
       <c r="N51" s="2" t="n"/>
       <c r="O51" s="2" t="n"/>
       <c r="P51" s="2" t="n"/>
-      <c r="Q51" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q51" s="2" t="n"/>
       <c r="R51" s="2" t="n"/>
-      <c r="S51" s="2" t="n"/>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T51" s="2" t="n"/>
       <c r="U51" s="2" t="n"/>
       <c r="V51" s="2" t="inlineStr">
@@ -3348,13 +3348,13 @@
       <c r="N52" s="2" t="n"/>
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="n"/>
-      <c r="Q52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q52" s="2" t="n"/>
       <c r="R52" s="2" t="n"/>
-      <c r="S52" s="2" t="n"/>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T52" s="2" t="n"/>
       <c r="U52" s="2" t="n"/>
       <c r="V52" s="2" t="inlineStr">
@@ -3404,13 +3404,13 @@
       <c r="N53" s="2" t="n"/>
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="n"/>
-      <c r="Q53" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q53" s="2" t="n"/>
       <c r="R53" s="2" t="n"/>
-      <c r="S53" s="2" t="n"/>
+      <c r="S53" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T53" s="2" t="n"/>
       <c r="U53" s="2" t="n"/>
       <c r="V53" s="2" t="inlineStr">
@@ -3460,13 +3460,13 @@
       <c r="N54" s="2" t="n"/>
       <c r="O54" s="2" t="n"/>
       <c r="P54" s="2" t="n"/>
-      <c r="Q54" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q54" s="2" t="n"/>
       <c r="R54" s="2" t="n"/>
-      <c r="S54" s="2" t="n"/>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T54" s="2" t="n"/>
       <c r="U54" s="2" t="n"/>
       <c r="V54" s="2" t="inlineStr">
@@ -3516,13 +3516,13 @@
       <c r="N55" s="2" t="n"/>
       <c r="O55" s="2" t="n"/>
       <c r="P55" s="2" t="n"/>
-      <c r="Q55" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q55" s="2" t="n"/>
       <c r="R55" s="2" t="n"/>
-      <c r="S55" s="2" t="n"/>
+      <c r="S55" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T55" s="2" t="n"/>
       <c r="U55" s="2" t="n"/>
       <c r="V55" s="2" t="inlineStr">
@@ -3572,13 +3572,13 @@
       <c r="N56" s="2" t="n"/>
       <c r="O56" s="2" t="n"/>
       <c r="P56" s="2" t="n"/>
-      <c r="Q56" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q56" s="2" t="n"/>
       <c r="R56" s="2" t="n"/>
-      <c r="S56" s="2" t="n"/>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T56" s="2" t="n"/>
       <c r="U56" s="2" t="n"/>
       <c r="V56" s="2" t="inlineStr">
@@ -3628,13 +3628,13 @@
       <c r="N57" s="2" t="n"/>
       <c r="O57" s="2" t="n"/>
       <c r="P57" s="2" t="n"/>
-      <c r="Q57" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q57" s="2" t="n"/>
       <c r="R57" s="2" t="n"/>
-      <c r="S57" s="2" t="n"/>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T57" s="2" t="n"/>
       <c r="U57" s="2" t="n"/>
       <c r="V57" s="2" t="inlineStr">
@@ -3684,13 +3684,13 @@
       <c r="N58" s="2" t="n"/>
       <c r="O58" s="2" t="n"/>
       <c r="P58" s="2" t="n"/>
-      <c r="Q58" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q58" s="2" t="n"/>
       <c r="R58" s="2" t="n"/>
-      <c r="S58" s="2" t="n"/>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T58" s="2" t="n"/>
       <c r="U58" s="2" t="n"/>
       <c r="V58" s="2" t="inlineStr">
@@ -3748,13 +3748,13 @@
       </c>
       <c r="M59" s="2" t="n"/>
       <c r="N59" s="2" t="n"/>
-      <c r="O59" s="2" t="n"/>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P59" s="2" t="n"/>
-      <c r="Q59" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q59" s="2" t="n"/>
       <c r="R59" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="S59" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T59" s="2" t="n"/>
@@ -3806,13 +3806,13 @@
       <c r="N60" s="3" t="n"/>
       <c r="O60" s="3" t="n"/>
       <c r="P60" s="3" t="n"/>
-      <c r="Q60" s="3" t="inlineStr">
+      <c r="Q60" s="3" t="n"/>
+      <c r="R60" s="3" t="n"/>
+      <c r="S60" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R60" s="3" t="n"/>
-      <c r="S60" s="3" t="n"/>
       <c r="T60" s="3" t="n"/>
       <c r="U60" s="3" t="n"/>
       <c r="V60" s="3" t="n"/>
@@ -3864,17 +3864,17 @@
         </is>
       </c>
       <c r="N61" s="2" t="n"/>
-      <c r="O61" s="2" t="n"/>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P61" s="2" t="n"/>
-      <c r="Q61" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q61" s="2" t="n"/>
       <c r="R61" s="2" t="n"/>
       <c r="S61" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T61" s="2" t="n"/>
@@ -3918,13 +3918,13 @@
       <c r="N62" s="3" t="n"/>
       <c r="O62" s="3" t="n"/>
       <c r="P62" s="3" t="n"/>
-      <c r="Q62" s="3" t="inlineStr">
+      <c r="Q62" s="3" t="n"/>
+      <c r="R62" s="3" t="n"/>
+      <c r="S62" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R62" s="3" t="n"/>
-      <c r="S62" s="3" t="n"/>
       <c r="T62" s="3" t="n"/>
       <c r="U62" s="3" t="n"/>
       <c r="V62" s="3" t="n"/>
@@ -3960,17 +3960,17 @@
       <c r="L63" s="4" t="n"/>
       <c r="M63" s="4" t="n"/>
       <c r="N63" s="4" t="n"/>
-      <c r="O63" s="4" t="n"/>
+      <c r="O63" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P63" s="4" t="n"/>
-      <c r="Q63" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q63" s="4" t="n"/>
       <c r="R63" s="4" t="n"/>
       <c r="S63" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="T63" s="4" t="n"/>
@@ -4012,17 +4012,17 @@
       <c r="L64" s="4" t="n"/>
       <c r="M64" s="4" t="n"/>
       <c r="N64" s="4" t="n"/>
-      <c r="O64" s="4" t="n"/>
+      <c r="O64" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P64" s="4" t="n"/>
-      <c r="Q64" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q64" s="4" t="n"/>
       <c r="R64" s="4" t="n"/>
       <c r="S64" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="T64" s="4" t="n"/>
@@ -4077,17 +4077,17 @@
       <c r="L65" s="2" t="n"/>
       <c r="M65" s="2" t="n"/>
       <c r="N65" s="2" t="n"/>
-      <c r="O65" s="2" t="n"/>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P65" s="2" t="n"/>
-      <c r="Q65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q65" s="2" t="n"/>
       <c r="R65" s="2" t="n"/>
       <c r="S65" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T65" s="2" t="n"/>
@@ -4144,13 +4144,13 @@
       <c r="N66" s="3" t="n"/>
       <c r="O66" s="3" t="n"/>
       <c r="P66" s="3" t="n"/>
-      <c r="Q66" s="3" t="inlineStr">
+      <c r="Q66" s="3" t="n"/>
+      <c r="R66" s="3" t="n"/>
+      <c r="S66" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R66" s="3" t="n"/>
-      <c r="S66" s="3" t="n"/>
       <c r="T66" s="3" t="n"/>
       <c r="U66" s="3" t="n"/>
       <c r="V66" s="3" t="n"/>
@@ -4186,17 +4186,17 @@
       <c r="L67" s="4" t="n"/>
       <c r="M67" s="4" t="n"/>
       <c r="N67" s="4" t="n"/>
-      <c r="O67" s="4" t="n"/>
+      <c r="O67" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P67" s="4" t="n"/>
-      <c r="Q67" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q67" s="4" t="n"/>
       <c r="R67" s="4" t="n"/>
       <c r="S67" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="T67" s="4" t="n"/>
@@ -4228,7 +4228,7 @@
           <t>occurrent</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr">
+      <c r="S68" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -4273,13 +4273,13 @@
       <c r="N69" s="4" t="n"/>
       <c r="O69" s="4" t="n"/>
       <c r="P69" s="4" t="n"/>
-      <c r="Q69" s="4" t="inlineStr">
+      <c r="Q69" s="4" t="n"/>
+      <c r="R69" s="4" t="n"/>
+      <c r="S69" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R69" s="4" t="n"/>
-      <c r="S69" s="4" t="n"/>
       <c r="T69" s="4" t="n"/>
       <c r="U69" s="4" t="n"/>
       <c r="V69" s="4" t="inlineStr">
@@ -4325,13 +4325,13 @@
       <c r="N70" s="4" t="n"/>
       <c r="O70" s="4" t="n"/>
       <c r="P70" s="4" t="n"/>
-      <c r="Q70" s="4" t="inlineStr">
+      <c r="Q70" s="4" t="n"/>
+      <c r="R70" s="4" t="n"/>
+      <c r="S70" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R70" s="4" t="n"/>
-      <c r="S70" s="4" t="n"/>
       <c r="T70" s="4" t="n"/>
       <c r="U70" s="4" t="n"/>
       <c r="V70" s="4" t="inlineStr">
@@ -4393,17 +4393,17 @@
       <c r="L71" s="2" t="n"/>
       <c r="M71" s="2" t="n"/>
       <c r="N71" s="2" t="n"/>
-      <c r="O71" s="2" t="n"/>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P71" s="2" t="n"/>
-      <c r="Q71" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q71" s="2" t="n"/>
       <c r="R71" s="2" t="n"/>
       <c r="S71" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="T71" s="2" t="n"/>
@@ -4446,7 +4446,7 @@
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr"/>
+      <c r="G72" s="3" t="n"/>
       <c r="H72" s="3" t="inlineStr">
         <is>
           <t>Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
@@ -4458,23 +4458,23 @@
           <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
         </is>
       </c>
-      <c r="J72" s="3" t="inlineStr"/>
-      <c r="K72" s="3" t="inlineStr"/>
-      <c r="L72" s="3" t="inlineStr"/>
-      <c r="M72" s="3" t="inlineStr"/>
-      <c r="N72" s="3" t="inlineStr"/>
-      <c r="O72" s="3" t="inlineStr"/>
-      <c r="P72" s="3" t="inlineStr"/>
-      <c r="Q72" s="3" t="inlineStr">
+      <c r="J72" s="3" t="n"/>
+      <c r="K72" s="3" t="n"/>
+      <c r="L72" s="3" t="n"/>
+      <c r="M72" s="3" t="n"/>
+      <c r="N72" s="3" t="n"/>
+      <c r="O72" s="3" t="n"/>
+      <c r="P72" s="3" t="n"/>
+      <c r="Q72" s="3" t="n"/>
+      <c r="R72" s="3" t="n"/>
+      <c r="S72" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R72" s="3" t="inlineStr"/>
-      <c r="S72" s="3" t="inlineStr"/>
-      <c r="T72" s="3" t="inlineStr"/>
-      <c r="U72" s="3" t="inlineStr"/>
-      <c r="V72" s="3" t="inlineStr"/>
+      <c r="T72" s="3" t="n"/>
+      <c r="U72" s="3" t="n"/>
+      <c r="V72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4503,7 +4503,11 @@
         </is>
       </c>
       <c r="F73" s="2" t="n"/>
-      <c r="G73" s="2" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>"is about" contact events or "is about" duration of contact events?</t>
+        </is>
+      </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
@@ -4528,15 +4532,11 @@
       <c r="N73" s="2" t="n"/>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>"is about" contact events or "is about" duration of contact events?</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="P73" s="2" t="n"/>
-      <c r="Q73" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q73" s="2" t="n"/>
       <c r="R73" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
@@ -4544,15 +4544,15 @@
       </c>
       <c r="S73" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T73" s="2" t="inlineStr">
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T73" s="2" t="n"/>
+      <c r="U73" s="2" t="inlineStr">
         <is>
           <t>what type of data item is this? (CM)</t>
         </is>
       </c>
-      <c r="U73" s="2" t="n"/>
       <c r="V73" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
@@ -4592,13 +4592,13 @@
       <c r="N74" s="3" t="n"/>
       <c r="O74" s="3" t="n"/>
       <c r="P74" s="3" t="n"/>
-      <c r="Q74" s="3" t="inlineStr">
+      <c r="Q74" s="3" t="n"/>
+      <c r="R74" s="3" t="n"/>
+      <c r="S74" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="R74" s="3" t="n"/>
-      <c r="S74" s="3" t="n"/>
       <c r="T74" s="3" t="n"/>
       <c r="U74" s="3" t="n"/>
       <c r="V74" s="3" t="n"/>
@@ -4644,13 +4644,13 @@
       <c r="N75" s="2" t="n"/>
       <c r="O75" s="2" t="n"/>
       <c r="P75" s="2" t="n"/>
-      <c r="Q75" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q75" s="2" t="n"/>
       <c r="R75" s="2" t="n"/>
-      <c r="S75" s="2" t="n"/>
+      <c r="S75" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="T75" s="2" t="n"/>
       <c r="U75" s="2" t="n"/>
       <c r="V75" s="2" t="inlineStr">
@@ -4698,29 +4698,29 @@
       </c>
       <c r="M76" s="4" t="n"/>
       <c r="N76" s="4" t="n"/>
-      <c r="O76" s="4" t="n"/>
+      <c r="O76" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P76" s="4" t="n"/>
-      <c r="Q76" s="4" t="inlineStr">
+      <c r="Q76" s="4" t="n"/>
+      <c r="R76" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S76" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R76" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S76" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T76" s="4" t="inlineStr">
+      <c r="T76" s="4" t="n"/>
+      <c r="U76" s="4" t="inlineStr">
         <is>
           <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
         </is>
       </c>
-      <c r="U76" s="4" t="n"/>
       <c r="V76" s="4" t="inlineStr">
         <is>
           <t>CM</t>
@@ -4750,7 +4750,11 @@
         </is>
       </c>
       <c r="F77" s="4" t="n"/>
-      <c r="G77" s="4" t="n"/>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>is about contact events or is about duration of contact events?</t>
+        </is>
+      </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
           <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
@@ -4772,31 +4776,27 @@
       <c r="N77" s="4" t="n"/>
       <c r="O77" s="4" t="inlineStr">
         <is>
-          <t>is about contact events or is about duration of contact events?</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="P77" s="4" t="n"/>
-      <c r="Q77" s="4" t="inlineStr">
+      <c r="Q77" s="4" t="n"/>
+      <c r="R77" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S77" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R77" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S77" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T77" s="4" t="inlineStr">
+      <c r="T77" s="4" t="n"/>
+      <c r="U77" s="4" t="inlineStr">
         <is>
           <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
-      <c r="U77" s="4" t="n"/>
       <c r="V77" s="4" t="inlineStr">
         <is>
           <t>CM</t>
@@ -4826,7 +4826,11 @@
         </is>
       </c>
       <c r="F78" s="4" t="n"/>
-      <c r="G78" s="4" t="n"/>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>is about contact events or is about duration of contact events?</t>
+        </is>
+      </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
           <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
@@ -4848,31 +4852,27 @@
       <c r="N78" s="4" t="n"/>
       <c r="O78" s="4" t="inlineStr">
         <is>
-          <t>is about contact events or is about duration of contact events?</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="P78" s="4" t="n"/>
-      <c r="Q78" s="4" t="inlineStr">
+      <c r="Q78" s="4" t="n"/>
+      <c r="R78" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S78" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R78" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S78" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T78" s="4" t="inlineStr">
+      <c r="T78" s="4" t="n"/>
+      <c r="U78" s="4" t="inlineStr">
         <is>
           <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
         </is>
       </c>
-      <c r="U78" s="4" t="n"/>
       <c r="V78" s="4" t="inlineStr">
         <is>
           <t>CM</t>
@@ -4918,29 +4918,29 @@
       </c>
       <c r="M79" s="4" t="n"/>
       <c r="N79" s="4" t="n"/>
-      <c r="O79" s="4" t="n"/>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P79" s="4" t="n"/>
-      <c r="Q79" s="4" t="inlineStr">
+      <c r="Q79" s="4" t="n"/>
+      <c r="R79" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S79" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R79" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S79" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T79" s="4" t="inlineStr">
+      <c r="T79" s="4" t="n"/>
+      <c r="U79" s="4" t="inlineStr">
         <is>
           <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
         </is>
       </c>
-      <c r="U79" s="4" t="n"/>
       <c r="V79" s="4" t="inlineStr">
         <is>
           <t>CM</t>
@@ -4962,7 +4962,11 @@
       <c r="D80" s="4" t="n"/>
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="n"/>
-      <c r="G80" s="4" t="n"/>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+        </is>
+      </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
           <t>This is not annotated but included due to relationship with duration of interval</t>
@@ -4976,19 +4980,15 @@
       <c r="N80" s="4" t="n"/>
       <c r="O80" s="4" t="inlineStr">
         <is>
-          <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="P80" s="4" t="n"/>
-      <c r="Q80" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q80" s="4" t="n"/>
       <c r="R80" s="4" t="n"/>
       <c r="S80" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="T80" s="4" t="n"/>
@@ -5044,29 +5044,29 @@
       </c>
       <c r="M81" s="4" t="n"/>
       <c r="N81" s="4" t="n"/>
-      <c r="O81" s="4" t="n"/>
+      <c r="O81" s="4" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="P81" s="4" t="n"/>
-      <c r="Q81" s="4" t="inlineStr">
+      <c r="Q81" s="4" t="n"/>
+      <c r="R81" s="4" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S81" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="R81" s="4" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S81" s="4" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T81" s="4" t="inlineStr">
+      <c r="T81" s="4" t="n"/>
+      <c r="U81" s="4" t="inlineStr">
         <is>
           <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
         </is>
       </c>
-      <c r="U81" s="4" t="n"/>
       <c r="V81" s="4" t="inlineStr">
         <is>
           <t>CM</t>

</xml_diff>

<commit_message>
Update 2 terms in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -457,14 +457,14 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Informal Definition</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Parent</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Elaboration</t>
@@ -472,24 +472,24 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Annotation rules</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'part of'</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Curator note</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Annotation rules</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Examples</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'part of'</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>REL 'has attribute' [RO:0000053]</t>
@@ -512,27 +512,27 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Definition_Source</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Aggregate</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>To be reviewed by</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Definition_Source</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Aggregate</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
@@ -567,24 +567,24 @@
           <t xml:space="preserve">An &lt;intervention contact event&gt; that is an occasion in which a member of a BCI population comes into contact with a BCI.  </t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>intervention contact event</t>
         </is>
       </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>All contact events are temporal parts, but not all temporal parts are contact events. Whilst contact events are single continuous events, temporal parts of an intervention can  group together multiple different contact events which might have similar features. For example, a set of 10 counselling sessions might be a temporal part within an intervention. The same intervention can have a set of 5 exercise sessions. These 5 sessions together make up another temporal part. Each single session within these parts  is a contact event.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>A counselling session; An online chat session; An advertisement display.</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>A counselling session; An online chat session; An advertisement display.</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
@@ -594,15 +594,15 @@
           <t>BCI contact event duration</t>
         </is>
       </c>
-      <c r="O2" s="2" t="n"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="inlineStr">
@@ -627,34 +627,34 @@
           <t>An &lt;intervention contact event duration&gt; between the start and end of a BCI contact event.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>intervention contact event duration</t>
         </is>
       </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>1 hour; 30 minutes; 2 minutes</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>1 hour; 30 minutes; 2 minutes</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="n"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S3" s="2" t="n"/>
       <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="n"/>
       <c r="V3" s="2" t="inlineStr">
@@ -681,27 +681,27 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>intervention contact event frequency</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>How often intervention sessions or digital contacts are planned to occur</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event frequency</t>
-        </is>
-      </c>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>twice a week; daily; one a week</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture descriptions of the frequency of contact events within a part.  
 Example annotation (in context): intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks" </t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>twice a week; daily; one a week</t>
-        </is>
-      </c>
+      <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="inlineStr">
@@ -711,15 +711,15 @@
       </c>
       <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="n"/>
-      <c r="O4" s="2" t="n"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P4" s="2" t="n"/>
       <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S4" s="2" t="n"/>
       <c r="T4" s="2" t="n"/>
       <c r="U4" s="2" t="n"/>
       <c r="V4" s="2" t="inlineStr">
@@ -746,16 +746,20 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>intervention duration</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>The planned duration of an intervention</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>intervention duration</t>
-        </is>
-      </c>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>6 weeks; 2 months; 1 year</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>This is used to capture the overall duration of intervention delivery from first to last contact of an intervention. It does not include follow-up periods during which no content is delivered. We annotate only the number and the unit is derived from the context. 
@@ -763,11 +767,7 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>6 weeks; 2 months; 1 year</t>
-        </is>
-      </c>
+      <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
@@ -775,7 +775,7 @@
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P5" s="2" t="n"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T5" s="2" t="n"/>
@@ -814,12 +814,12 @@
           <t xml:space="preserve">A &lt;BCI attribute&gt; that is its temporal organisation </t>
         </is>
       </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">BCI attribute </t>
         </is>
       </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Includes the start and end of a BCI, its parts, and their organisation around relevant timepoints.</t>
@@ -837,15 +837,15 @@
         </is>
       </c>
       <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P6" s="2" t="n"/>
       <c r="Q6" s="2" t="n"/>
       <c r="R6" s="2" t="n"/>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S6" s="2" t="n"/>
       <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="n"/>
       <c r="V6" s="2" t="inlineStr">
@@ -857,143 +857,134 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008505</t>
+          <t>BCIO:008565</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part</t>
+          <t>BCI temporal part duration</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>A &lt;planned process&gt; that is a part of a BCI.</t>
+          <t>An &lt;intervention temporal part duration&gt; between the start and end of a behaviour change intervention temporal part.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>A planned part of an intervention</t>
+          <t>intervention temporal part duration</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Temporal parts are defined by the authors of reports. They usually group contact events with similar delivery (e.g. face-to-face), content (e.g. CBT), or contextual features (e.g. school lessons), in order to describe their schedule. </t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n"/>
+          <t>The planned duration of a part of an intervention</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>6 weeks; 2 weeks</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Interventions can be broken down into any number of parts, however, we only annotate this entity when the author has named a part AND used it to describe an aspect of the intervention schedule (e.g. given it a duration, defined the frequency of contact events within it, or an interval relative to a timepoint/another part).
-Example Annotations (in context):
-The "counselling sessions" took place each week for 6 weeks, and lasted roughly one hour; During the "first 6 weeks", participants received a phone call every two weeks, then for the "last 4 weeks", this was reduced to a weekly call;</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>counselling sessions; the first 6 weeks of the intervention; group discussion; a presentation; the last 4 weeks of the intervention</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>behaviour change intervention</t>
-        </is>
-      </c>
+          <t xml:space="preserve">This is used to capture the overall duration of parts. We annotate only the number and the unit is derived from the context 
+Example annotation (in context): The counselling sessions ran over a "6" week period, whilst the exercise classes took place over "2" weeks 
+This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>BCI temporal part duration</t>
-        </is>
-      </c>
+      <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P7" s="2" t="n"/>
       <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="n"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="n"/>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>CM; EJH; PS</t>
+          <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008565</t>
+          <t>BCIO:008710</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part duration</t>
+          <t>BCI temporal part frequency</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part duration&gt; between the start and end of a behaviour change intervention temporal part.</t>
+          <t>An &lt;intervention temporal part frequency&gt; that is how often intervention temporal parts occur within a BCI.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>The planned duration of a part of an intervention</t>
+          <t>intervention temporal part frequency</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal part duration</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
+          <t>How often intervention parts are planned to occur</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is useful when grouping contact events together to the schedule of an intervention. For example, authors may describe participants as taking part in 90 minutes of physical activity weekly. These 90 minutes could be split across several contact events, however together these contact events form an intervention part which occurs weekly. </t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Participants took part in 90 minutes of PA "weekly"</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is used to capture the overall duration of parts. We annotate only the number and the unit is derived from the context 
-Example annotation (in context): The counselling sessions ran over a "6" week period, whilst the exercise classes took place over "2" weeks 
-This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>6 weeks; 2 weeks</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Use this entity to annotate descriptions of the frequency of intervention temporal parts  that may be spread over multiple sessions. Usually descriptions refer to the frequency of a single session (e.g. a weekly telephone call) in which case you can annotate using contact event frequency. However, occasionally authors describe frequencies which may take place over multiple contact events. For example, participants may be required to take part in a certain amount of physical activity each week, which can be split over multiple sessions. In this case, annotate using intervention temporal part frequency.  
+Example annotation in context: Participants took part in 90 minutes of PA "weekly" </t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>BCI temporal part</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="n"/>
       <c r="T8" s="2" t="n"/>
       <c r="U8" s="2" t="n"/>
       <c r="V8" s="2" t="inlineStr">
@@ -1005,336 +996,311 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008710</t>
+          <t>BCIO:003000</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal part frequency</t>
+          <t>behaviour change intervention</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part frequency&gt; that is how often intervention temporal parts occur within a BCI.</t>
+          <t>An intervention that has the aim of influencing human behaviour.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>How often intervention parts are planned to occur</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>intervention temporal part frequency</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This is useful when grouping contact events together to the schedule of an intervention. For example, authors may describe participants as taking part in 90 minutes of physical activity weekly. These 90 minutes could be split across several contact events, however together these contact events form an intervention part which occurs weekly. </t>
-        </is>
-      </c>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Use this entity to annotate descriptions of the frequency of intervention temporal parts  that may be spread over multiple sessions. Usually descriptions refer to the frequency of a single session (e.g. a weekly telephone call) in which case you can annotate using contact event frequency. However, occasionally authors describe frequencies which may take place over multiple contact events. For example, participants may be required to take part in a certain amount of physical activity each week, which can be split over multiple sessions. In this case, annotate using intervention temporal part frequency.  
-Example annotation in context: Participants took part in 90 minutes of PA "weekly" </t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Participants took part in 90 minutes of PA "weekly"</t>
-        </is>
-      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>BCI temporal part</t>
-        </is>
-      </c>
+      <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
-      <c r="O9" s="2" t="n"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>BCI duration</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="n"/>
       <c r="R9" s="2" t="n"/>
-      <c r="S9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S9" s="2" t="n"/>
       <c r="T9" s="2" t="n"/>
       <c r="U9" s="2" t="n"/>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="V9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:003000</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>behaviour change intervention</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>An intervention that has the aim of influencing human behaviour.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>intervention</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>BCI duration</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T10" s="2" t="n"/>
-      <c r="U10" s="2" t="n"/>
-      <c r="V10" s="2" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PATO:0000044</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A physical quality which inheres in a bearer by virtue of the number of the bearer's repetitive actions in a particular time.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>JH; PS</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>PATO:0000044</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>frequency</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>A physical quality which inheres in a bearer by virtue of the number of the bearer's repetitive actions in a particular time.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>specifically dependent continuant</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>JH; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>BCIO:008575</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>interval between BCI temporal parts</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>An &lt;interval between intervention temporal parts&gt; between the end of one BCI temporal part and the beginning of a subsequent BCI temporal part.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>interval between intervention temporal parts</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>The planned duration of a break between two parts of an intervention</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>interval between intervention temporal parts</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>"2 weeks"; "1 day"</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture intervals between BCI parts and timepoints. We annotate only the number and the unit is derived from the context 
 Example annotation (in context): Exercise classes started "2 weeks" after the education phase of the intervention. 
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>"2 weeks"; "1 day"</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>BCI temporal part</t>
         </is>
       </c>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="n"/>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="P12" s="2" t="n"/>
-      <c r="Q12" s="2" t="n"/>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T12" s="2" t="n"/>
-      <c r="U12" s="2" t="n"/>
-      <c r="V12" s="2" t="inlineStr">
+      <c r="T11" s="2" t="n"/>
+      <c r="U11" s="2" t="n"/>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051017</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>interval between intervention temporal parts</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the end of one intervention temporal part and the beginning of a subsequent intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
+      <c r="N12" s="3" t="n"/>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="n"/>
+      <c r="Q12" s="3" t="n"/>
+      <c r="R12" s="3" t="n"/>
+      <c r="S12" s="3" t="n"/>
+      <c r="T12" s="3" t="n"/>
+      <c r="U12" s="3" t="n"/>
+      <c r="V12" s="3" t="n"/>
+    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051017</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>interval between intervention temporal parts</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; between the end of one intervention temporal part and the beginning of a subsequent intervention temporal part.</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3" t="n"/>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:051010</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2" t="n"/>
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="2" t="n"/>
+      <c r="T13" s="2" t="n"/>
+      <c r="U13" s="2" t="n"/>
+      <c r="V13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051009</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
+      <c r="N14" s="3" t="n"/>
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="T13" s="3" t="n"/>
-      <c r="U13" s="3" t="n"/>
-      <c r="V13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:051010</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>intervention attribute</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="n"/>
-      <c r="Q14" s="2" t="n"/>
-      <c r="R14" s="2" t="n"/>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T14" s="2" t="n"/>
-      <c r="U14" s="2" t="n"/>
-      <c r="V14" s="2" t="n"/>
+      <c r="P14" s="3" t="n"/>
+      <c r="Q14" s="3" t="n"/>
+      <c r="R14" s="3" t="n"/>
+      <c r="S14" s="3" t="n"/>
+      <c r="T14" s="3" t="n"/>
+      <c r="U14" s="3" t="n"/>
+      <c r="V14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>BCIO:051009</t>
+          <t>BCIO:051018</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>intervention contact event</t>
+          <t>intervention contact event duration</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>intervention temporal part</t>
-        </is>
-      </c>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
@@ -1344,185 +1310,197 @@
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
       <c r="N15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n"/>
       <c r="R15" s="3" t="n"/>
-      <c r="S15" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S15" s="3" t="n"/>
       <c r="T15" s="3" t="n"/>
       <c r="U15" s="3" t="n"/>
       <c r="V15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051018</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>intervention contact event duration</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="3" t="n"/>
-      <c r="Q16" s="3" t="n"/>
-      <c r="R16" s="3" t="n"/>
-      <c r="S16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050505</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>intervention contact event duration statistic</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event durations.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event duration</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="2" t="n"/>
+      <c r="R16" s="2" t="n"/>
+      <c r="S16" s="2" t="n"/>
+      <c r="T16" s="2" t="n"/>
+      <c r="U16" s="2" t="n"/>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051001</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event frequency</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="T16" s="3" t="n"/>
-      <c r="U16" s="3" t="n"/>
-      <c r="V16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050505</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event duration statistic</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event durations.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="P17" s="3" t="n"/>
+      <c r="Q17" s="3" t="n"/>
+      <c r="R17" s="3" t="n"/>
+      <c r="S17" s="3" t="n"/>
+      <c r="T17" s="3" t="n"/>
+      <c r="U17" s="3" t="n"/>
+      <c r="V17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050903</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>intervention contact event frequency statistic</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event duration</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="n"/>
-      <c r="Q17" s="2" t="n"/>
-      <c r="R17" s="2" t="n"/>
-      <c r="S17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T17" s="2" t="n"/>
-      <c r="U17" s="2" t="n"/>
-      <c r="V17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event frequency</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="n"/>
+      <c r="Q18" s="2" t="n"/>
+      <c r="R18" s="2" t="n"/>
+      <c r="S18" s="2" t="n"/>
+      <c r="T18" s="2" t="n"/>
+      <c r="U18" s="2" t="n"/>
+      <c r="V18" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051001</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>intervention contact event frequency</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
-      <c r="O18" s="3" t="n"/>
-      <c r="P18" s="3" t="n"/>
-      <c r="Q18" s="3" t="n"/>
-      <c r="R18" s="3" t="n"/>
-      <c r="S18" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T18" s="3" t="n"/>
-      <c r="U18" s="3" t="n"/>
-      <c r="V18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050903</t>
+          <t>BCIO:050904</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="inlineStr">
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -1535,20 +1513,20 @@
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="n"/>
-      <c r="O19" s="2" t="n"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P19" s="2" t="n"/>
       <c r="Q19" s="2" t="n"/>
       <c r="R19" s="2" t="n"/>
-      <c r="S19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S19" s="2" t="n"/>
       <c r="T19" s="2" t="n"/>
       <c r="U19" s="2" t="n"/>
       <c r="V19" s="2" t="inlineStr">
@@ -1558,248 +1536,271 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050904</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event number statistic</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051002</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>intervention duration</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="3" t="n"/>
+      <c r="N20" s="3" t="n"/>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="n"/>
+      <c r="Q20" s="3" t="n"/>
+      <c r="R20" s="3" t="n"/>
+      <c r="S20" s="3" t="n"/>
+      <c r="T20" s="3" t="n"/>
+      <c r="U20" s="3" t="n"/>
+      <c r="V20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050905</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>intervention duration statistic</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>number of BCI contact events</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="n"/>
-      <c r="S20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T20" s="2" t="n"/>
-      <c r="U20" s="2" t="n"/>
-      <c r="V20" s="2" t="inlineStr">
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>BCI duration</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2" t="n"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n"/>
+      <c r="Q21" s="2" t="n"/>
+      <c r="R21" s="2" t="n"/>
+      <c r="S21" s="2" t="n"/>
+      <c r="T21" s="2" t="n"/>
+      <c r="U21" s="2" t="n"/>
+      <c r="V21" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051002</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>intervention duration</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
-      <c r="P21" s="3" t="n"/>
-      <c r="Q21" s="3" t="n"/>
-      <c r="R21" s="3" t="n"/>
-      <c r="S21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051011</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>An &lt;intervention attribute&gt; that is its temporal organisation.</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3" t="n"/>
+      <c r="N22" s="3" t="n"/>
+      <c r="O22" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="T21" s="3" t="n"/>
-      <c r="U21" s="3" t="n"/>
-      <c r="V21" s="3" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050905</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>intervention duration statistic</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="n"/>
-      <c r="K22" s="2" t="n"/>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>BCI duration</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n"/>
-      <c r="N22" s="2" t="n"/>
-      <c r="O22" s="2" t="n"/>
-      <c r="P22" s="2" t="n"/>
-      <c r="Q22" s="2" t="n"/>
-      <c r="R22" s="2" t="n"/>
-      <c r="S22" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T22" s="2" t="n"/>
-      <c r="U22" s="2" t="n"/>
-      <c r="V22" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="P22" s="3" t="n"/>
+      <c r="Q22" s="3" t="n"/>
+      <c r="R22" s="3" t="n"/>
+      <c r="S22" s="3" t="n"/>
+      <c r="T22" s="3" t="n"/>
+      <c r="U22" s="3" t="n"/>
+      <c r="V22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051011</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>intervention schedule of delivery</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>An &lt;intervention attribute&gt; that is its temporal organisation.</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>intervention attribute</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
-      <c r="O23" s="3" t="n"/>
-      <c r="P23" s="3" t="n"/>
-      <c r="Q23" s="3" t="n"/>
-      <c r="R23" s="3" t="n"/>
-      <c r="S23" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T23" s="3" t="n"/>
-      <c r="U23" s="3" t="n"/>
-      <c r="V23" s="3" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008505</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>intervention temporal part</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;planned process&gt; that is a part of an intervention.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>A planned part of an intervention</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Temporal parts are defined by the authors of reports. They usually group contact events with similar delivery (e.g. face-to-face), content (e.g. CBT), or contextual features (e.g. school lessons), in order to describe their schedule. 
+This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>counselling sessions; the first 6 weeks of the intervention; group discussion; a presentation; the last 4 weeks of the intervention</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Interventions can be broken down into any number of parts, however, we only annotate this entity when the author has named a part AND used it to describe an aspect of the intervention schedule (e.g. given it a duration, defined the frequency of contact events within it, or an interval relative to a timepoint/another part).
+Example Annotations (in context):
+The "counselling sessions" took place each week for 6 weeks, and lasted roughly one hour; During the "first 6 weeks", participants received a phone call every two weeks, then for the "last 4 weeks", this was reduced to a weekly call;</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>behaviour change intervention</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>BCI temporal part duration</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="n"/>
+      <c r="Q23" s="2" t="n"/>
+      <c r="R23" s="2" t="n"/>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="n"/>
+      <c r="U23" s="2" t="n"/>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>CM; EJH; PS</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>BCIO:051008</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>intervention temporal part</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>A &lt;planned process&gt; that is a part of an intervention.</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="n"/>
-      <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="n"/>
-      <c r="Q24" s="2" t="n"/>
-      <c r="R24" s="2" t="n"/>
-      <c r="S24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T24" s="2" t="n"/>
-      <c r="U24" s="2" t="n"/>
-      <c r="V24" s="2" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
+      <c r="M24" s="4" t="n"/>
+      <c r="N24" s="4" t="n"/>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="n"/>
+      <c r="Q24" s="4" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="n"/>
+      <c r="T24" s="4" t="n"/>
+      <c r="U24" s="4" t="n"/>
+      <c r="V24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1817,12 +1818,12 @@
           <t>A &lt;temporal interval&gt; between the start and end of an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
+      <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
@@ -1832,15 +1833,15 @@
       <c r="L25" s="3" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
-      <c r="O25" s="3" t="n"/>
-      <c r="P25" s="3" t="n"/>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr"/>
       <c r="Q25" s="3" t="n"/>
       <c r="R25" s="3" t="n"/>
-      <c r="S25" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S25" s="3" t="n"/>
       <c r="T25" s="3" t="n"/>
       <c r="U25" s="3" t="n"/>
       <c r="V25" s="3" t="n"/>
@@ -1861,12 +1862,12 @@
           <t>A &lt;data item&gt; that is about a collection of intervention temporal part durations.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -1884,15 +1885,15 @@
       </c>
       <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="n"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
-      <c r="S26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S26" s="2" t="n"/>
       <c r="T26" s="2" t="n"/>
       <c r="U26" s="2" t="n"/>
       <c r="V26" s="2" t="inlineStr">
@@ -1917,12 +1918,12 @@
           <t>A &lt;data item&gt; that is how often intervention temporal parts occur within an intervention.</t>
         </is>
       </c>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">This is useful when grouping contact events together to the schedule of an intervention. For example, authors may describe participants as taking part in 90 minutes of physical activity weekly. These 90 minutes could be split across several contact events, however together these contact events form an intervention part which occurs weekly. </t>
@@ -1936,15 +1937,15 @@
       <c r="L27" s="3" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n"/>
       <c r="R27" s="3" t="n"/>
-      <c r="S27" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S27" s="3" t="n"/>
       <c r="T27" s="3" t="n"/>
       <c r="U27" s="3" t="n"/>
       <c r="V27" s="3" t="n"/>
@@ -1965,12 +1966,12 @@
           <t>A &lt;data item&gt; that is about a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -1988,15 +1989,15 @@
       </c>
       <c r="M28" s="2" t="n"/>
       <c r="N28" s="2" t="n"/>
-      <c r="O28" s="2" t="n"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P28" s="2" t="n"/>
       <c r="Q28" s="2" t="n"/>
       <c r="R28" s="2" t="n"/>
-      <c r="S28" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S28" s="2" t="n"/>
       <c r="T28" s="2" t="n"/>
       <c r="U28" s="2" t="n"/>
       <c r="V28" s="2" t="inlineStr">
@@ -2023,27 +2024,27 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
+          <t>irregular intervention schedule</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>irregular intervention schedule</t>
-        </is>
-      </c>
       <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
 Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks" </t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
-        </is>
-      </c>
+      <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="n"/>
@@ -2051,7 +2052,7 @@
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P29" s="2" t="n"/>
@@ -2059,7 +2060,7 @@
       <c r="R29" s="2" t="n"/>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T29" s="2" t="n"/>
@@ -2092,41 +2093,41 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>intervention schedule of delivery</t>
-        </is>
-      </c>
       <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
+        </is>
+      </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
 Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks"  </t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
-        </is>
-      </c>
+      <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="3" t="n"/>
       <c r="L30" s="3" t="n"/>
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3" t="n"/>
-      <c r="O30" s="3" t="n"/>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P30" s="3" t="n"/>
       <c r="Q30" s="3" t="n"/>
       <c r="R30" s="3" t="n"/>
-      <c r="S30" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S30" s="3" t="n"/>
       <c r="T30" s="3" t="n"/>
       <c r="U30" s="3" t="n"/>
       <c r="V30" s="3" t="n"/>
@@ -2147,12 +2148,12 @@
           <t>An &lt;intervention contact event duration statistic&gt; that is the highest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2170,15 +2171,15 @@
       </c>
       <c r="M31" s="2" t="n"/>
       <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P31" s="2" t="n"/>
       <c r="Q31" s="2" t="n"/>
       <c r="R31" s="2" t="n"/>
-      <c r="S31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S31" s="2" t="n"/>
       <c r="T31" s="2" t="n"/>
       <c r="U31" s="2" t="n"/>
       <c r="V31" s="2" t="inlineStr">
@@ -2203,12 +2204,12 @@
           <t>An &lt;intervention contact event frequency statistic&gt; that is the highest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>intervention contact event frequency statistic</t>
         </is>
       </c>
+      <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2226,15 +2227,15 @@
       </c>
       <c r="M32" s="2" t="n"/>
       <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="n"/>
       <c r="R32" s="2" t="n"/>
-      <c r="S32" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S32" s="2" t="n"/>
       <c r="T32" s="2" t="n"/>
       <c r="U32" s="2" t="n"/>
       <c r="V32" s="2" t="inlineStr">
@@ -2259,12 +2260,12 @@
           <t>An &lt;intervention contact event number statistic&gt; that is the highest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>intervention contact event number statistic</t>
         </is>
       </c>
+      <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2282,15 +2283,15 @@
       </c>
       <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P33" s="2" t="n"/>
       <c r="Q33" s="2" t="n"/>
       <c r="R33" s="2" t="n"/>
-      <c r="S33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S33" s="2" t="n"/>
       <c r="T33" s="2" t="n"/>
       <c r="U33" s="2" t="n"/>
       <c r="V33" s="2" t="inlineStr">
@@ -2315,12 +2316,12 @@
           <t>An &lt;intervention duration statistic&gt; that is the highest value from a collection of intervention durations.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>intervention duration statistic</t>
         </is>
       </c>
+      <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2338,15 +2339,15 @@
       </c>
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P34" s="2" t="n"/>
       <c r="Q34" s="2" t="n"/>
       <c r="R34" s="2" t="n"/>
-      <c r="S34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S34" s="2" t="n"/>
       <c r="T34" s="2" t="n"/>
       <c r="U34" s="2" t="n"/>
       <c r="V34" s="2" t="inlineStr">
@@ -2371,12 +2372,12 @@
           <t>An &lt;intervention temporal part duration statistic&gt; that denotes the highest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part duration statistic</t>
         </is>
       </c>
+      <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2394,15 +2395,15 @@
       </c>
       <c r="M35" s="2" t="n"/>
       <c r="N35" s="2" t="n"/>
-      <c r="O35" s="2" t="n"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P35" s="2" t="n"/>
       <c r="Q35" s="2" t="n"/>
       <c r="R35" s="2" t="n"/>
-      <c r="S35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S35" s="2" t="n"/>
       <c r="T35" s="2" t="n"/>
       <c r="U35" s="2" t="n"/>
       <c r="V35" s="2" t="inlineStr">
@@ -2427,12 +2428,12 @@
           <t>An &lt;intervention temporal part frequency statistic&gt; that is the highest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
+      <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2450,15 +2451,15 @@
       </c>
       <c r="M36" s="2" t="n"/>
       <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P36" s="2" t="n"/>
       <c r="Q36" s="2" t="n"/>
       <c r="R36" s="2" t="n"/>
-      <c r="S36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S36" s="2" t="n"/>
       <c r="T36" s="2" t="n"/>
       <c r="U36" s="2" t="n"/>
       <c r="V36" s="2" t="inlineStr">
@@ -2483,12 +2484,12 @@
           <t>A &lt;total intervention contact event duration statistic&gt; that is the highest value from a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2506,15 +2507,15 @@
       </c>
       <c r="M37" s="2" t="n"/>
       <c r="N37" s="2" t="n"/>
-      <c r="O37" s="2" t="n"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P37" s="2" t="n"/>
       <c r="Q37" s="2" t="n"/>
       <c r="R37" s="2" t="n"/>
-      <c r="S37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S37" s="2" t="n"/>
       <c r="T37" s="2" t="n"/>
       <c r="U37" s="2" t="n"/>
       <c r="V37" s="2" t="inlineStr">
@@ -2539,12 +2540,12 @@
           <t>An &lt;intervention contact event duration statistic&gt; that is the average value calculated from a collection of intervention contact event durations.</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2562,15 +2563,15 @@
       </c>
       <c r="M38" s="2" t="n"/>
       <c r="N38" s="2" t="n"/>
-      <c r="O38" s="2" t="n"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P38" s="2" t="n"/>
       <c r="Q38" s="2" t="n"/>
       <c r="R38" s="2" t="n"/>
-      <c r="S38" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S38" s="2" t="n"/>
       <c r="T38" s="2" t="n"/>
       <c r="U38" s="2" t="n"/>
       <c r="V38" s="2" t="inlineStr">
@@ -2595,12 +2596,12 @@
           <t>An &lt;intervention contact event frequency statistic&gt; that is the average value calculated from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>intervention contact event frequency statistic</t>
         </is>
       </c>
+      <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2618,15 +2619,15 @@
       </c>
       <c r="M39" s="2" t="n"/>
       <c r="N39" s="2" t="n"/>
-      <c r="O39" s="2" t="n"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P39" s="2" t="n"/>
       <c r="Q39" s="2" t="n"/>
       <c r="R39" s="2" t="n"/>
-      <c r="S39" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S39" s="2" t="n"/>
       <c r="T39" s="2" t="n"/>
       <c r="U39" s="2" t="n"/>
       <c r="V39" s="2" t="inlineStr">
@@ -2651,12 +2652,12 @@
           <t>An &lt;intervention contact event number statistic&gt; that is the average value calculated from a collection of intervention contact event numbers.</t>
         </is>
       </c>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>intervention contact event number statistic</t>
         </is>
       </c>
+      <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2674,15 +2675,15 @@
       </c>
       <c r="M40" s="2" t="n"/>
       <c r="N40" s="2" t="n"/>
-      <c r="O40" s="2" t="n"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P40" s="2" t="n"/>
       <c r="Q40" s="2" t="n"/>
       <c r="R40" s="2" t="n"/>
-      <c r="S40" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S40" s="2" t="n"/>
       <c r="T40" s="2" t="n"/>
       <c r="U40" s="2" t="n"/>
       <c r="V40" s="2" t="inlineStr">
@@ -2707,12 +2708,12 @@
           <t>An &lt;intervention duration statistic&gt; that is the average value calculated from a collection of intervention durations.</t>
         </is>
       </c>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>intervention duration statistic</t>
         </is>
       </c>
+      <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2730,15 +2731,15 @@
       </c>
       <c r="M41" s="2" t="n"/>
       <c r="N41" s="2" t="n"/>
-      <c r="O41" s="2" t="n"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P41" s="2" t="n"/>
       <c r="Q41" s="2" t="n"/>
       <c r="R41" s="2" t="n"/>
-      <c r="S41" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S41" s="2" t="n"/>
       <c r="T41" s="2" t="n"/>
       <c r="U41" s="2" t="n"/>
       <c r="V41" s="2" t="inlineStr">
@@ -2763,12 +2764,12 @@
           <t>An &lt;intervention temporal part duration statistic&gt; that is the average value calculated from a collection of intervention temporal part durations.</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part duration statistic</t>
         </is>
       </c>
+      <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2786,15 +2787,15 @@
       </c>
       <c r="M42" s="2" t="n"/>
       <c r="N42" s="2" t="n"/>
-      <c r="O42" s="2" t="n"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P42" s="2" t="n"/>
       <c r="Q42" s="2" t="n"/>
       <c r="R42" s="2" t="n"/>
-      <c r="S42" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S42" s="2" t="n"/>
       <c r="T42" s="2" t="n"/>
       <c r="U42" s="2" t="n"/>
       <c r="V42" s="2" t="inlineStr">
@@ -2819,12 +2820,12 @@
           <t>An &lt;intervention temporal part frequency statistic&gt; that is the average value calculated from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
+      <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2842,15 +2843,15 @@
       </c>
       <c r="M43" s="2" t="n"/>
       <c r="N43" s="2" t="n"/>
-      <c r="O43" s="2" t="n"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P43" s="2" t="n"/>
       <c r="Q43" s="2" t="n"/>
       <c r="R43" s="2" t="n"/>
-      <c r="S43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S43" s="2" t="n"/>
       <c r="T43" s="2" t="n"/>
       <c r="U43" s="2" t="n"/>
       <c r="V43" s="2" t="inlineStr">
@@ -2875,12 +2876,12 @@
           <t>A &lt;total intervention contact event duration statistic&gt; that is the average value calculated from a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2898,15 +2899,15 @@
       </c>
       <c r="M44" s="2" t="n"/>
       <c r="N44" s="2" t="n"/>
-      <c r="O44" s="2" t="n"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P44" s="2" t="n"/>
       <c r="Q44" s="2" t="n"/>
       <c r="R44" s="2" t="n"/>
-      <c r="S44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S44" s="2" t="n"/>
       <c r="T44" s="2" t="n"/>
       <c r="U44" s="2" t="n"/>
       <c r="V44" s="2" t="inlineStr">
@@ -2931,12 +2932,12 @@
           <t>An &lt;intervention contact event duration statistic&gt; that is the central value of a collection of intervention contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -2954,15 +2955,15 @@
       </c>
       <c r="M45" s="2" t="n"/>
       <c r="N45" s="2" t="n"/>
-      <c r="O45" s="2" t="n"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P45" s="2" t="n"/>
       <c r="Q45" s="2" t="n"/>
       <c r="R45" s="2" t="n"/>
-      <c r="S45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S45" s="2" t="n"/>
       <c r="T45" s="2" t="n"/>
       <c r="U45" s="2" t="n"/>
       <c r="V45" s="2" t="inlineStr">
@@ -2987,12 +2988,12 @@
           <t>An &lt;intervention contact event frequency statistic&gt; that is the central value of a collection of  intervention contact event frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>intervention contact event frequency statistic</t>
         </is>
       </c>
+      <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3010,15 +3011,15 @@
       </c>
       <c r="M46" s="2" t="n"/>
       <c r="N46" s="2" t="n"/>
-      <c r="O46" s="2" t="n"/>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P46" s="2" t="n"/>
       <c r="Q46" s="2" t="n"/>
       <c r="R46" s="2" t="n"/>
-      <c r="S46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S46" s="2" t="n"/>
       <c r="T46" s="2" t="n"/>
       <c r="U46" s="2" t="n"/>
       <c r="V46" s="2" t="inlineStr">
@@ -3043,12 +3044,12 @@
           <t>An &lt;intervention contact event number statistic&gt; that is the central value of a collection of  intervention contact event numbers when they are arranged in ascending order.</t>
         </is>
       </c>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>intervention contact event number statistic</t>
         </is>
       </c>
+      <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3066,15 +3067,15 @@
       </c>
       <c r="M47" s="2" t="n"/>
       <c r="N47" s="2" t="n"/>
-      <c r="O47" s="2" t="n"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P47" s="2" t="n"/>
       <c r="Q47" s="2" t="n"/>
       <c r="R47" s="2" t="n"/>
-      <c r="S47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S47" s="2" t="n"/>
       <c r="T47" s="2" t="n"/>
       <c r="U47" s="2" t="n"/>
       <c r="V47" s="2" t="inlineStr">
@@ -3099,12 +3100,12 @@
           <t>An &lt;intervention duration statistic&gt; that is the central value of a collection of intervention durations when they are arranged in ascending order.</t>
         </is>
       </c>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>intervention duration statistic</t>
         </is>
       </c>
+      <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3122,15 +3123,15 @@
       </c>
       <c r="M48" s="2" t="n"/>
       <c r="N48" s="2" t="n"/>
-      <c r="O48" s="2" t="n"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P48" s="2" t="n"/>
       <c r="Q48" s="2" t="n"/>
       <c r="R48" s="2" t="n"/>
-      <c r="S48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S48" s="2" t="n"/>
       <c r="T48" s="2" t="n"/>
       <c r="U48" s="2" t="n"/>
       <c r="V48" s="2" t="inlineStr">
@@ -3155,12 +3156,12 @@
           <t>An &lt;intervention temporal part duration statistic&gt; that is the central value of a collection of intervention temporal part durations when they are arranged in ascending order.</t>
         </is>
       </c>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part duration statistic</t>
         </is>
       </c>
+      <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3178,15 +3179,15 @@
       </c>
       <c r="M49" s="2" t="n"/>
       <c r="N49" s="2" t="n"/>
-      <c r="O49" s="2" t="n"/>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P49" s="2" t="n"/>
       <c r="Q49" s="2" t="n"/>
       <c r="R49" s="2" t="n"/>
-      <c r="S49" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S49" s="2" t="n"/>
       <c r="T49" s="2" t="n"/>
       <c r="U49" s="2" t="n"/>
       <c r="V49" s="2" t="inlineStr">
@@ -3211,12 +3212,12 @@
           <t>An &lt;intervention temporal part frequency statistic&gt; that is the central value of a collection of intervention temporal part frequencies when they are arranged in ascending order.</t>
         </is>
       </c>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
+      <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3234,15 +3235,15 @@
       </c>
       <c r="M50" s="2" t="n"/>
       <c r="N50" s="2" t="n"/>
-      <c r="O50" s="2" t="n"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P50" s="2" t="n"/>
       <c r="Q50" s="2" t="n"/>
       <c r="R50" s="2" t="n"/>
-      <c r="S50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S50" s="2" t="n"/>
       <c r="T50" s="2" t="n"/>
       <c r="U50" s="2" t="n"/>
       <c r="V50" s="2" t="inlineStr">
@@ -3267,12 +3268,12 @@
           <t>A &lt;total intervention contact event duration statistic&gt; that is the central value of a collection of total contact event durations when they are arranged in ascending order.</t>
         </is>
       </c>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3290,15 +3291,15 @@
       </c>
       <c r="M51" s="2" t="n"/>
       <c r="N51" s="2" t="n"/>
-      <c r="O51" s="2" t="n"/>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P51" s="2" t="n"/>
       <c r="Q51" s="2" t="n"/>
       <c r="R51" s="2" t="n"/>
-      <c r="S51" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S51" s="2" t="n"/>
       <c r="T51" s="2" t="n"/>
       <c r="U51" s="2" t="n"/>
       <c r="V51" s="2" t="inlineStr">
@@ -3323,12 +3324,12 @@
           <t>An &lt;intervention contact event duration statistic&gt; that is the lowest value from a collection of intervention contact event durations.</t>
         </is>
       </c>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3346,15 +3347,15 @@
       </c>
       <c r="M52" s="2" t="n"/>
       <c r="N52" s="2" t="n"/>
-      <c r="O52" s="2" t="n"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P52" s="2" t="n"/>
       <c r="Q52" s="2" t="n"/>
       <c r="R52" s="2" t="n"/>
-      <c r="S52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S52" s="2" t="n"/>
       <c r="T52" s="2" t="n"/>
       <c r="U52" s="2" t="n"/>
       <c r="V52" s="2" t="inlineStr">
@@ -3379,12 +3380,12 @@
           <t>An &lt;intervention contact event frequency statistic&gt; that is the lowest value from a collection of intervention contact event frequencies.</t>
         </is>
       </c>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>intervention contact event frequency statistic</t>
         </is>
       </c>
+      <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3402,15 +3403,15 @@
       </c>
       <c r="M53" s="2" t="n"/>
       <c r="N53" s="2" t="n"/>
-      <c r="O53" s="2" t="n"/>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P53" s="2" t="n"/>
       <c r="Q53" s="2" t="n"/>
       <c r="R53" s="2" t="n"/>
-      <c r="S53" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S53" s="2" t="n"/>
       <c r="T53" s="2" t="n"/>
       <c r="U53" s="2" t="n"/>
       <c r="V53" s="2" t="inlineStr">
@@ -3435,12 +3436,12 @@
           <t>An &lt;intervention contact event number statistic&gt; that is the lowest value from a collection of intervention contact event numbers.</t>
         </is>
       </c>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>intervention contact event number statistic</t>
         </is>
       </c>
+      <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3458,15 +3459,15 @@
       </c>
       <c r="M54" s="2" t="n"/>
       <c r="N54" s="2" t="n"/>
-      <c r="O54" s="2" t="n"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P54" s="2" t="n"/>
       <c r="Q54" s="2" t="n"/>
       <c r="R54" s="2" t="n"/>
-      <c r="S54" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S54" s="2" t="n"/>
       <c r="T54" s="2" t="n"/>
       <c r="U54" s="2" t="n"/>
       <c r="V54" s="2" t="inlineStr">
@@ -3491,12 +3492,12 @@
           <t>An &lt;intervention duration statistic&gt; that is the lowest value from a collection of intervention durations.</t>
         </is>
       </c>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>intervention duration statistic</t>
         </is>
       </c>
+      <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3514,15 +3515,15 @@
       </c>
       <c r="M55" s="2" t="n"/>
       <c r="N55" s="2" t="n"/>
-      <c r="O55" s="2" t="n"/>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P55" s="2" t="n"/>
       <c r="Q55" s="2" t="n"/>
       <c r="R55" s="2" t="n"/>
-      <c r="S55" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S55" s="2" t="n"/>
       <c r="T55" s="2" t="n"/>
       <c r="U55" s="2" t="n"/>
       <c r="V55" s="2" t="inlineStr">
@@ -3547,12 +3548,12 @@
           <t>An &lt;intervention temporal part duration statistic&gt; that denotes the lowest value from a collection of intervention temporal part durations.</t>
         </is>
       </c>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part duration statistic</t>
         </is>
       </c>
+      <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3570,15 +3571,15 @@
       </c>
       <c r="M56" s="2" t="n"/>
       <c r="N56" s="2" t="n"/>
-      <c r="O56" s="2" t="n"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P56" s="2" t="n"/>
       <c r="Q56" s="2" t="n"/>
       <c r="R56" s="2" t="n"/>
-      <c r="S56" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S56" s="2" t="n"/>
       <c r="T56" s="2" t="n"/>
       <c r="U56" s="2" t="n"/>
       <c r="V56" s="2" t="inlineStr">
@@ -3603,12 +3604,12 @@
           <t>An &lt;intervention temporal part frequency statistic&gt; that is the lowest value from a collection of intervention temporal part frequencies.</t>
         </is>
       </c>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>intervention temporal part frequency statistic</t>
         </is>
       </c>
+      <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3626,15 +3627,15 @@
       </c>
       <c r="M57" s="2" t="n"/>
       <c r="N57" s="2" t="n"/>
-      <c r="O57" s="2" t="n"/>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P57" s="2" t="n"/>
       <c r="Q57" s="2" t="n"/>
       <c r="R57" s="2" t="n"/>
-      <c r="S57" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S57" s="2" t="n"/>
       <c r="T57" s="2" t="n"/>
       <c r="U57" s="2" t="n"/>
       <c r="V57" s="2" t="inlineStr">
@@ -3659,12 +3660,12 @@
           <t>A &lt;total intervention contact event duration statistic&gt; that is the lowest value from a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>total intervention contact event duration statistic</t>
         </is>
       </c>
+      <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -3682,15 +3683,15 @@
       </c>
       <c r="M58" s="2" t="n"/>
       <c r="N58" s="2" t="n"/>
-      <c r="O58" s="2" t="n"/>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P58" s="2" t="n"/>
       <c r="Q58" s="2" t="n"/>
       <c r="R58" s="2" t="n"/>
-      <c r="S58" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S58" s="2" t="n"/>
       <c r="T58" s="2" t="n"/>
       <c r="U58" s="2" t="n"/>
       <c r="V58" s="2" t="inlineStr">
@@ -3717,16 +3718,20 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
+          <t>number of intervention contact events</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
           <t>The planned total number of sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>number of intervention contact events</t>
-        </is>
-      </c>
       <c r="F59" s="2" t="n"/>
-      <c r="G59" s="2" t="n"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>one; 6; 12; twenty</t>
+        </is>
+      </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This entity is used to capture the number of contacts in an intervention or part. We annotate only the number and include the sentence as context. When there is only one session in a part, we can annotate non-numerical words to indicate this, e.g. 'participants attended "a" gp visit'. Sometimes authors will break parts down in which case we annotate the number of contact events which add together to create a total e.g. 'at the first "two" sessions participants received counslling and at the final "six" they took part in exercise classes'. 
@@ -3734,11 +3739,7 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
-        <is>
-          <t>one; 6; 12; twenty</t>
-        </is>
-      </c>
+      <c r="I59" s="2" t="n"/>
       <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="inlineStr">
@@ -3750,7 +3751,7 @@
       <c r="N59" s="2" t="n"/>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P59" s="2" t="n"/>
@@ -3762,7 +3763,7 @@
       </c>
       <c r="S59" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T59" s="2" t="n"/>
@@ -3789,12 +3790,12 @@
           <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D60" s="3" t="n"/>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E60" s="3" t="n"/>
       <c r="F60" s="3" t="n"/>
       <c r="G60" s="3" t="n"/>
       <c r="H60" s="3" t="n"/>
@@ -3804,15 +3805,15 @@
       <c r="L60" s="3" t="n"/>
       <c r="M60" s="3" t="n"/>
       <c r="N60" s="3" t="n"/>
-      <c r="O60" s="3" t="n"/>
+      <c r="O60" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n"/>
       <c r="R60" s="3" t="n"/>
-      <c r="S60" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S60" s="3" t="n"/>
       <c r="T60" s="3" t="n"/>
       <c r="U60" s="3" t="n"/>
       <c r="V60" s="3" t="n"/>
@@ -3833,20 +3834,14 @@
           <t>An &lt;order of intervention temporal parts&gt; that is the  temporal positioning of BCI temporal parts.</t>
         </is>
       </c>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>order of intervention temporal parts</t>
         </is>
       </c>
+      <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
-      <c r="G61" s="2" t="n"/>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>This is annotated as an open code when any aspect of order is described</t>
-        </is>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>"After questionnaires were completed, feedback was selected
 out of a database with messages for each possible combination
@@ -3855,6 +3850,12 @@
 levels to the PA guidelines."</t>
         </is>
       </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>This is annotated as an open code when any aspect of order is described</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="n"/>
       <c r="J61" s="2" t="n"/>
       <c r="K61" s="2" t="n"/>
       <c r="L61" s="2" t="n"/>
@@ -3866,7 +3867,7 @@
       <c r="N61" s="2" t="n"/>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P61" s="2" t="n"/>
@@ -3874,7 +3875,7 @@
       <c r="R61" s="2" t="n"/>
       <c r="S61" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T61" s="2" t="n"/>
@@ -3901,12 +3902,12 @@
           <t>An &lt;intervention attribute&gt; that is the  temporal positioning of intervention temporal parts.</t>
         </is>
       </c>
-      <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
+      <c r="E62" s="3" t="n"/>
       <c r="F62" s="3" t="n"/>
       <c r="G62" s="3" t="n"/>
       <c r="H62" s="3" t="n"/>
@@ -3916,15 +3917,15 @@
       <c r="L62" s="3" t="n"/>
       <c r="M62" s="3" t="n"/>
       <c r="N62" s="3" t="n"/>
-      <c r="O62" s="3" t="n"/>
+      <c r="O62" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n"/>
       <c r="R62" s="3" t="n"/>
-      <c r="S62" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S62" s="3" t="n"/>
       <c r="T62" s="3" t="n"/>
       <c r="U62" s="3" t="n"/>
       <c r="V62" s="3" t="n"/>
@@ -3962,7 +3963,7 @@
       <c r="N63" s="4" t="n"/>
       <c r="O63" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P63" s="4" t="n"/>
@@ -3970,7 +3971,7 @@
       <c r="R63" s="4" t="n"/>
       <c r="S63" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T63" s="4" t="n"/>
@@ -4014,7 +4015,7 @@
       <c r="N64" s="4" t="n"/>
       <c r="O64" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P64" s="4" t="n"/>
@@ -4022,7 +4023,7 @@
       <c r="R64" s="4" t="n"/>
       <c r="S64" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T64" s="4" t="n"/>
@@ -4051,27 +4052,27 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
+          <t>regular intervention schedule</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>regular intervention schedule</t>
-        </is>
-      </c>
       <c r="F65" s="2" t="n"/>
-      <c r="G65" s="2" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
+        </is>
+      </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention" </t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
-        </is>
-      </c>
+      <c r="I65" s="2" t="n"/>
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
       <c r="L65" s="2" t="n"/>
@@ -4079,7 +4080,7 @@
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P65" s="2" t="n"/>
@@ -4087,7 +4088,7 @@
       <c r="R65" s="2" t="n"/>
       <c r="S65" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T65" s="2" t="n"/>
@@ -4116,41 +4117,41 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>intervention schedule of delivery</t>
-        </is>
-      </c>
       <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
+        </is>
+      </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
           <t>This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention"</t>
         </is>
       </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
-        </is>
-      </c>
+      <c r="I66" s="3" t="n"/>
       <c r="J66" s="3" t="n"/>
       <c r="K66" s="3" t="n"/>
       <c r="L66" s="3" t="n"/>
       <c r="M66" s="3" t="n"/>
       <c r="N66" s="3" t="n"/>
-      <c r="O66" s="3" t="n"/>
+      <c r="O66" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P66" s="3" t="n"/>
       <c r="Q66" s="3" t="n"/>
       <c r="R66" s="3" t="n"/>
-      <c r="S66" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S66" s="3" t="n"/>
       <c r="T66" s="3" t="n"/>
       <c r="U66" s="3" t="n"/>
       <c r="V66" s="3" t="n"/>
@@ -4188,7 +4189,7 @@
       <c r="N67" s="4" t="n"/>
       <c r="O67" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P67" s="4" t="n"/>
@@ -4196,7 +4197,7 @@
       <c r="R67" s="4" t="n"/>
       <c r="S67" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T67" s="4" t="n"/>
@@ -4223,12 +4224,12 @@
           <t>A one-dimensional temporal region is a temporal region that is extended.</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="S68" t="inlineStr">
+      <c r="O68" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -4256,12 +4257,12 @@
 </t>
         </is>
       </c>
-      <c r="D69" s="4" t="n"/>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
+      <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="n"/>
       <c r="G69" s="4" t="n"/>
       <c r="H69" s="4" t="n"/>
@@ -4271,15 +4272,15 @@
       <c r="L69" s="4" t="n"/>
       <c r="M69" s="4" t="n"/>
       <c r="N69" s="4" t="n"/>
-      <c r="O69" s="4" t="n"/>
+      <c r="O69" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="P69" s="4" t="n"/>
       <c r="Q69" s="4" t="n"/>
       <c r="R69" s="4" t="n"/>
-      <c r="S69" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="S69" s="4" t="n"/>
       <c r="T69" s="4" t="n"/>
       <c r="U69" s="4" t="n"/>
       <c r="V69" s="4" t="inlineStr">
@@ -4304,34 +4305,34 @@
           <t>A data item between the start and end of an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D70" s="4" t="n"/>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
+      <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
-      <c r="G70" s="4" t="n"/>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>6 weeks; 2 weeks</t>
+        </is>
+      </c>
       <c r="H70" s="4" t="n"/>
-      <c r="I70" s="4" t="inlineStr">
-        <is>
-          <t>6 weeks; 2 weeks</t>
-        </is>
-      </c>
+      <c r="I70" s="4" t="n"/>
       <c r="J70" s="4" t="n"/>
       <c r="K70" s="4" t="n"/>
       <c r="L70" s="4" t="n"/>
       <c r="M70" s="4" t="n"/>
       <c r="N70" s="4" t="n"/>
-      <c r="O70" s="4" t="n"/>
+      <c r="O70" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="P70" s="4" t="n"/>
       <c r="Q70" s="4" t="n"/>
       <c r="R70" s="4" t="n"/>
-      <c r="S70" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="S70" s="4" t="n"/>
       <c r="T70" s="4" t="n"/>
       <c r="U70" s="4" t="n"/>
       <c r="V70" s="4" t="inlineStr">
@@ -4358,12 +4359,12 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
+          <t>temporal reference associated with the intervention</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
           <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>temporal reference associated with the intervention</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -4372,7 +4373,11 @@
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G71" s="2" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
+        </is>
+      </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
@@ -4381,21 +4386,17 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr">
-        <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
+      <c r="J71" s="2" t="n"/>
       <c r="K71" s="2" t="n"/>
       <c r="L71" s="2" t="n"/>
       <c r="M71" s="2" t="n"/>
       <c r="N71" s="2" t="n"/>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P71" s="2" t="n"/>
@@ -4403,7 +4404,7 @@
       <c r="R71" s="2" t="n"/>
       <c r="S71" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T71" s="2" t="n"/>
@@ -4432,12 +4433,12 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
           <t>A statement which describes how the delivery of intervention parts is scheduled relative to associated external events.</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>temporal region</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -4446,32 +4447,32 @@
 We often refer to timepoints when we mean a specific time or some extended period (e.g., Monday). This class allows for the natural usage of a term while maintaining ontological coherence.</t>
         </is>
       </c>
-      <c r="G72" s="3" t="n"/>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
+        </is>
+      </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
           <t>Annotate the words used by authors to describe key events which are not themselves part of the intervention but are relevant to the description of the schedule of the intervention. 
 Example annotation in context: "A feedback call was scheduled to be delivered around 6 months after the birth of the baby".</t>
         </is>
       </c>
-      <c r="I72" s="3" t="inlineStr">
-        <is>
-          <t>A feedback call was scheduled to be delivered around 6 months after the birth of the baby; The smoking intervention started 2 weeks after participants were enrolled into an inpatient setting</t>
-        </is>
-      </c>
+      <c r="I72" s="3" t="n"/>
       <c r="J72" s="3" t="n"/>
       <c r="K72" s="3" t="n"/>
       <c r="L72" s="3" t="n"/>
       <c r="M72" s="3" t="n"/>
       <c r="N72" s="3" t="n"/>
-      <c r="O72" s="3" t="n"/>
+      <c r="O72" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P72" s="3" t="n"/>
       <c r="Q72" s="3" t="n"/>
       <c r="R72" s="3" t="n"/>
-      <c r="S72" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S72" s="3" t="n"/>
       <c r="T72" s="3" t="n"/>
       <c r="U72" s="3" t="n"/>
       <c r="V72" s="3" t="n"/>
@@ -4494,18 +4495,18 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
+          <t>total intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
           <t>The planned total duration of all sessions or digital contacts in an intervention or part</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>total intervention contact event duration</t>
         </is>
       </c>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>"is about" contact events or "is about" duration of contact events?</t>
+          <t>150 minutes; 12 hours</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -4516,12 +4517,12 @@
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>150 minutes; 12 hours</t>
-        </is>
-      </c>
-      <c r="J73" s="2" t="n"/>
+      <c r="I73" s="2" t="n"/>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>"is about" contact events or "is about" duration of contact events?</t>
+        </is>
+      </c>
       <c r="K73" s="2" t="n"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
@@ -4532,7 +4533,7 @@
       <c r="N73" s="2" t="n"/>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="P73" s="2" t="n"/>
@@ -4544,7 +4545,7 @@
       </c>
       <c r="S73" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T73" s="2" t="n"/>
@@ -4575,12 +4576,12 @@
           <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
         </is>
       </c>
-      <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
+      <c r="E74" s="3" t="n"/>
       <c r="F74" s="3" t="n"/>
       <c r="G74" s="3" t="n"/>
       <c r="H74" s="3" t="n"/>
@@ -4590,15 +4591,15 @@
       <c r="L74" s="3" t="n"/>
       <c r="M74" s="3" t="n"/>
       <c r="N74" s="3" t="n"/>
-      <c r="O74" s="3" t="n"/>
+      <c r="O74" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="P74" s="3" t="n"/>
       <c r="Q74" s="3" t="n"/>
       <c r="R74" s="3" t="n"/>
-      <c r="S74" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="S74" s="3" t="n"/>
       <c r="T74" s="3" t="n"/>
       <c r="U74" s="3" t="n"/>
       <c r="V74" s="3" t="n"/>
@@ -4619,12 +4620,12 @@
           <t>A &lt;data item&gt; that is about a collection of total contact event durations.</t>
         </is>
       </c>
-      <c r="D75" s="2" t="n"/>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E75" s="2" t="n"/>
       <c r="F75" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -4642,15 +4643,15 @@
       </c>
       <c r="M75" s="2" t="n"/>
       <c r="N75" s="2" t="n"/>
-      <c r="O75" s="2" t="n"/>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="P75" s="2" t="n"/>
       <c r="Q75" s="2" t="n"/>
       <c r="R75" s="2" t="n"/>
-      <c r="S75" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="S75" s="2" t="n"/>
       <c r="T75" s="2" t="n"/>
       <c r="U75" s="2" t="n"/>
       <c r="V75" s="2" t="inlineStr">
@@ -4678,17 +4679,17 @@
       <c r="D76" s="4" t="n"/>
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
-      <c r="G76" s="4" t="n"/>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>Participants received "3" emails every 2 weeks</t>
+        </is>
+      </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
           <t>This is annotated when a frequency is described using a period and a number of repetitions, rather than a single word.</t>
         </is>
       </c>
-      <c r="I76" s="4" t="inlineStr">
-        <is>
-          <t>Participants received "3" emails every 2 weeks</t>
-        </is>
-      </c>
+      <c r="I76" s="4" t="n"/>
       <c r="J76" s="4" t="n"/>
       <c r="K76" s="4" t="n"/>
       <c r="L76" s="4" t="inlineStr">
@@ -4700,7 +4701,7 @@
       <c r="N76" s="4" t="n"/>
       <c r="O76" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P76" s="4" t="n"/>
@@ -4712,7 +4713,7 @@
       </c>
       <c r="S76" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T76" s="4" t="n"/>
@@ -4743,29 +4744,29 @@
           <t>A data item that is the sum duration of a subset of contact events in a BCI or temporal part</t>
         </is>
       </c>
-      <c r="D77" s="4" t="n"/>
-      <c r="E77" s="4" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="inlineStr">
         <is>
+          <t>The participants took part in "90" minutes of PA weekly</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="n"/>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
           <t>is about contact events or is about duration of contact events?</t>
         </is>
       </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
-        </is>
-      </c>
-      <c r="I77" s="4" t="inlineStr">
-        <is>
-          <t>The participants took part in "90" minutes of PA weekly</t>
-        </is>
-      </c>
-      <c r="J77" s="4" t="n"/>
       <c r="K77" s="4" t="n"/>
       <c r="L77" s="4" t="inlineStr">
         <is>
@@ -4776,7 +4777,7 @@
       <c r="N77" s="4" t="n"/>
       <c r="O77" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P77" s="4" t="n"/>
@@ -4788,7 +4789,7 @@
       </c>
       <c r="S77" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T77" s="4" t="n"/>
@@ -4819,29 +4820,29 @@
           <t>A data item which describes how often a specified sum duration of contact events occured during a BCI or temporal part</t>
         </is>
       </c>
-      <c r="D78" s="4" t="n"/>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
+      <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="inlineStr">
         <is>
+          <t>The participants took part in 90 minutes of PA "weekly"</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="n"/>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
           <t>is about contact events or is about duration of contact events?</t>
         </is>
       </c>
-      <c r="H78" s="4" t="inlineStr">
-        <is>
-          <t>This entity is used when authors describe the frequency of contact within an intervention where the frequency relates to the summed duration of several contact events.</t>
-        </is>
-      </c>
-      <c r="I78" s="4" t="inlineStr">
-        <is>
-          <t>The participants took part in 90 minutes of PA "weekly"</t>
-        </is>
-      </c>
-      <c r="J78" s="4" t="n"/>
       <c r="K78" s="4" t="n"/>
       <c r="L78" s="4" t="inlineStr">
         <is>
@@ -4852,7 +4853,7 @@
       <c r="N78" s="4" t="n"/>
       <c r="O78" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P78" s="4" t="n"/>
@@ -4864,7 +4865,7 @@
       </c>
       <c r="S78" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T78" s="4" t="n"/>
@@ -4895,20 +4896,20 @@
           <t>A temporal interval that is the length of time from start to end of an intervention temporal part</t>
         </is>
       </c>
-      <c r="D79" s="4" t="n"/>
-      <c r="E79" s="4" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t>Temporal Interval (renamed from BFO BFO_0000038)</t>
         </is>
       </c>
+      <c r="E79" s="4" t="n"/>
       <c r="F79" s="4" t="n"/>
-      <c r="G79" s="4" t="n"/>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>Participants received 3 emails every "2" weeks</t>
+        </is>
+      </c>
       <c r="H79" s="4" t="n"/>
-      <c r="I79" s="4" t="inlineStr">
-        <is>
-          <t>Participants received 3 emails every "2" weeks</t>
-        </is>
-      </c>
+      <c r="I79" s="4" t="n"/>
       <c r="J79" s="4" t="n"/>
       <c r="K79" s="4" t="n"/>
       <c r="L79" s="4" t="inlineStr">
@@ -4920,7 +4921,7 @@
       <c r="N79" s="4" t="n"/>
       <c r="O79" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P79" s="4" t="n"/>
@@ -4932,7 +4933,7 @@
       </c>
       <c r="S79" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T79" s="4" t="n"/>
@@ -4962,25 +4963,25 @@
       <c r="D80" s="4" t="n"/>
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="n"/>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>This is not annotated but included due to relationship with duration of interval</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="n"/>
+      <c r="J80" s="4" t="inlineStr">
         <is>
           <t>entity added so duration of interval can be specified. not sure what parent/relationships should be</t>
         </is>
       </c>
-      <c r="H80" s="4" t="inlineStr">
-        <is>
-          <t>This is not annotated but included due to relationship with duration of interval</t>
-        </is>
-      </c>
-      <c r="I80" s="4" t="n"/>
-      <c r="J80" s="4" t="n"/>
       <c r="K80" s="4" t="n"/>
       <c r="L80" s="4" t="n"/>
       <c r="M80" s="4" t="n"/>
       <c r="N80" s="4" t="n"/>
       <c r="O80" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P80" s="4" t="n"/>
@@ -4988,7 +4989,7 @@
       <c r="R80" s="4" t="n"/>
       <c r="S80" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T80" s="4" t="n"/>
@@ -5015,12 +5016,12 @@
           <t>An attribute of a BCI schedule of delivery that is how often intervention temporal parts occur within a BCI.</t>
         </is>
       </c>
-      <c r="D81" s="4" t="n"/>
-      <c r="E81" s="4" t="inlineStr">
+      <c r="D81" s="4" t="inlineStr">
         <is>
           <t>process attribute</t>
         </is>
       </c>
+      <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
           <t>Contact events are intervention temporal parts so this entity also describes the frequency of contact events.</t>
@@ -5046,7 +5047,7 @@
       <c r="N81" s="4" t="n"/>
       <c r="O81" s="4" t="inlineStr">
         <is>
-          <t>JH, SM, RW</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="P81" s="4" t="n"/>
@@ -5058,7 +5059,7 @@
       </c>
       <c r="S81" s="4" t="inlineStr">
         <is>
-          <t>Obsolete</t>
+          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="T81" s="4" t="n"/>

</xml_diff>

<commit_message>
Update 5 terms in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -554,42 +554,38 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BCIO:008500</t>
+          <t>BCIO:003000</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
+          <t>behaviour change intervention</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A &lt;BCI attribute&gt; that is its temporal organisation </t>
+          <t>An intervention that has the aim of influencing human behaviour.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BCI attribute </t>
+          <t>intervention</t>
         </is>
       </c>
       <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Includes the start and end of a BCI, its parts, and their organisation around relevant timepoints.</t>
-        </is>
-      </c>
+      <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>behaviour change intervention delivery</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>BCI duration</t>
+        </is>
+      </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -601,245 +597,250 @@
       <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="V2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:003000</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>behaviour change intervention</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>An intervention that has the aim of influencing human behaviour.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>intervention</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>BCI duration</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="n"/>
-      <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="n"/>
-      <c r="U3" s="2" t="n"/>
-      <c r="V3" s="2" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PATO:0000044</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A physical quality which inheres in a bearer by virtue of the number of the bearer's repetitive actions in a particular time.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>JH; PS</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>PATO:0000044</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>frequency</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>A physical quality which inheres in a bearer by virtue of the number of the bearer's repetitive actions in a particular time.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>specifically dependent continuant</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>JH; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>BCIO:008575</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>interval between intervention temporal parts</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>A &lt;temporal interval&gt; between the end of one intervention temporal part and the beginning of a subsequent intervention temporal part.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>temporal interval</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>The planned duration of a break between two parts of an intervention</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>"2 weeks"; "1 day"</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This is used to capture intervals between BCI parts and timepoints. We annotate only the number and the unit is derived from the context 
 Example annotation (in context): Exercise classes started "2 weeks" after the education phase of the intervention. 
 This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author </t>
         </is>
       </c>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>BCI temporal part</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="2" t="n"/>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2" t="n"/>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T5" s="2" t="n"/>
-      <c r="U5" s="2" t="n"/>
-      <c r="V5" s="2" t="inlineStr">
+      <c r="T4" s="2" t="n"/>
+      <c r="U4" s="2" t="n"/>
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051017</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>interval between intervention temporal parts</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the end of one intervention temporal part and the beginning of a subsequent intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="n"/>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="n"/>
+      <c r="S5" s="3" t="n"/>
+      <c r="T5" s="3" t="n"/>
+      <c r="U5" s="3" t="n"/>
+      <c r="V5" s="3" t="n"/>
+    </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051017</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>interval between intervention temporal parts</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; between the end of one intervention temporal part and the beginning of a subsequent intervention temporal part.</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="n"/>
-      <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="3" t="n"/>
-      <c r="U6" s="3" t="n"/>
-      <c r="V6" s="3" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:051010</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2" t="n"/>
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="2" t="n"/>
+      <c r="U6" s="2" t="n"/>
+      <c r="V6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BCIO:051010</t>
+          <t>BCIO:008510</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>intervention attribute</t>
+          <t>intervention contact event</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
+          <t xml:space="preserve">An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.  </t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>process attribute</t>
+          <t>intervention temporal part</t>
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>All contact events are temporal parts, but not all temporal parts are contact events. Whilst contact events are single continuous events, temporal parts of an intervention can  group together multiple different contact events which might have similar features. For example, a set of 10 counselling sessions might be a temporal part within an intervention. The same intervention can have a set of 5 exercise sessions. These 5 sessions together make up another temporal part. Each single session within these parts  is a contact event.
+This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>A counselling session; An online chat session; An advertisement display.</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event duration</t>
+        </is>
+      </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -851,227 +852,226 @@
       <c r="S7" s="2" t="n"/>
       <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="n"/>
-      <c r="V7" s="2" t="n"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:008510</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051009</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>intervention contact event</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.  </t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>intervention temporal part</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>All contact events are temporal parts, but not all temporal parts are contact events. Whilst contact events are single continuous events, temporal parts of an intervention can  group together multiple different contact events which might have similar features. For example, a set of 10 counselling sessions might be a temporal part within an intervention. The same intervention can have a set of 5 exercise sessions. These 5 sessions together make up another temporal part. Each single session within these parts  is a contact event.
-This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>A counselling session; An online chat session; An advertisement display.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
+      <c r="N8" s="3" t="n"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="n"/>
+      <c r="Q8" s="3" t="n"/>
+      <c r="R8" s="3" t="n"/>
+      <c r="S8" s="3" t="n"/>
+      <c r="T8" s="3" t="n"/>
+      <c r="U8" s="3" t="n"/>
+      <c r="V8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008525</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>An &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>1 hour; 30 minutes; 2 minutes</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2" t="n"/>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="n"/>
+      <c r="U9" s="2" t="n"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051018</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="n"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="n"/>
+      <c r="Q10" s="3" t="n"/>
+      <c r="R10" s="3" t="n"/>
+      <c r="S10" s="3" t="n"/>
+      <c r="T10" s="3" t="n"/>
+      <c r="U10" s="3" t="n"/>
+      <c r="V10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050505</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>intervention contact event duration statistic</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event durations.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>BCI contact event duration</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="P8" s="2" t="n"/>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="n"/>
-      <c r="T8" s="2" t="n"/>
-      <c r="U8" s="2" t="n"/>
-      <c r="V8" s="2" t="inlineStr">
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="n"/>
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="2" t="n"/>
+      <c r="T11" s="2" t="n"/>
+      <c r="U11" s="2" t="n"/>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051009</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>intervention contact event</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>An &lt;intervention temporal part&gt; that is an occasion in which a member of an intervention population comes into contact with an intervention.</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>intervention temporal part</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3" t="n"/>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="3" t="n"/>
-      <c r="U9" s="3" t="n"/>
-      <c r="V9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:008525</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event duration</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>An &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>1 hour; 30 minutes; 2 minutes</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="n"/>
-      <c r="T10" s="2" t="n"/>
-      <c r="U10" s="2" t="n"/>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051018</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>intervention contact event duration</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; between the start and end of an intervention contact event.</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="P11" s="3" t="n"/>
-      <c r="Q11" s="3" t="n"/>
-      <c r="R11" s="3" t="n"/>
-      <c r="S11" s="3" t="n"/>
-      <c r="T11" s="3" t="n"/>
-      <c r="U11" s="3" t="n"/>
-      <c r="V11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050505</t>
+          <t>BCIO:008700</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event duration statistic</t>
+          <t>intervention contact event frequency</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event durations.</t>
+          <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1079,20 +1079,33 @@
           <t>data item</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>How often intervention sessions or digital contacts are planned to occur</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>twice a week; daily; one a week</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is used to capture descriptions of the frequency of contact events within a part.  
+Example annotation (in context): intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks" </t>
+        </is>
+      </c>
       <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>BCI contact event</t>
         </is>
       </c>
       <c r="M12" s="2" t="n"/>
@@ -1110,137 +1123,124 @@
       <c r="U12" s="2" t="n"/>
       <c r="V12" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051001</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event frequency</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="n"/>
+      <c r="Q13" s="3" t="n"/>
+      <c r="R13" s="3" t="n"/>
+      <c r="S13" s="3" t="n"/>
+      <c r="T13" s="3" t="n"/>
+      <c r="U13" s="3" t="n"/>
+      <c r="V13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050903</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>intervention contact event frequency statistic</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>BCI contact event frequency</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2" t="n"/>
+      <c r="T14" s="2" t="n"/>
+      <c r="U14" s="2" t="n"/>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:008700</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>intervention contact event frequency</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>How often intervention sessions or digital contacts are planned to occur</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>twice a week; daily; one a week</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This is used to capture descriptions of the frequency of contact events within a part.  
-Example annotation (in context): intervention sessions took place "weekly" at the participants home; participants received a call from the interventionist "every two weeks" </t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>BCI contact event</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="n"/>
-      <c r="Q13" s="2" t="n"/>
-      <c r="R13" s="2" t="n"/>
-      <c r="S13" s="2" t="n"/>
-      <c r="T13" s="2" t="n"/>
-      <c r="U13" s="2" t="n"/>
-      <c r="V13" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051001</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>intervention contact event frequency</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;data item&gt; about the number times an intervention contact event occurs per unit of time.</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="n"/>
-      <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3" t="n"/>
-      <c r="T14" s="3" t="n"/>
-      <c r="U14" s="3" t="n"/>
-      <c r="V14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050903</t>
+          <t>BCIO:050904</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event frequency statistic</t>
+          <t>intervention contact event number statistic</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event frequencies.</t>
+          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>number of BCI contact events</t>
         </is>
       </c>
       <c r="M15" s="2" t="n"/>
@@ -1286,40 +1286,50 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050904</t>
+          <t>BCIO:008560</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>intervention contact event number statistic</t>
+          <t>intervention duration</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention contact event numbers.</t>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>The planned duration of an intervention</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>6 weeks; 2 months; 1 year</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>This is used to capture the overall duration of intervention delivery from first to last contact of an intervention. It does not include follow-up periods during which no content is delivered. We annotate only the number and the unit is derived from the context. 
+Example Annotation (in context): The intervention ran over "6" weeks, with weekly counselling sessions and biweekly exercise classes 
+This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>number of BCI contact events</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="n"/>
       <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="inlineStr">
@@ -1329,159 +1339,149 @@
       </c>
       <c r="P16" s="2" t="n"/>
       <c r="Q16" s="2" t="n"/>
-      <c r="R16" s="2" t="n"/>
-      <c r="S16" s="2" t="n"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
       <c r="T16" s="2" t="n"/>
       <c r="U16" s="2" t="n"/>
       <c r="V16" s="2" t="inlineStr">
         <is>
+          <t>CM; RW; JH; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051002</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>intervention duration</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="n"/>
+      <c r="Q17" s="3" t="n"/>
+      <c r="R17" s="3" t="n"/>
+      <c r="S17" s="3" t="n"/>
+      <c r="T17" s="3" t="n"/>
+      <c r="U17" s="3" t="n"/>
+      <c r="V17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050905</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>intervention duration statistic</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>BCI duration</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="n"/>
+      <c r="Q18" s="2" t="n"/>
+      <c r="R18" s="2" t="n"/>
+      <c r="S18" s="2" t="n"/>
+      <c r="T18" s="2" t="n"/>
+      <c r="U18" s="2" t="n"/>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:008560</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>intervention duration</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>The planned duration of an intervention</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>6 weeks; 2 months; 1 year</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>This is used to capture the overall duration of intervention delivery from first to last contact of an intervention. It does not include follow-up periods during which no content is delivered. We annotate only the number and the unit is derived from the context. 
-Example Annotation (in context): The intervention ran over "6" weeks, with weekly counselling sessions and biweekly exercise classes 
-This entity has aggregate entities (mean, min, max, median) which should be annotated if explicitly stated by the author</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="n"/>
-      <c r="Q17" s="2" t="n"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
-      <c r="S17" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
-        </is>
-      </c>
-      <c r="T17" s="2" t="n"/>
-      <c r="U17" s="2" t="n"/>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>CM; RW; JH; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:051002</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>intervention duration</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>temporal interval</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
-      <c r="O18" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="P18" s="3" t="n"/>
-      <c r="Q18" s="3" t="n"/>
-      <c r="R18" s="3" t="n"/>
-      <c r="S18" s="3" t="n"/>
-      <c r="T18" s="3" t="n"/>
-      <c r="U18" s="3" t="n"/>
-      <c r="V18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050905</t>
+          <t>BCIO:008500</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>intervention duration statistic</t>
+          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about a collection of intervention durations.</t>
+          <t xml:space="preserve">A &lt;BCI attribute&gt; that is its temporal organisation </t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t xml:space="preserve">BCI attribute </t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+          <t>Includes the start and end of a BCI, its parts, and their organisation around relevant timepoints.</t>
         </is>
       </c>
       <c r="G19" s="2" t="n"/>
@@ -1489,12 +1489,12 @@
       <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>BCI duration</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>behaviour change intervention delivery</t>
+        </is>
+      </c>
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -2036,17 +2036,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>irregular BCI schedule</t>
+          <t>irregular intervention schedule</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An &lt;irregular intervention schedule&gt; in which the frequency and duration of contact events change over the course of a temporal part or intervention.  </t>
+          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or intervention.  </t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>irregular intervention schedule</t>
+          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2054,7 +2054,11 @@
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
           <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
@@ -2098,61 +2102,61 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>BCIO:051013</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>irregular intervention schedule</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of contact events change over the course of a temporal part or intervention.  </t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts vary across the course of an intervention</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>telephone feedback sessions were more frequent during the first 6 weeks; participants were free to access the app whenever they desired</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">We use this to capture instances when authors state that the schedule (i.e. duration and frequency of contact events) varies over the course of a part or intervention. 
 Example annotation in context: "participants were free to access the app as and when they desired";"telephone feedback sessions were more frequent during the first 6 weeks"  </t>
         </is>
       </c>
-      <c r="I30" s="4" t="n"/>
-      <c r="J30" s="4" t="n"/>
-      <c r="K30" s="4" t="n"/>
-      <c r="L30" s="4" t="n"/>
-      <c r="M30" s="4" t="n"/>
-      <c r="N30" s="4" t="n"/>
-      <c r="O30" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P30" s="4" t="n"/>
-      <c r="Q30" s="4" t="n"/>
-      <c r="R30" s="4" t="n"/>
-      <c r="S30" s="4" t="n"/>
-      <c r="T30" s="4" t="n"/>
-      <c r="U30" s="4" t="n"/>
-      <c r="V30" s="4" t="n"/>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="n"/>
+      <c r="N30" s="3" t="n"/>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="n"/>
+      <c r="Q30" s="3" t="n"/>
+      <c r="R30" s="3" t="n"/>
+      <c r="S30" s="3" t="n"/>
+      <c r="T30" s="3" t="n"/>
+      <c r="U30" s="3" t="n"/>
+      <c r="V30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4064,17 +4068,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>regular BCI schedule</t>
+          <t>regular intervention schedule</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A &lt;regular intervention schedule&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
+          <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of Intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>regular intervention schedule</t>
+          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -4082,7 +4086,11 @@
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="F65" s="2" t="n"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
@@ -4122,61 +4130,61 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>BCIO:051014</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>regular intervention schedule</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">An &lt;intervention schedule of delivery&gt; in which the frequency and duration of intervention temporal parts are uniform across the course of an intervention or intervention part.  </t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>A type of schedule which plans that the duration and frequency of sessions or digital contacts remain constant across the course of an intervention</t>
         </is>
       </c>
-      <c r="F66" s="4" t="n"/>
-      <c r="G66" s="4" t="inlineStr">
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>the length and regularity of sessions were consistent across the duration of the intervention, taking place for an hour each week</t>
         </is>
       </c>
-      <c r="H66" s="4" t="inlineStr">
+      <c r="H66" s="3" t="inlineStr">
         <is>
           <t>This is used to capture when the author specifies that the schedule (length and frequency of contact events) does not change over the course of a part. This is rarely annotated as it is not usually explicitly stated. 
 Example annotation in context: "The length and regularity of sessions were consistent across the duration of the intervention"</t>
         </is>
       </c>
-      <c r="I66" s="4" t="n"/>
-      <c r="J66" s="4" t="n"/>
-      <c r="K66" s="4" t="n"/>
-      <c r="L66" s="4" t="n"/>
-      <c r="M66" s="4" t="n"/>
-      <c r="N66" s="4" t="n"/>
-      <c r="O66" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P66" s="4" t="n"/>
-      <c r="Q66" s="4" t="n"/>
-      <c r="R66" s="4" t="n"/>
-      <c r="S66" s="4" t="n"/>
-      <c r="T66" s="4" t="n"/>
-      <c r="U66" s="4" t="n"/>
-      <c r="V66" s="4" t="n"/>
+      <c r="I66" s="3" t="n"/>
+      <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="n"/>
+      <c r="L66" s="3" t="n"/>
+      <c r="M66" s="3" t="n"/>
+      <c r="N66" s="3" t="n"/>
+      <c r="O66" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P66" s="3" t="n"/>
+      <c r="Q66" s="3" t="n"/>
+      <c r="R66" s="3" t="n"/>
+      <c r="S66" s="3" t="n"/>
+      <c r="T66" s="3" t="n"/>
+      <c r="U66" s="3" t="n"/>
+      <c r="V66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update number of intervention contact events in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -3734,12 +3734,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>number of BCI contact events</t>
+          <t>number of intervention contact events</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>A &lt;number of intervention contact events&gt; that is the number of contact events in a BCI temporal part.</t>
+          <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update 4 terms in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -3744,7 +3744,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>number of intervention contact events</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3752,7 +3752,11 @@
           <t>The planned total number of sessions or digital contacts in an intervention or part</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
           <t>one; 6; 12; twenty</t>
@@ -3801,73 +3805,121 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>BCIO:051005</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>number of intervention contact events</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E60" s="4" t="n"/>
-      <c r="F60" s="4" t="n"/>
-      <c r="G60" s="4" t="n"/>
-      <c r="H60" s="4" t="n"/>
-      <c r="I60" s="4" t="n"/>
-      <c r="J60" s="4" t="n"/>
-      <c r="K60" s="4" t="n"/>
-      <c r="L60" s="4" t="n"/>
-      <c r="M60" s="4" t="n"/>
-      <c r="N60" s="4" t="n"/>
-      <c r="O60" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P60" s="4" t="n"/>
-      <c r="Q60" s="4" t="n"/>
-      <c r="R60" s="4" t="n"/>
-      <c r="S60" s="4" t="n"/>
-      <c r="T60" s="4" t="n"/>
-      <c r="U60" s="4" t="n"/>
-      <c r="V60" s="4" t="n"/>
+      <c r="E60" s="3" t="n"/>
+      <c r="F60" s="3" t="n"/>
+      <c r="G60" s="3" t="n"/>
+      <c r="H60" s="3" t="n"/>
+      <c r="I60" s="3" t="n"/>
+      <c r="J60" s="3" t="n"/>
+      <c r="K60" s="3" t="n"/>
+      <c r="L60" s="3" t="n"/>
+      <c r="M60" s="3" t="n"/>
+      <c r="N60" s="3" t="n"/>
+      <c r="O60" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P60" s="3" t="n"/>
+      <c r="Q60" s="3" t="n"/>
+      <c r="R60" s="3" t="n"/>
+      <c r="S60" s="3" t="n"/>
+      <c r="T60" s="3" t="n"/>
+      <c r="U60" s="3" t="n"/>
+      <c r="V60" s="3" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:051012</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>order of intervention temporal parts</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>An &lt;intervention attribute&gt; that is the  temporal positioning of intervention temporal parts.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
+      <c r="I61" s="3" t="n"/>
+      <c r="J61" s="3" t="n"/>
+      <c r="K61" s="3" t="n"/>
+      <c r="L61" s="3" t="n"/>
+      <c r="M61" s="3" t="n"/>
+      <c r="N61" s="3" t="n"/>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P61" s="3" t="n"/>
+      <c r="Q61" s="3" t="n"/>
+      <c r="R61" s="3" t="n"/>
+      <c r="S61" s="3" t="n"/>
+      <c r="T61" s="3" t="n"/>
+      <c r="U61" s="3" t="n"/>
+      <c r="V61" s="3" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>BCIO:008580</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">order of BCI temporal parts </t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>An &lt;order of intervention temporal parts&gt; that is the  temporal positioning of BCI temporal parts.</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>order of intervention temporal parts</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">order of intervention temporal parts </t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>An &lt;intervention attribute&gt; that is the  temporal positioning of intervention temporal parts.</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>"After questionnaires were completed, feedback was selected
 out of a database with messages for each possible combination
@@ -3876,85 +3928,41 @@
 levels to the PA guidelines."</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>This is annotated as an open code when any aspect of order is described</t>
         </is>
       </c>
-      <c r="I61" s="2" t="n"/>
-      <c r="J61" s="2" t="n"/>
-      <c r="K61" s="2" t="n"/>
-      <c r="L61" s="2" t="n"/>
-      <c r="M61" s="2" t="inlineStr">
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="n"/>
+      <c r="K62" s="2" t="n"/>
+      <c r="L62" s="2" t="n"/>
+      <c r="M62" s="2" t="inlineStr">
         <is>
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="N61" s="2" t="n"/>
-      <c r="O61" s="2" t="inlineStr">
+      <c r="N62" s="2" t="n"/>
+      <c r="O62" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="P61" s="2" t="n"/>
-      <c r="Q61" s="2" t="n"/>
-      <c r="R61" s="2" t="n"/>
-      <c r="S61" s="2" t="inlineStr">
+      <c r="P62" s="2" t="n"/>
+      <c r="Q62" s="2" t="n"/>
+      <c r="R62" s="2" t="n"/>
+      <c r="S62" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="T61" s="2" t="n"/>
-      <c r="U61" s="2" t="n"/>
-      <c r="V61" s="2" t="inlineStr">
+      <c r="T62" s="2" t="n"/>
+      <c r="U62" s="2" t="n"/>
+      <c r="V62" s="2" t="inlineStr">
         <is>
           <t>CM; PS</t>
         </is>
       </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:051012</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>order of intervention temporal parts</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>An &lt;intervention attribute&gt; that is the  temporal positioning of intervention temporal parts.</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>intervention attribute</t>
-        </is>
-      </c>
-      <c r="E62" s="4" t="n"/>
-      <c r="F62" s="4" t="n"/>
-      <c r="G62" s="4" t="n"/>
-      <c r="H62" s="4" t="n"/>
-      <c r="I62" s="4" t="n"/>
-      <c r="J62" s="4" t="n"/>
-      <c r="K62" s="4" t="n"/>
-      <c r="L62" s="4" t="n"/>
-      <c r="M62" s="4" t="n"/>
-      <c r="N62" s="4" t="n"/>
-      <c r="O62" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P62" s="4" t="n"/>
-      <c r="Q62" s="4" t="n"/>
-      <c r="R62" s="4" t="n"/>
-      <c r="S62" s="4" t="n"/>
-      <c r="T62" s="4" t="n"/>
-      <c r="U62" s="4" t="n"/>
-      <c r="V62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update total intervention contact event duration in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -4524,12 +4524,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>total intervention contact event duration</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>A &lt;total intervention contact event duration&gt; that is the total of intervention temporal parts within a behaviour change intervention.</t>
+          <t>A &lt;temporal interval&gt; that is the total of intervention temporal parts within an intervention.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update intervention schedule of delivery in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -620,32 +620,32 @@
           <t>BCI attribute</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Includes the start and end of the BCI and its parts.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
+      <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr"/>
-      <c r="Q3" s="3" t="inlineStr"/>
-      <c r="R3" s="3" t="inlineStr"/>
-      <c r="S3" s="3" t="inlineStr"/>
-      <c r="T3" s="3" t="inlineStr"/>
-      <c r="U3" s="3" t="inlineStr"/>
-      <c r="V3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="n"/>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="n"/>
+      <c r="S3" s="3" t="n"/>
+      <c r="T3" s="3" t="n"/>
+      <c r="U3" s="3" t="n"/>
+      <c r="V3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1562,48 +1562,48 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>BCIO:051011</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>An &lt;intervention attribute&gt; that is its temporal organisation.</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
-      <c r="O21" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P21" s="3" t="n"/>
-      <c r="Q21" s="3" t="n"/>
-      <c r="R21" s="3" t="n"/>
-      <c r="S21" s="3" t="n"/>
-      <c r="T21" s="3" t="n"/>
-      <c r="U21" s="3" t="n"/>
-      <c r="V21" s="3" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4" t="n"/>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="n"/>
+      <c r="Q21" s="4" t="n"/>
+      <c r="R21" s="4" t="n"/>
+      <c r="S21" s="4" t="n"/>
+      <c r="T21" s="4" t="n"/>
+      <c r="U21" s="4" t="n"/>
+      <c r="V21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update 3 terms in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -1084,7 +1084,7 @@
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event duration</t>
+          <t>intervention contact event duration</t>
         </is>
       </c>
       <c r="M12" s="2" t="n"/>
@@ -1149,11 +1149,11 @@
         </is>
       </c>
       <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event</t>
+          <t>intervention contact event</t>
         </is>
       </c>
       <c r="M13" s="2" t="n"/>
@@ -1253,7 +1253,7 @@
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event frequency</t>
+          <t>intervention contact event frequency</t>
         </is>
       </c>
       <c r="M15" s="2" t="n"/>

</xml_diff>

<commit_message>
Update 6 terms in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -3752,7 +3752,7 @@
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>total intervention contact event duration</t>
         </is>
       </c>
       <c r="M59" s="2" t="n"/>
@@ -3822,7 +3822,7 @@
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event</t>
+          <t>intervention contact event</t>
         </is>
       </c>
       <c r="M60" s="2" t="n"/>
@@ -3987,7 +3987,7 @@
       <c r="L63" s="2" t="n"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
+          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="N63" s="2" t="n"/>
@@ -4473,10 +4473,10 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="n"/>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="n"/>
       <c r="L72" s="2" t="n"/>
       <c r="M72" s="2" t="n"/>
@@ -4617,7 +4617,7 @@
       <c r="K74" s="2" t="n"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>BCI contact event</t>
+          <t>intervention contact event</t>
         </is>
       </c>
       <c r="M74" s="2" t="n"/>
@@ -4729,7 +4729,7 @@
       <c r="K76" s="2" t="n"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>total BCI contact event duration</t>
+          <t>total intervention contact event duration</t>
         </is>
       </c>
       <c r="M76" s="2" t="n"/>

</xml_diff>